<commit_message>
feat(media): say Radium in the media wording too
Tracker decision D25 kept media untouched. On 2026-09-13 the user was
shown the three media messages that still said "Radium Chat" and asked
for them to say "Radium" as well. Scope is exactly those strings:

- containers/media/MediaPreview.tsx (protected - accepted by the next,
  isolated re-baseline commit)
- containers/media/params/MediaParamField.tsx
- services/media/adapters/atomicWorker.ts
- locales/en/media.json

"Radium Media", the media code, types, ids and the credential service
name are unchanged. tests/radium-product-name.test.mjs no longer skips
media.json, so the locale check now covers it. Tracker: D25 amended,
T21-S08 and T21-S13 noted.

Verified: media suites 19 files / 398 tests pass; contract test 8/8.
The guard was run after this change and named exactly one file,
MediaPreview.tsx.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -9053,7 +9053,7 @@
       </c>
       <c r="I160" s="15" t="inlineStr">
         <is>
-          <t>Done 2026-09-13. About 300 strings across 100+ files, reviewed as a dry run before writing. KEPT by design (D24): config-file markers and provider keys other code looks up, the CLI ownership marker, the media credential name. KEPT per D25: media wording still saying 'Radium Chat'. 'Radium Chat Q8_0' corrected to 'AtomicChat Q8_0' (those drafts are the AtomicChat Hugging Face org's). Assistant-extension migration v4 renames saved instructions and the default assistant's name; 12 tests. | Earlier note: NOT a find-and-replace: D13 had to revert 25 files where the name was part of a real path. Paths, ids, the atomic.chat domain and upstream links are excluded unless D24 says otherwise.</t>
+          <t>Done 2026-09-13. About 300 strings across 100+ files, reviewed as a dry run before writing. KEPT by design (D24): config-file markers and provider keys other code looks up, the CLI ownership marker, the media credential name. KEPT per D25: media wording still saying 'Radium Chat'. 'Radium Chat Q8_0' corrected to 'AtomicChat Q8_0' (those drafts are the AtomicChat Hugging Face org's). Assistant-extension migration v4 renames saved instructions and the default assistant's name; 12 tests. | Earlier note: NOT a find-and-replace: D13 had to revert 25 files where the name was part of a real path. Paths, ids, the atomic.chat domain and upstream links are excluded unless D24 says otherwise. | 2026-09-13 AMENDMENT (D25): the three media messages now say Radium too; the contract test covers media.json again.</t>
         </is>
       </c>
     </row>
@@ -9258,7 +9258,7 @@
       </c>
       <c r="I165" s="15" t="inlineStr">
         <is>
-          <t>ADR 2026-09-13-rename-the-product-to-radium-and-move-the-data-folder.md and the INDEX entry are written. NOT committed: waiting for the user's authorisation.</t>
+          <t>2026-09-13: rename committed as 1df96dc89 with the user's authorisation. The media-wording change (D25 amendment) and its isolated guard re-baseline follow as two commits. NOT pushed, no PR yet: each needs the user's authorisation.</t>
         </is>
       </c>
     </row>
@@ -10457,7 +10457,7 @@
       </c>
       <c r="E32" s="15" t="inlineStr">
         <is>
-          <t>ANSWERED BY THE USER 2026-09-13: yes - keep 'Radium Media' and leave every media file alone. No protected file is edited and the guard is not re-baselined for Task 21.</t>
+          <t>ANSWERED BY THE USER 2026-09-13: yes - keep 'Radium Media' and leave every media file alone. No protected file is edited and the guard is not re-baselined for Task 21. AMENDED BY THE USER 2026-09-13, after being shown the three media messages that still said 'Radium Chat': change the media WORDING to Radium too. Scope is exactly those strings - MediaPreview.tsx (protected), MediaParamField.tsx, adapters/atomicWorker.ts and locales/en/media.json. The name 'Radium Media', the media code, types, ids and the credential service name are unchanged. The one protected file is accepted by an isolated guard re-baseline commit, as Q1 requires.</t>
         </is>
       </c>
       <c r="F32" s="13" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): record the backup, test build and PR #9
Task 21 progress, 2026-09-13:

- T21-S12 In progress: the data folder was backed up to the Desktop
  (2846 files / 3,542,750,285 bytes, identical to %APPDATA%\Atomic Chat,
  copied with the app and llama-server confirmed closed), and test
  build run 34765539327 is building the installer from 4402b9749.
- T21-S13 In progress: the three rename commits are pushed and PR #9 is
  open on top of PR #8. It stays open until #8 merges and #9 is
  retargeted to main.
- Handover: current branch, latest commit, and the next action - the
  install check over the Atomic Chat 2.0.23 MSI, then the merge order.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1069,7 +1069,7 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>main. Open on 2026-09-13: chore/upstream-v2.0.37 (PR #8, the v2.0.37 sync) and feat/radium-product-name (Task 21, uncommitted draft only)</t>
+          <t>2026-09-13: feat/radium-product-name (PR #9, Task 21) stacked on chore/upstream-v2.0.37 (PR #8, the v2.0.37 sync). Merge #8 first, then retarget #9 to main.</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>6c3909482 on chore/upstream-v2.0.37, pushed as PR #8: the v2.0.37 merge d64fb7ded plus a test-quality fix. feat/radium-product-name branches from it with NO commits of its own - only the uncommitted Task 21 draft.</t>
+          <t>4402b9749 on feat/radium-product-name, pushed: chore(guard) re-baseline accepting MediaPreview.tsx. Before it: a22ac62da media wording, 1df96dc89 the rename, 810c0a48a the Task 21 tracker entry.</t>
         </is>
       </c>
     </row>
@@ -1093,7 +1093,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>2026-09-13: Task 21 (rename the product to Radium) is IN PROGRESS. D24 and D25 answered; next is T21-S03, the failing contract test. | Earlier: Tasks 0-8, 10-16 and 18 Done. Task 9 SKIPPED. Tasks 14, 15, 17 PARTIAL - each blocked only on hardware, another repo, or translators. NEW: TASK 19, a full sync to upstream v2.0.35, added 2026-09-11 when the user answered Q6. There are now NO open decisions. Task 19 is the next piece of work, and T19-S01 says to land PRs #3 and #2 first so the sync happens against a stable main.</t>
+          <t>2026-09-13: Task 21 S01-S11 Done; S12 (install test on this PC) and S13 (merge) In progress. Data backed up to the Desktop; test build run 34765539327 is running. | Earlier: Tasks 0-8, 10-16 and 18 Done. Task 9 SKIPPED. Tasks 14, 15, 17 PARTIAL - each blocked only on hardware, another repo, or translators. NEW: TASK 19, a full sync to upstream v2.0.35, added 2026-09-11 when the user answered Q6. There are now NO open decisions. Task 19 is the next piece of work, and T19-S01 says to land PRs #3 and #2 first so the sync happens against a stable main.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-13: work Task 21 from T21-S03 (contract test first) on feat/radium-product-name. Media must stay untouched - make test-selective-v2032 with NO re-baseline. Ask before committing, pushing or creating branches. | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
+          <t>2026-09-13: when run 34765539327 finishes, install its NSIS exe over the Atomic Chat 2.0.23 MSI and check: old MSI entry gone, Radium in Apps and the Start menu, %APPDATA%\Radium\data holds the 4 threads and the models, both settings.json repointed, app.log records the move, a model chats. Backup: Desktop\Atomic Chat backup 2026-09-13. Then merge PR #8, retarget PR #9 to main, merge. Ask before committing, pushing or merging. | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
         </is>
       </c>
     </row>
@@ -2488,7 +2488,11 @@
           <t>tests/radium-product-name.test.mjs green; make test-selective-v2032 green with NO re-baseline; full verify; upgrade over the installed Atomic Chat 2.0.23 MSI verified on this PC with data intact</t>
         </is>
       </c>
-      <c r="I24" s="13" t="n"/>
+      <c r="I24" s="13" t="inlineStr">
+        <is>
+          <t>1df96dc89, a22ac62da, 4402b9749 (PR #9)</t>
+        </is>
+      </c>
       <c r="J24" s="14" t="inlineStr">
         <is>
           <t>ADDED 2026-09-13 at the user's instruction, in two parts. First: rename the GitHub repo, the saved data folder and the installer (scope chosen by the user: 'data folder + installer name'; repo name 'Radium'). Then, correcting the name: "Radium, NOT Radium Chat. Update everything, retain all previous code where possible, especially media." Not in the original plan. This IS the data-folder migration that D13 said had to exist before productName could change. Design: C:\Users\Warwick\.claude\plans\swift-honking-dragonfly.md (written for 'Radium Chat': the name changes to 'Radium', the design does not).</t>
@@ -9201,7 +9205,7 @@
       </c>
       <c r="E164" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F164" s="13" t="n"/>
@@ -9217,7 +9221,7 @@
       </c>
       <c r="I164" s="15" t="inlineStr">
         <is>
-          <t>The only real proof the migration is safe with real data. If anything is wrong: rename the folder back and restore data_folder in both settings.json files. | 2026-09-13: needs a commit, a push and a test build first, each of which needs the user's authorisation.</t>
+          <t>2026-09-13 IN PROGRESS. BACKUP DONE: C:\Users\Warwick\Desktop\Atomic Chat backup 2026-09-13, 2846 files / 3,542,750,285 bytes, identical count and size to %APPDATA%\Atomic Chat; robocopy 0 failed (exit code 1 means files copied). Copied with Atomic Chat and llama-server confirmed not running. TEST BUILD RUNNING: windows-test-build.yml run 34765539327 on feat/radium-product-name at 4402b9749, https://github.com/walladanger/Radium/actions/runs/34765539327 - the first build to compile the new NSIS pre-install hook. Next: install the NSIS exe over the Atomic Chat 2.0.23 MSI and check the expectations in the Command column. | Earlier note: The only real proof the migration is safe with real data. If anything is wrong: rename the folder back and restore data_folder in both settings.json files. | 2026-09-13: needs a commit, a push and a test build first, each of which needs the user's authorisation.</t>
         </is>
       </c>
     </row>
@@ -9258,7 +9262,7 @@
       </c>
       <c r="I165" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13: rename committed as 1df96dc89 with the user's authorisation. The media-wording change (D25 amendment) and its isolated guard re-baseline follow as two commits. NOT pushed, no PR yet: each needs the user's authorisation.</t>
+          <t>2026-09-13: commits 1df96dc89 (rename), a22ac62da (media wording, D25 amendment) and 4402b9749 (isolated guard re-baseline accepting only MediaPreview.tsx), each authorised by the user. Pushed, and PR #9 opened with the user's authorisation: https://github.com/walladanger/Radium/pull/9, base chore/upstream-v2.0.37, 4 commits, mergeable. Stays open until PR #8 merges and #9 is retargeted to main and merged. This tracker update is itself uncommitted until the user says so.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): record the install test result on this PC
Task 21, 2026-09-13. The test build from 4402b9749 was installed over
the Atomic Chat 2.0.23 MSI, and the rename and data move worked on real
data:

- the old MSI entry and Start menu shortcut are gone; Radium 2.0.37 is
  installed per-user with its own shortcut
- app.log recorded the move of Atomic Chat\data to Radium\data with both
  settings.json files updated; a relaunch logged AlreadyMigrated
- all 2846 backed-up files are present in the new folder, and a model
  loaded

T21-S12 stays In progress: the user has not yet confirmed a chat reply,
and the empty Radium Chat folder was not removed. That gap is new step
T21-S14, with the evidence gathered so far and the causes ruled out.

Also recorded: D27, GitHub's Node.js 20 deprecation warning for the
workflow actions, as a small separate PR after Task 21 merges.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1093,7 +1093,7 @@
       </c>
       <c r="B8" s="22" t="inlineStr">
         <is>
-          <t>2026-09-13: Task 21 S01-S11 Done; S12 (install test on this PC) and S13 (merge) In progress. Data backed up to the Desktop; test build run 34765539327 is running. | Earlier: Tasks 0-8, 10-16 and 18 Done. Task 9 SKIPPED. Tasks 14, 15, 17 PARTIAL - each blocked only on hardware, another repo, or translators. NEW: TASK 19, a full sync to upstream v2.0.35, added 2026-09-11 when the user answered Q6. There are now NO open decisions. Task 19 is the next piece of work, and T19-S01 says to land PRs #3 and #2 first so the sync happens against a stable main.</t>
+          <t>2026-09-13: Task 21's install test on this PC PASSED on real data (T21-S12). Open: a chat-reply confirmation from the user, T21-S14 (stray Radium Chat folder not removed), and merging PR #8 then #9. | Earlier: Tasks 0-8, 10-16 and 18 Done. Task 9 SKIPPED. Tasks 14, 15, 17 PARTIAL - each blocked only on hardware, another repo, or translators. NEW: TASK 19, a full sync to upstream v2.0.35, added 2026-09-11 when the user answered Q6. There are now NO open decisions. Task 19 is the next piece of work, and T19-S01 says to land PRs #3 and #2 first so the sync happens against a stable main.</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-13: when run 34765539327 finishes, install its NSIS exe over the Atomic Chat 2.0.23 MSI and check: old MSI entry gone, Radium in Apps and the Start menu, %APPDATA%\Radium\data holds the 4 threads and the models, both settings.json repointed, app.log records the move, a model chats. Backup: Desktop\Atomic Chat backup 2026-09-13. Then merge PR #8, retarget PR #9 to main, merge. Ask before committing, pushing or merging. | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
+          <t>2026-09-13: (1) the user confirms a chat gets a reply in Radium; (2) T21-S14 - reproduce and fix why the empty %APPDATA%\Radium Chat folder survived the migration, failing test first; (3) merge PR #8, retarget PR #9 to main, merge. Backup kept at Desktop\Atomic Chat backup 2026-09-13 until the user is happy. Then D27 (Node 20 actions) as its own PR. Ask before committing, pushing or merging. | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
         </is>
       </c>
     </row>
@@ -2500,7 +2500,7 @@
       </c>
       <c r="K24" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13 PROGRESS: S01-S11 Done and verified (see Steps). Open: S12 install test on this PC, S13 commit and PR - both wait for the user. STILL SAYING 'Radium Chat' OR 'Atomic Chat', each deliberate and reported to the user: media wording in MediaPreview.tsx (protected), MediaParamField.tsx, atomicWorker.ts and en/media.json (D25); the entry name Radium writes into Zed and Droid, which their config uses as a lookup key; LICENSE header (legal - user's call); the sidebar wordmark in AppLogo.tsx, drawn as SVG and owned by the separate wordmark task. PRE-EXISTING, found on the way, not fixed: CLI_OWNERSHIP_MARKER is b"Radium Chat" since D13, but the legacy jan binaries it is meant to recognise would contain 'Atomic Chat'; src-tauri/tauri.bundle.windows.nsis.template is not referenced by any build config. | Earlier: 2026-09-13, STATE BEFORE CODE STARTS, stated plainly. DONE: GitHub repo renamed walladanger/Atomic-Chat -&gt; walladanger/Radium, authorised by the user; local origin repointed; PR #8 and Windows test build run 34761971349 followed the rename and old URLs redirect. NOT DONE, DRAFT ONLY: branch feat/radium-product-name (off chore/upstream-v2.0.37 at 6c3909482) holds UNCOMMITTED edits written for 'Radium Chat' - a data-folder migration module with 11 unit tests, an NSIS pre-install hook, a launch-at-startup migration command, a contract test, an ADR and doc edits. NONE OF IT HAS BEEN COMPILED OR RUN. It will be re-targeted to 'Radium' and verified from scratch, not trusted as written. THE AGENT CREATED THAT BRANCH WITHOUT ASKING, which the working agreement forbids; recorded here rather than hidden. MEASURED ON THIS PC, not assumed: the data folder C:\Users\Warwick\AppData\Roaming\Atomic Chat\data is 3.4 GB and stores no absolute path to itself (model.yml paths are relative), so a same-volume rename is safe. BOTH settings.json files - %APPDATA%\chat.atomic.app and the legacy %APPDATA%\Atomic-Chat, which wins while it exists - name that path, so changing productName alone moves nothing and the migration must repoint both. The installed app is an MSI (v2.0.23, WiX key {64542677-4056-4D46-BBEE-094163B8EC1A}): the MSI channel upgrades in place because its upgradeCode is pinned, but the NSIS installer finds a previous install by productName and would install side by side without a pre-install hook. A stray, empty %APPDATA%\Radium Chat\data (one 0-byte db file, made by jan-cli) exists - see D26. Launch-at-startup is OFF on this PC today. MEDIA: nothing in this task needs a protected file, and the guard must pass untouched.</t>
+          <t>2026-09-13 INSTALL TEST ON THIS PC: the rename and data move WORKED on real data - see T21-S12 for the measurements. Open: the user confirming a chat reply, and T21-S14 (the empty Radium Chat folder was not removed). Also recorded: D27, the Node.js 20 deprecation warning in the workflows. | Earlier: 2026-09-13 PROGRESS: S01-S11 Done and verified (see Steps). Open: S12 install test on this PC, S13 commit and PR - both wait for the user. STILL SAYING 'Radium Chat' OR 'Atomic Chat', each deliberate and reported to the user: media wording in MediaPreview.tsx (protected), MediaParamField.tsx, atomicWorker.ts and en/media.json (D25); the entry name Radium writes into Zed and Droid, which their config uses as a lookup key; LICENSE header (legal - user's call); the sidebar wordmark in AppLogo.tsx, drawn as SVG and owned by the separate wordmark task. PRE-EXISTING, found on the way, not fixed: CLI_OWNERSHIP_MARKER is b"Radium Chat" since D13, but the legacy jan binaries it is meant to recognise would contain 'Atomic Chat'; src-tauri/tauri.bundle.windows.nsis.template is not referenced by any build config. | Earlier: 2026-09-13, STATE BEFORE CODE STARTS, stated plainly. DONE: GitHub repo renamed walladanger/Atomic-Chat -&gt; walladanger/Radium, authorised by the user; local origin repointed; PR #8 and Windows test build run 34761971349 followed the rename and old URLs redirect. NOT DONE, DRAFT ONLY: branch feat/radium-product-name (off chore/upstream-v2.0.37 at 6c3909482) holds UNCOMMITTED edits written for 'Radium Chat' - a data-folder migration module with 11 unit tests, an NSIS pre-install hook, a launch-at-startup migration command, a contract test, an ADR and doc edits. NONE OF IT HAS BEEN COMPILED OR RUN. It will be re-targeted to 'Radium' and verified from scratch, not trusted as written. THE AGENT CREATED THAT BRANCH WITHOUT ASKING, which the working agreement forbids; recorded here rather than hidden. MEASURED ON THIS PC, not assumed: the data folder C:\Users\Warwick\AppData\Roaming\Atomic Chat\data is 3.4 GB and stores no absolute path to itself (model.yml paths are relative), so a same-volume rename is safe. BOTH settings.json files - %APPDATA%\chat.atomic.app and the legacy %APPDATA%\Atomic-Chat, which wins while it exists - name that path, so changing productName alone moves nothing and the migration must repoint both. The installed app is an MSI (v2.0.23, WiX key {64542677-4056-4D46-BBEE-094163B8EC1A}): the MSI channel upgrades in place because its upgradeCode is pinned, but the NSIS installer finds a previous install by productName and would install side by side without a pre-install hook. A stray, empty %APPDATA%\Radium Chat\data (one 0-byte db file, made by jan-cli) exists - see D26. Launch-at-startup is OFF on this PC today. MEDIA: nothing in this task needs a protected file, and the guard must pass untouched.</t>
         </is>
       </c>
     </row>
@@ -2521,7 +2521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I165"/>
+  <dimension ref="A1:I166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9221,7 +9221,7 @@
       </c>
       <c r="I164" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13 IN PROGRESS. BACKUP DONE: C:\Users\Warwick\Desktop\Atomic Chat backup 2026-09-13, 2846 files / 3,542,750,285 bytes, identical count and size to %APPDATA%\Atomic Chat; robocopy 0 failed (exit code 1 means files copied). Copied with Atomic Chat and llama-server confirmed not running. TEST BUILD RUNNING: windows-test-build.yml run 34765539327 on feat/radium-product-name at 4402b9749, https://github.com/walladanger/Radium/actions/runs/34765539327 - the first build to compile the new NSIS pre-install hook. Next: install the NSIS exe over the Atomic Chat 2.0.23 MSI and check the expectations in the Command column. | Earlier note: The only real proof the migration is safe with real data. If anything is wrong: rename the folder back and restore data_folder in both settings.json files. | 2026-09-13: needs a commit, a push and a test build first, each of which needs the user's authorisation.</t>
+          <t>2026-09-13 INSTALL TEST, MEASURED ON THIS PC (installer from run 34765539327 at 4402b9749). PASSED: the Atomic Chat 2.0.23 MSI entry ({64542677-...}) is gone; Radium 2.0.37 is installed per-user (HKCU Uninstall\Radium, C:\Users\Warwick\AppData\Local\Radium) with Start menu Radium.lnk, and the old Atomic Chat Start menu shortcut is gone. app.log at 16:45:38 UTC: 'Moved the data folder from ...\Atomic Chat\data to ...\Radium\data (2 settings file(s) updated)'. %APPDATA%\Atomic Chat no longer exists; BOTH settings.json (chat.atomic.app and Atomic-Chat) name %APPDATA%\Radium\data. All 2846 backed-up files are present in the new folder (0 missing; it now has 2904, as the app has been used since: 5 threads against 4 in the backup, 2 model.yml against 1). A relaunch at 17:58:59 UTC logged 'Data folder migration not needed: AlreadyMigrated'. A llama.cpp model loaded at 16:53:23. Launch at startup was off before and has no entry now, which is correct. STILL OPEN: (1) the user has not yet confirmed a chat gets a reply in the app - a model loading is not the same thing; (2) the empty %APPDATA%\Radium Chat\data\db\__status__.db folder was NOT removed although the migration should have removed it - see T21-S14. SEEN IN THE LOG, NOT CAUSED BY THE RENAME: two model downloads at 18:02 UTC failed with 'dns error: No such host is known' (the PC was offline); ollama gemma4-latest.gguf is rejected by llama.cpp with 'wrong number of tensors; expected 2131, got 720' (an incompatible file, not a path problem). SEEN ONCE, CAUSE NOT ESTABLISHED: at 16:54:21 UTC, after 'App cleanup completed', the app logged 'Application panic: cannot move state from Destroyed' in tao-0.34.8 event_loop/runner.rs:371 - i.e. during shutdown. Absent from the older logs, but those are rotated 10 MB files, so that proves little. | Earlier note: 2026-09-13 IN PROGRESS. BACKUP DONE: C:\Users\Warwick\Desktop\Atomic Chat backup 2026-09-13, 2846 files / 3,542,750,285 bytes, identical count and size to %APPDATA%\Atomic Chat; robocopy 0 failed (exit code 1 means files copied). Copied with Atomic Chat and llama-server confirmed not running. TEST BUILD RUNNING: windows-test-build.yml run 34765539327 on feat/radium-product-name at 4402b9749, https://github.com/walladanger/Radium/actions/runs/34765539327 - the first build to compile the new NSIS pre-install hook. Next: install the NSIS exe over the Atomic Chat 2.0.23 MSI and check the expectations in the Command column. | Earlier note: The only real proof the migration is safe with real data. If anything is wrong: rename the folder back and restore data_folder in both settings.json files. | 2026-09-13: needs a commit, a push and a test build first, each of which needs the user's authorisation.</t>
         </is>
       </c>
     </row>
@@ -9263,6 +9263,47 @@
       <c r="I165" s="15" t="inlineStr">
         <is>
           <t>2026-09-13: commits 1df96dc89 (rename), a22ac62da (media wording, D25 amendment) and 4402b9749 (isolated guard re-baseline accepting only MediaPreview.tsx), each authorised by the user. Pushed, and PR #9 opened with the user's authorisation: https://github.com/walladanger/Radium/pull/9, base chore/upstream-v2.0.37, 4 commits, mergeable. Stays open until PR #8 merges and #9 is retargeted to main and merged. This tracker update is itself uncommitted until the user says so.</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="6" t="inlineStr">
+        <is>
+          <t>T21-S14</t>
+        </is>
+      </c>
+      <c r="B166" s="17" t="inlineStr">
+        <is>
+          <t>Task 21</t>
+        </is>
+      </c>
+      <c r="C166" s="6" t="n">
+        <v>14</v>
+      </c>
+      <c r="D166" s="14" t="inlineStr">
+        <is>
+          <t>Find why the empty %APPDATA%\Radium Chat folder was not removed on the install test</t>
+        </is>
+      </c>
+      <c r="E166" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F166" s="13" t="n"/>
+      <c r="G166" s="14" t="inlineStr">
+        <is>
+          <t>Reproduce with this PC's real layout (vector-db creates Radium\data\db at plugin init, before setup; stray Radium Chat\data\db\__status__.db, 0 bytes) and fix with a failing test first.</t>
+        </is>
+      </c>
+      <c r="H166" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I166" s="15" t="inlineStr">
+        <is>
+          <t>FOUND 2026-09-13 on the install test. Expected: after 'Moved the data folder', the cleanup loop in data_migration.rs (lines 141-150 at 4402b9749) deletes any other old default folder that holds no data. Observed: C:\Users\Warwick\AppData\Roaming\Radium Chat\data\db\__status__.db still there, 0 bytes, created and last written 2026-09-11 08:18 - so it was never removed, not removed and recreated. Ruled out: not locked, not read-only (attrs=Archive), owned by the user, and a copy deletes fine. The installed code is identical to the branch, and unit test removes_the_empty_radium_chat_folder_jan_cli_left_behind passes, so the cause is not known yet. HARMLESS in the meantime: no code in the installed build writes to that folder, and removing it by hand loses nothing.</t>
         </is>
       </c>
     </row>
@@ -9283,7 +9324,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="A1:G34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10507,6 +10548,43 @@
         </is>
       </c>
       <c r="G33" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>D27</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>CI MAINTENANCE, not a question yet: GitHub warns that Node.js 20 is deprecated for the actions the workflows use (actions/checkout, actions/cache, actions/setup-node, actions/setup-python, actions/upload-artifact). Seen as an annotation on test build run 34765539327.</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Nothing today: GitHub forces those actions onto Node.js 24 and the build passed. It would bite only if GitHub stops forcing that and the old action versions stop running.</t>
+        </is>
+      </c>
+      <c r="D34" s="14" t="inlineStr">
+        <is>
+          <t>Do it AFTER Task 21 merges, as its own small PR: raise each named action to its current major version in windows-test-build.yml and release.yml (check each version on GitHub first rather than assuming numbers), then run one test build to prove the installer still builds. Keep the release.yml change minimal - it is upstream's file, so every line edited is a possible conflict on the next sync.</t>
+        </is>
+      </c>
+      <c r="E34" s="15" t="inlineStr">
+        <is>
+          <t>Agent recommendation, 2026-09-13; the user asked whether it needs updating and was told not yet.</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="inlineStr">
+        <is>
+          <t>Noted</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): add Task 22, move API and Cloud into Settings
The user asked on 2026-09-13 for API and Cloud to live in Settings
rather than in the sidebar, where the v2.0.35 sync put them (upstream
d887d3817). Task 22 covers it in nine steps, starting after PR #9 merges
on a new branch off main.

D28 answered by the user: option B. Both pages render inside the
Settings layout at /settings/api and /settings/cloud, and the old /api
and /cloud addresses redirect there so existing links keep working. The
accepted cost is a few more changed files and more upstream merge
conflicts than plain links would have.

Scope was measured before writing the steps: the pages, the four places
that link to them, and how far the touched files already differ from
upstream. No protected media file is involved, and Media stays in the
sidebar.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-13: (1) the user confirms a chat gets a reply in Radium; (2) T21-S14 - reproduce and fix why the empty %APPDATA%\Radium Chat folder survived the migration, failing test first; (3) merge PR #8, retarget PR #9 to main, merge. Backup kept at Desktop\Atomic Chat backup 2026-09-13 until the user is happy. Then D27 (Node 20 actions) as its own PR. Ask before committing, pushing or merging. | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
+          <t>2026-09-13 (later): finish Task 21 first (chat-reply confirmation, T21-S14, merge PR #8 then #9). NEW: Task 22 moves API and Cloud from the sidebar into Settings - get D28 answered, then branch off main after #9 merges. Ask before committing, pushing, merging or creating branches. | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K24"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2504,6 +2504,55 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="B25" s="11" t="inlineStr">
+        <is>
+          <t>10 - Navigation</t>
+        </is>
+      </c>
+      <c r="C25" s="14" t="inlineStr">
+        <is>
+          <t>Move API and Cloud out of the sidebar and into Settings</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="E25" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F25" s="13" t="n"/>
+      <c r="G25" s="14" t="inlineStr">
+        <is>
+          <t>D28 answered 2026-09-13 (option B). Waits only for PR #9 to merge; then a new branch off main.</t>
+        </is>
+      </c>
+      <c r="H25" s="14" t="inlineStr">
+        <is>
+          <t>Neither API nor Cloud appears in the sidebar; both are reachable from Settings; every existing link and old address still lands on the right page; web tests, typecheck and lint green; guard untouched.</t>
+        </is>
+      </c>
+      <c r="I25" s="13" t="n"/>
+      <c r="J25" s="14" t="inlineStr">
+        <is>
+          <t>ADDED 2026-09-13 at the user's instruction: "API and cloud need to live in settings." Prompted by comparing the sidebar before and after the v2.0.35 sync, which is what put them there. Not in the original plan.</t>
+        </is>
+      </c>
+      <c r="K25" s="15" t="inlineStr">
+        <is>
+          <t>SCOPE MEASURED 2026-09-13, not assumed. Today: web-app/src/components/left-sidebar/NavMain.tsx renders top-level Cloud (route.cloud.index = /cloud/, routes/cloud/index.tsx, 243 lines, the cloud provider registry) and API (route.api.index = /api/, routes/api/index.tsx, 148 lines, the local API server page). Upstream put them there DELIBERATELY in d887d3817 (Mike, 2026-09-03, 'Improve/agent flow #265'): /settings/local-api-server now only redirects to /api, and Settings &gt; Model providers &gt; a provider navigates to /cloud. OTHER PLACES THAT LINK TO THEM and must keep working: containers/DropdownModelProvider.tsx (to /cloud), containers/LocalApiServerStatusRow.tsx (to /api), routes/settings/providers/$providerName.tsx (to /cloud), routes/settings/local-api-server.tsx (redirect to /api). Settings menu: containers/SettingsMenu.tsx. MERGE COST: this reverses an upstream design choice, so NavMain.tsx, SettingsMenu.tsx and constants/routes.ts will conflict on upstream syncs that touch them. They differ from v2.0.37 today by only +18, +6 and +3 lines, so keep the change small and in as few upstream files as possible. MEDIA: none of these files is protected, and Media stays in the sidebar.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:K40"/>
   <dataValidations count="1">
@@ -2521,7 +2570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I166"/>
+  <dimension ref="A1:I175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9306,6 +9355,371 @@
           <t>FOUND 2026-09-13 on the install test. Expected: after 'Moved the data folder', the cleanup loop in data_migration.rs (lines 141-150 at 4402b9749) deletes any other old default folder that holds no data. Observed: C:\Users\Warwick\AppData\Roaming\Radium Chat\data\db\__status__.db still there, 0 bytes, created and last written 2026-09-11 08:18 - so it was never removed, not removed and recreated. Ruled out: not locked, not read-only (attrs=Archive), owned by the user, and a copy deletes fine. The installed code is identical to the branch, and unit test removes_the_empty_radium_chat_folder_jan_cli_left_behind passes, so the cause is not known yet. HARMLESS in the meantime: no code in the installed build writes to that folder, and removing it by hand loses nothing.</t>
         </is>
       </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="6" t="inlineStr">
+        <is>
+          <t>T22-S01</t>
+        </is>
+      </c>
+      <c r="B167" s="17" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="C167" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" s="14" t="inlineStr">
+        <is>
+          <t>Get D28 answered: how API and Cloud should live in Settings</t>
+        </is>
+      </c>
+      <c r="E167" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F167" s="13" t="n"/>
+      <c r="G167" s="14" t="inlineStr">
+        <is>
+          <t>Decisions sheet D28. The user's call.</t>
+        </is>
+      </c>
+      <c r="H167" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I167" s="15" t="inlineStr">
+        <is>
+          <t>Do not start code until it is answered. | 2026-09-13: answered by the user - option B.</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="6" t="inlineStr">
+        <is>
+          <t>T22-S02</t>
+        </is>
+      </c>
+      <c r="B168" s="17" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="C168" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D168" s="14" t="inlineStr">
+        <is>
+          <t>Branch off main once PR #9 has merged</t>
+        </is>
+      </c>
+      <c r="E168" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F168" s="13" t="n"/>
+      <c r="G168" s="14" t="inlineStr">
+        <is>
+          <t>git switch -c feat/api-cloud-in-settings main (ask before creating it)</t>
+        </is>
+      </c>
+      <c r="H168" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I168" s="15" t="inlineStr">
+        <is>
+          <t>Keeps this out of the #8 / #9 stack.</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="6" t="inlineStr">
+        <is>
+          <t>T22-S03</t>
+        </is>
+      </c>
+      <c r="B169" s="17" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="C169" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D169" s="14" t="inlineStr">
+        <is>
+          <t>Write failing tests first</t>
+        </is>
+      </c>
+      <c r="E169" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F169" s="13" t="n"/>
+      <c r="G169" s="14" t="inlineStr">
+        <is>
+          <t>Sidebar test: no Cloud or API entry. Settings menu test: both entries present and route correctly. Route tests: old /api and /cloud addresses (and any outside link) still land on the right page. Run them and confirm they fail for the RIGHT reason.</t>
+        </is>
+      </c>
+      <c r="H169" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I169" s="15" t="inlineStr">
+        <is>
+          <t>Existing tests to extend: routes/api/__tests__, routes/cloud/__tests__, containers/__tests__/SettingsMenu.test.tsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="6" t="inlineStr">
+        <is>
+          <t>T22-S04</t>
+        </is>
+      </c>
+      <c r="B170" s="17" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="C170" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D170" s="14" t="inlineStr">
+        <is>
+          <t>Add API and Cloud to the Settings menu</t>
+        </is>
+      </c>
+      <c r="E170" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F170" s="13" t="n"/>
+      <c r="G170" s="14" t="inlineStr">
+        <is>
+          <t>containers/SettingsMenu.tsx, in the shape D28 chooses</t>
+        </is>
+      </c>
+      <c r="H170" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I170" s="15" t="inlineStr">
+        <is>
+          <t>Reuse the existing pages - do not rewrite them. | D28 = B: add Settings entries for the pages rendered inside the Settings layout at /settings/api and /settings/cloud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>T22-S05</t>
+        </is>
+      </c>
+      <c r="B171" s="17" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="C171" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D171" s="14" t="inlineStr">
+        <is>
+          <t>Remove Cloud and API from the sidebar</t>
+        </is>
+      </c>
+      <c r="E171" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F171" s="13" t="n"/>
+      <c r="G171" s="14" t="inlineStr">
+        <is>
+          <t>components/left-sidebar/NavMain.tsx</t>
+        </is>
+      </c>
+      <c r="H171" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I171" s="15" t="inlineStr">
+        <is>
+          <t>Media and the rest of the sidebar stay exactly as they are.</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="6" t="inlineStr">
+        <is>
+          <t>T22-S06</t>
+        </is>
+      </c>
+      <c r="B172" s="17" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="C172" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D172" s="14" t="inlineStr">
+        <is>
+          <t>Keep every existing link and old address working</t>
+        </is>
+      </c>
+      <c r="E172" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F172" s="13" t="n"/>
+      <c r="G172" s="14" t="inlineStr">
+        <is>
+          <t>DropdownModelProvider.tsx, LocalApiServerStatusRow.tsx, settings/providers/$providerName.tsx, settings/local-api-server.tsx, plus redirects from /api and /cloud if D28 moves the pages</t>
+        </is>
+      </c>
+      <c r="H172" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I172" s="15" t="inlineStr">
+        <is>
+          <t>A link that silently 404s is the likeliest regression. | D28 = B: /api and /cloud must redirect to /settings/api and /settings/cloud.</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="6" t="inlineStr">
+        <is>
+          <t>T22-S07</t>
+        </is>
+      </c>
+      <c r="B173" s="17" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="C173" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D173" s="14" t="inlineStr">
+        <is>
+          <t>Check every locale still has the labels</t>
+        </is>
+      </c>
+      <c r="E173" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F173" s="13" t="n"/>
+      <c r="G173" s="14" t="inlineStr">
+        <is>
+          <t>Settings menu titles exist in all 14 locales</t>
+        </is>
+      </c>
+      <c r="H173" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I173" s="15" t="inlineStr">
+        <is>
+          <t>New keys need the English default at least.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="6" t="inlineStr">
+        <is>
+          <t>T22-S08</t>
+        </is>
+      </c>
+      <c r="B174" s="17" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="C174" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D174" s="14" t="inlineStr">
+        <is>
+          <t>Full verification</t>
+        </is>
+      </c>
+      <c r="E174" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F174" s="13" t="n"/>
+      <c r="G174" s="14" t="inlineStr">
+        <is>
+          <t>web tests, typecheck, lint, test-quality, hardening contracts, make test-selective-v2032 (no re-baseline)</t>
+        </is>
+      </c>
+      <c r="H174" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I174" s="15" t="inlineStr">
+        <is>
+          <t>Run cargo and yarn commands directly under Git Bash.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>T22-S09</t>
+        </is>
+      </c>
+      <c r="B175" s="17" t="inlineStr">
+        <is>
+          <t>Task 22</t>
+        </is>
+      </c>
+      <c r="C175" s="6" t="n">
+        <v>9</v>
+      </c>
+      <c r="D175" s="14" t="inlineStr">
+        <is>
+          <t>Commit, PR, and a look in the real app</t>
+        </is>
+      </c>
+      <c r="E175" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F175" s="13" t="n"/>
+      <c r="G175" s="14" t="inlineStr">
+        <is>
+          <t>Commit and PR only with the user's authorisation; then a test build or dev run to see Settings with the new entries</t>
+        </is>
+      </c>
+      <c r="H175" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I175" s="15" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -9324,7 +9738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -10585,6 +10999,43 @@
         </is>
       </c>
       <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>D28</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>HOW SHOULD API AND CLOUD 'LIVE IN SETTINGS'? The user wants both out of the sidebar and inside Settings (Task 22). There are two reasonable shapes.</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Task 22 from S03 on.</t>
+        </is>
+      </c>
+      <c r="D35" s="14" t="inlineStr">
+        <is>
+          <t>Option B - show them inside Settings. (A) Settings menu entries that LINK to today's /api and /cloud pages: the smallest change and the fewest conflicts with upstream, but clicking one leaves the Settings layout, so it does not really feel like it lives in Settings. (B) Render the same pages INSIDE the Settings layout at /settings/api and /settings/cloud, with /api and /cloud redirecting there: it genuinely lives in Settings and old links keep working, at the cost of a few more changed files and more upstream merge conflicts. COST OF CHANGING LATER: low either way - A can become B later without breaking anything.</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>ANSWERED BY THE USER 2026-09-13: Option B. API and Cloud are rendered INSIDE the Settings layout at /settings/api and /settings/cloud, and the old /api and /cloud addresses redirect there so every existing link keeps working. Accepted cost: a few more changed files and more upstream merge conflicts than option A.</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): add Task 25, the upstream update gateway
The user asked on 2026-09-13 for a way to know, before an upstream update
is merged, what it would break or change in the work this fork has
built. D31 answered by the user: option A - a Fork features register
with a check per feature, a trial-merge report written to an Upstream
impact sheet in plain language, the user's decision on every flagged
row, and a gate that blocks the real merge until each row is decided.
Automatic stripping of upstream changes was rejected: it would also drop
upstream's bug and security fixes and can leave code that does not
build.

The need is measured, not assumed: the only guard hash-checks 9 media
files, while the fork differs from upstream v2.0.37 in 447 files. That
is how the v2.0.35 merge dropped the window controls (Task 23) without
anything failing. Task 25 must be in place before the next upstream
sync.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-13 (latest): URGENT FIRST - Task 23, the window has no Minimize/Maximize/Close buttons on main since the v2.0.35 merge. Get D30 answered, then fix on a branch off main. Then finish Task 21 (merge PR #8, retarget and merge PR #9), then Task 22 (D29 open) and Task 24. Ask before committing, pushing, merging or creating branches. | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
+          <t>2026-09-13 (latest): URGENT - Task 23 window controls (D30 = A) on a branch off main. Then finish Task 21 (merge PR #8, retarget and merge PR #9), then Tasks 22 and 24. Task 25, the upstream update gateway, must be in place before the NEXT upstream sync - no upstream merge without it. Ask before committing, pushing, merging or creating branches. | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
         </is>
       </c>
     </row>
@@ -1300,7 +1300,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2651,6 +2651,55 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>Task 25</t>
+        </is>
+      </c>
+      <c r="B28" s="11" t="inlineStr">
+        <is>
+          <t>12 - Upstream safety</t>
+        </is>
+      </c>
+      <c r="C28" s="14" t="inlineStr">
+        <is>
+          <t>Upstream update gateway: know, and decide, what an upstream update would break before it is merged</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="E28" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F28" s="13" t="n"/>
+      <c r="G28" s="14" t="inlineStr">
+        <is>
+          <t>D31 answered (option A). Nothing blocks it. It must be in place BEFORE the next upstream sync.</t>
+        </is>
+      </c>
+      <c r="H28" s="14" t="inlineStr">
+        <is>
+          <t>Every row on the Fork features sheet has a check that passes; a dry run against upstream fills the Upstream impact sheet; the gate refuses while any flagged row has no user decision and passes once all are decided; after a merge, every feature's check runs in make verify.</t>
+        </is>
+      </c>
+      <c r="I28" s="13" t="n"/>
+      <c r="J28" s="14" t="inlineStr">
+        <is>
+          <t>ADDED 2026-09-13 at the user's instruction: "we need to set an alert or a guard or some other method of knowing what updates will break or change things we've already done... when you're updating or planning on updating, the updates get passed through an Excel tracker gateway... or list, identify the changes or the repercussions of the changes onto the tracker and make the user fully aware." The user chose option A: the report AND a gate, not automatic stripping.</t>
+        </is>
+      </c>
+      <c r="K28" s="15" t="inlineStr">
+        <is>
+          <t>WHY, MEASURED 2026-09-13: the only guard today (scripts/verify-selective-v2032.mjs) hash-checks 9 media files and forbids Atomic Code paths and text. The fork differs from upstream v2.0.37 in 447 files, almost all unguarded. The window controls (Task 23) lived in web-app/src/routes/__root.tsx, which was not protected, and their only test rendered the component on its own - so the v2.0.35 merge dropped them and nothing failed. WHY NOT AUTO-STRIP: silently discarding upstream changes to a file also discards its bug and security fixes, and a half-removed change often does not build; the gateway stops and asks instead. BUILD NOTE: writing the .xlsx from a script needs either Python openpyxl (on this PC, not a repo dependency) or a Node library such as exceljs (a NEW dependency - AGENTS.md rule 6 requires the user's ok naming it). Settle in S04, ask first.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A2:K40"/>
   <dataValidations count="1">
@@ -2668,7 +2717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I188"/>
+  <dimension ref="A1:I195"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -10331,6 +10380,289 @@
         </is>
       </c>
       <c r="I188" s="15" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="6" t="inlineStr">
+        <is>
+          <t>T25-S01</t>
+        </is>
+      </c>
+      <c r="B189" s="17" t="inlineStr">
+        <is>
+          <t>Task 25</t>
+        </is>
+      </c>
+      <c r="C189" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D189" s="14" t="inlineStr">
+        <is>
+          <t>Record the approach (D31)</t>
+        </is>
+      </c>
+      <c r="E189" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F189" s="13" t="n"/>
+      <c r="G189" s="14" t="inlineStr">
+        <is>
+          <t>Decisions sheet D31: option A - report, user decision per row, gate, and a check per feature.</t>
+        </is>
+      </c>
+      <c r="H189" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I189" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-13: answered by the user.</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="6" t="inlineStr">
+        <is>
+          <t>T25-S02</t>
+        </is>
+      </c>
+      <c r="B190" s="17" t="inlineStr">
+        <is>
+          <t>Task 25</t>
+        </is>
+      </c>
+      <c r="C190" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D190" s="14" t="inlineStr">
+        <is>
+          <t>Build the Fork features register</t>
+        </is>
+      </c>
+      <c r="E190" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F190" s="13" t="n"/>
+      <c r="G190" s="14" t="inlineStr">
+        <is>
+          <t>New 'Fork features' sheet: ID, feature, what it does for the user, files it lives in (paths or globs), the check that proves it still works (test or command), decision or ADR, status. Seed it with everything built so far: Radium Media (the 9 protected files and the media paths), the product rename and data-folder migration, window controls, no auto-update, the Atomic Code removal, Windows backend bundling, assistant name migrations, and, as they land, Settings &gt; Chat, API and Cloud in Settings, and the Uncensored filter.</t>
+        </is>
+      </c>
+      <c r="H190" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I190" s="15" t="inlineStr">
+        <is>
+          <t>Flag every row that has no check yet - those are the gaps that let the window controls go.</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="6" t="inlineStr">
+        <is>
+          <t>T25-S03</t>
+        </is>
+      </c>
+      <c r="B191" s="17" t="inlineStr">
+        <is>
+          <t>Task 25</t>
+        </is>
+      </c>
+      <c r="C191" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D191" s="14" t="inlineStr">
+        <is>
+          <t>Give every feature a check that fails when it is gone</t>
+        </is>
+      </c>
+      <c r="E191" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F191" s="13" t="n"/>
+      <c r="G191" s="14" t="inlineStr">
+        <is>
+          <t>Add a test per unchecked row, starting with the window-controls mount test (T23-S03). Each check is run red once by removing the feature in a scratch copy, so it is known to catch the loss.</t>
+        </is>
+      </c>
+      <c r="H191" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I191" s="15" t="inlineStr">
+        <is>
+          <t>A check that cannot fail is not a check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="6" t="inlineStr">
+        <is>
+          <t>T25-S04</t>
+        </is>
+      </c>
+      <c r="B192" s="17" t="inlineStr">
+        <is>
+          <t>Task 25</t>
+        </is>
+      </c>
+      <c r="C192" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D192" s="14" t="inlineStr">
+        <is>
+          <t>Write the impact report script</t>
+        </is>
+      </c>
+      <c r="E192" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F192" s="13" t="n"/>
+      <c r="G192" s="14" t="inlineStr">
+        <is>
+          <t>scripts/upstream-impact: fetch upstream, trial-merge in a throwaway worktree and discard it, never touching the real branch. For each Fork features row: upstream commits touching its files, and whether each file is edited, conflicting or deleted; run the feature's check on the trial result. Write the 'Upstream impact' sheet: feature, what upstream changed (commits), kind, check result, plain-language consequence, recommendation, user decision (keep ours / take theirs / adapt), decided on. Tests against a small fake upstream repo.</t>
+        </is>
+      </c>
+      <c r="H192" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I192" s="15" t="inlineStr">
+        <is>
+          <t>Ask before adding any dependency (see the task notes).</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="6" t="inlineStr">
+        <is>
+          <t>T25-S05</t>
+        </is>
+      </c>
+      <c r="B193" s="17" t="inlineStr">
+        <is>
+          <t>Task 25</t>
+        </is>
+      </c>
+      <c r="C193" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D193" s="14" t="inlineStr">
+        <is>
+          <t>Build the gate</t>
+        </is>
+      </c>
+      <c r="E193" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F193" s="13" t="n"/>
+      <c r="G193" s="14" t="inlineStr">
+        <is>
+          <t>A make target that reads the Upstream impact sheet and exits non-zero while any flagged row has no user decision, naming the rows. After a merge, make verify runs every Fork features check. Tests for both: refuses with one unanswered row, passes when all are answered.</t>
+        </is>
+      </c>
+      <c r="H193" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I193" s="15" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="6" t="inlineStr">
+        <is>
+          <t>T25-S06</t>
+        </is>
+      </c>
+      <c r="B194" s="17" t="inlineStr">
+        <is>
+          <t>Task 25</t>
+        </is>
+      </c>
+      <c r="C194" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D194" s="14" t="inlineStr">
+        <is>
+          <t>Make it the only way to sync upstream</t>
+        </is>
+      </c>
+      <c r="E194" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F194" s="13" t="n"/>
+      <c r="G194" s="14" t="inlineStr">
+        <is>
+          <t>AGENTS.md rule, a DEVELOP.md upstream-sync section and a tracker README item: no upstream merge without the report, the user's decisions and a green gate. ADR in docs/decisions with an INDEX entry.</t>
+        </is>
+      </c>
+      <c r="H194" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I194" s="15" t="inlineStr">
+        <is>
+          <t>Keep AGENTS.md under its size limit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="6" t="inlineStr">
+        <is>
+          <t>T25-S07</t>
+        </is>
+      </c>
+      <c r="B195" s="17" t="inlineStr">
+        <is>
+          <t>Task 25</t>
+        </is>
+      </c>
+      <c r="C195" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D195" s="14" t="inlineStr">
+        <is>
+          <t>Dry run against upstream and review it with the user</t>
+        </is>
+      </c>
+      <c r="E195" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F195" s="13" t="n"/>
+      <c r="G195" s="14" t="inlineStr">
+        <is>
+          <t>Run the report against upstream/main now, walk the user through every flagged row in plain language, and record their decisions. Commit and PR only with the user's authorisation.</t>
+        </is>
+      </c>
+      <c r="H195" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I195" s="15" t="inlineStr">
+        <is>
+          <t>This is the proof the gateway works before it is needed for real.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -10349,7 +10681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G37"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -11721,6 +12053,43 @@
         </is>
       </c>
       <c r="G37" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>D31</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="inlineStr">
+        <is>
+          <t>HOW SHOULD WE KNOW WHAT AN UPSTREAM UPDATE WOULD BREAK OR CHANGE IN WHAT WE HAVE BUILT? (Task 25)</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>Every future upstream sync.</t>
+        </is>
+      </c>
+      <c r="D38" s="14" t="inlineStr">
+        <is>
+          <t>Option A: a Fork features register with a check per feature; before any sync, a trial merge fills an Upstream impact sheet in plain language; the user decides each flagged row (keep ours, take theirs, adapt); a gate blocks the real merge until every row is decided; after the merge every feature's check runs. Option B: the report only - makes the user aware but blocks nothing. Automatic stripping of upstream changes was rejected: it would also drop upstream's bug and security fixes and can leave code that does not build.</t>
+        </is>
+      </c>
+      <c r="E38" s="15" t="inlineStr">
+        <is>
+          <t>ANSWERED BY THE USER 2026-09-13: Option A.</t>
+        </is>
+      </c>
+      <c r="F38" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G38" s="13" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): record Task 23 progress and the T21-S14 fix
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1189,7 +1189,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-13 (latest): URGENT - Task 23 window controls (D30 = A) on a branch off main. Then finish Task 21 (merge PR #8, retarget and merge PR #9), then Tasks 22 and 24. Task 25, the upstream update gateway, must be in place before the NEXT upstream sync - no upstream merge without it. Ask before committing, pushing, merging or creating branches. | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
+          <t>2026-09-13 (latest): Task 23 fix is in PR #10; install the test build from run 34790472605 and check the window bar (T23-S05). T21-S14 fixed in code on PR #9. Then merge #8, retarget and merge #9, rebase and merge #10. Then Task 24, Task 22, Task 25. The user has authorised acting without asking (2026-09-13). | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="E26" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F26" s="13" t="n"/>
@@ -2590,7 +2590,11 @@
           <t>On Windows the app can be minimised, maximised/restored, closed, moved and resized again, and a test fails if the controls ever stop being rendered.</t>
         </is>
       </c>
-      <c r="I26" s="13" t="n"/>
+      <c r="I26" s="13" t="inlineStr">
+        <is>
+          <t>d692991dd (PR #10)</t>
+        </is>
+      </c>
       <c r="J26" s="14" t="inlineStr">
         <is>
           <t>ADDED 2026-09-13 at the user's instruction: "somewhere along the way we lost ... the x to close the window, the minimize window button and the resize button. These need to be worked back into the app. It's kind of an app breaking feature. Can't resize or close the app." Windows' own names: Minimize, Maximize (Restore Down when maximised) and Close, together the caption buttons or window controls.</t>
@@ -9483,7 +9487,7 @@
       </c>
       <c r="E166" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F166" s="13" t="n"/>
@@ -9499,7 +9503,7 @@
       </c>
       <c r="I166" s="15" t="inlineStr">
         <is>
-          <t>FOUND 2026-09-13 on the install test. Expected: after 'Moved the data folder', the cleanup loop in data_migration.rs (lines 141-150 at 4402b9749) deletes any other old default folder that holds no data. Observed: C:\Users\Warwick\AppData\Roaming\Radium Chat\data\db\__status__.db still there, 0 bytes, created and last written 2026-09-11 08:18 - so it was never removed, not removed and recreated. Ruled out: not locked, not read-only (attrs=Archive), owned by the user, and a copy deletes fine. The installed code is identical to the branch, and unit test removes_the_empty_radium_chat_folder_jan_cli_left_behind passes, so the cause is not known yet. HARMLESS in the meantime: no code in the installed build writes to that folder, and removing it by hand loses nothing.</t>
+          <t>FOUND 2026-09-13 on the install test. Expected: after 'Moved the data folder', the cleanup loop in data_migration.rs (lines 141-150 at 4402b9749) deletes any other old default folder that holds no data. Observed: C:\Users\Warwick\AppData\Roaming\Radium Chat\data\db\__status__.db still there, 0 bytes, created and last written 2026-09-11 08:18 - so it was never removed, not removed and recreated. Ruled out: not locked, not read-only (attrs=Archive), owned by the user, and a copy deletes fine. The installed code is identical to the branch, and unit test removes_the_empty_radium_chat_folder_jan_cli_left_behind passes, so the cause is not known yet. HARMLESS in the meantime: no code in the installed build writes to that folder, and removing it by hand loses nothing. | 2026-09-13: FIXED IN CODE, commit 15438a573 on feat/radium-product-name. Cause at that moment still unknown (not locked or read-only afterwards), so the fix is robust rather than a guess: cleanup now runs on every launch while the data lives at the new default, and every old folder is logged as Removed, HoldsData or Failed with the error. Tests first; 18 migration tests pass; clippy clean. Done once an installed build logs 'Removed the empty old data folder ...\Radium Chat\data' on this PC.</t>
         </is>
       </c>
     </row>
@@ -10053,7 +10057,7 @@
       </c>
       <c r="E180" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F180" s="13" t="n"/>
@@ -10067,7 +10071,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I180" s="15" t="n"/>
+      <c r="I180" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-13: branch fix/window-controls off main (f8f2d173e), user authorised.</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="6" t="inlineStr">
@@ -10090,7 +10098,7 @@
       </c>
       <c r="E181" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F181" s="13" t="n"/>
@@ -10106,7 +10114,7 @@
       </c>
       <c r="I181" s="15" t="inlineStr">
         <is>
-          <t>The existing WindowControls.test.tsx renders the component on its own, so it kept passing while nothing showed it. This test is the one that would have caught the loss.</t>
+          <t>The existing WindowControls.test.tsx renders the component on its own, so it kept passing while nothing showed it. This test is the one that would have caught the loss. | 2026-09-13: tests/window-controls.test.mjs (wiring contract, in make test-hardening-contracts) and components/__tests__/WindowFrame.test.tsx, both run RED first for the right reason. DEVIATION: a full render of the root layout was not practical (it mounts every provider), so the contract pins the wiring from source instead; each assertion was proved by removing that piece in a scratch copy.</t>
         </is>
       </c>
     </row>
@@ -10131,7 +10139,7 @@
       </c>
       <c r="E182" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F182" s="13" t="n"/>
@@ -10147,7 +10155,7 @@
       </c>
       <c r="I182" s="15" t="inlineStr">
         <is>
-          <t>D30 = A: re-mount WindowControls and the drag region in __root.tsx; decorations stays false.</t>
+          <t>D30 = A: re-mount WindowControls and the drag region in __root.tsx; decorations stays false. | 2026-09-13: components/WindowFrame.tsx + lib/window-chrome.ts, wrapped in routes/__root.tsx. FOUND ON THE WAY: 3b147addc's August bar never shortened ~25 full-height layouts (h-svh, min-h-svh, the fixed sidebar), so it would have cut the bottom off every page; index.css now does that inside the frame, and the contract test pins those rules too.</t>
         </is>
       </c>
     </row>
@@ -10213,7 +10221,7 @@
       </c>
       <c r="E184" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F184" s="13" t="n"/>
@@ -10227,7 +10235,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I184" s="15" t="n"/>
+      <c r="I184" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-13: web 3515 passed / 0 failed, typecheck clean, lint 0 errors, hardening contracts 36/36, test-quality pass, selective media guard verified (no re-baseline).</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="6" t="inlineStr">
@@ -10250,7 +10262,7 @@
       </c>
       <c r="E185" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F185" s="13" t="n"/>
@@ -10264,7 +10276,11 @@
           <t>This PC</t>
         </is>
       </c>
-      <c r="I185" s="15" t="n"/>
+      <c r="I185" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-13: commit d692991dd; PR #10 https://github.com/walladanger/Radium/pull/10 into main. Test build run 34790472605 on throwaway branch test/radium-window-controls (rename + fix, never to be merged; its Makefile hardening list lacks the window-controls test because a scripted conflict fix failed - harmless for a build). S05 (see it in a real window) waits for that installer.</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): record Task 22 and 24, the #8/#9 merges, and add Task 26 for Radium Media
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1037,6 +1037,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1069,7 +1070,7 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>2026-09-13: feat/radium-product-name (PR #9, Task 21) stacked on chore/upstream-v2.0.37 (PR #8, the v2.0.37 sync). Merge #8 first, then retarget #9 to main.</t>
+          <t>2026-09-13 (latest): feat/api-cloud-chat-in-settings (Task 22) off main. Open PRs: #10 fix/window-controls (Task 23), #11 feat/uncensored-in-filter-menu (Task 24). PR #8 and #9 are merged.</t>
         </is>
       </c>
     </row>
@@ -1081,7 +1082,7 @@
       </c>
       <c r="B7" s="22" t="inlineStr">
         <is>
-          <t>4402b9749 on feat/radium-product-name, pushed: chore(guard) re-baseline accepting MediaPreview.tsx. Before it: a22ac62da media wording, 1df96dc89 the rename, 810c0a48a the Task 21 tracker entry.</t>
+          <t>2026-09-13: Task 22 on feat/api-cloud-chat-in-settings - see the Tasks sheet for the SHA once committed.</t>
         </is>
       </c>
     </row>
@@ -1189,10 +1190,11 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-13 (latest): Task 23 fix is in PR #10; install the test build from run 34790472605 and check the window bar (T23-S05). T21-S14 fixed in code on PR #9. Then merge #8, retarget and merge #9, rebase and merge #10. Then Task 24, Task 22, Task 25. The user has authorised acting without asking (2026-09-13). | Earlier: Task 19 (upstream sync) is next, but land PR #3 then PR #2 into main first. The prerequisite the user set - Media untouched - is MECHANICAL, not a promise: T19-S05 runs make test-selective-v2032 before anything else, and a failure there means a protected file moved in the merge. Do NOT re-baseline the guard to make it pass; that would defeat the only check standing between an upstream merge and the media platform. Still waiting on hardware or another repo: one GPU generation (T17-S09, Evidence 8); the atomic-chat-conf PR (T15-S06); translators for 13 locales. KNOWN AND UNFIXED: the release build degrades src-tauri/icons/icon.png (149710 -&gt; 56994 bytes) by overwriting the master with a generated variant - the same failure c54856d2e was meant to prevent, so that fix does not cover the release path. Never commit that file after a release build.</t>
-        </is>
-      </c>
-    </row>
+          <t>2026-09-13 (latest): (1) the user installs the test build from run 34791322213 (PR #10) and checks the window bar (T23-S05) and the app log for T21-S14; then merge #10 and #11. (2) Review and merge the Task 22 PR. (3) Task 25 gateway before any upstream sync. (4) Task 26: get Radium Media actually generating.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -1300,7 +1302,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2500,7 +2502,7 @@
       </c>
       <c r="K24" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13 INSTALL TEST ON THIS PC: the rename and data move WORKED on real data - see T21-S12 for the measurements. Open: the user confirming a chat reply, and T21-S14 (the empty Radium Chat folder was not removed). Also recorded: D27, the Node.js 20 deprecation warning in the workflows. | Earlier: 2026-09-13 PROGRESS: S01-S11 Done and verified (see Steps). Open: S12 install test on this PC, S13 commit and PR - both wait for the user. STILL SAYING 'Radium Chat' OR 'Atomic Chat', each deliberate and reported to the user: media wording in MediaPreview.tsx (protected), MediaParamField.tsx, atomicWorker.ts and en/media.json (D25); the entry name Radium writes into Zed and Droid, which their config uses as a lookup key; LICENSE header (legal - user's call); the sidebar wordmark in AppLogo.tsx, drawn as SVG and owned by the separate wordmark task. PRE-EXISTING, found on the way, not fixed: CLI_OWNERSHIP_MARKER is b"Radium Chat" since D13, but the legacy jan binaries it is meant to recognise would contain 'Atomic Chat'; src-tauri/tauri.bundle.windows.nsis.template is not referenced by any build config. | Earlier: 2026-09-13, STATE BEFORE CODE STARTS, stated plainly. DONE: GitHub repo renamed walladanger/Atomic-Chat -&gt; walladanger/Radium, authorised by the user; local origin repointed; PR #8 and Windows test build run 34761971349 followed the rename and old URLs redirect. NOT DONE, DRAFT ONLY: branch feat/radium-product-name (off chore/upstream-v2.0.37 at 6c3909482) holds UNCOMMITTED edits written for 'Radium Chat' - a data-folder migration module with 11 unit tests, an NSIS pre-install hook, a launch-at-startup migration command, a contract test, an ADR and doc edits. NONE OF IT HAS BEEN COMPILED OR RUN. It will be re-targeted to 'Radium' and verified from scratch, not trusted as written. THE AGENT CREATED THAT BRANCH WITHOUT ASKING, which the working agreement forbids; recorded here rather than hidden. MEASURED ON THIS PC, not assumed: the data folder C:\Users\Warwick\AppData\Roaming\Atomic Chat\data is 3.4 GB and stores no absolute path to itself (model.yml paths are relative), so a same-volume rename is safe. BOTH settings.json files - %APPDATA%\chat.atomic.app and the legacy %APPDATA%\Atomic-Chat, which wins while it exists - name that path, so changing productName alone moves nothing and the migration must repoint both. The installed app is an MSI (v2.0.23, WiX key {64542677-4056-4D46-BBEE-094163B8EC1A}): the MSI channel upgrades in place because its upgradeCode is pinned, but the NSIS installer finds a previous install by productName and would install side by side without a pre-install hook. A stray, empty %APPDATA%\Radium Chat\data (one 0-byte db file, made by jan-cli) exists - see D26. Launch-at-startup is OFF on this PC today. MEDIA: nothing in this task needs a protected file, and the guard must pass untouched.</t>
+          <t>2026-09-13 INSTALL TEST ON THIS PC: the rename and data move WORKED on real data - see T21-S12 for the measurements. Open: the user confirming a chat reply, and T21-S14 (the empty Radium Chat folder was not removed). Also recorded: D27, the Node.js 20 deprecation warning in the workflows. | Earlier: 2026-09-13 PROGRESS: S01-S11 Done and verified (see Steps). Open: S12 install test on this PC, S13 commit and PR - both wait for the user. STILL SAYING 'Radium Chat' OR 'Atomic Chat', each deliberate and reported to the user: media wording in MediaPreview.tsx (protected), MediaParamField.tsx, atomicWorker.ts and en/media.json (D25); the entry name Radium writes into Zed and Droid, which their config uses as a lookup key; LICENSE header (legal - user's call); the sidebar wordmark in AppLogo.tsx, drawn as SVG and owned by the separate wordmark task. PRE-EXISTING, found on the way, not fixed: CLI_OWNERSHIP_MARKER is b"Radium Chat" since D13, but the legacy jan binaries it is meant to recognise would contain 'Atomic Chat'; src-tauri/tauri.bundle.windows.nsis.template is not referenced by any build config. | Earlier: 2026-09-13, STATE BEFORE CODE STARTS, stated plainly. DONE: GitHub repo renamed walladanger/Atomic-Chat -&gt; walladanger/Radium, authorised by the user; local origin repointed; PR #8 and Windows test build run 34761971349 followed the rename and old URLs redirect. NOT DONE, DRAFT ONLY: branch feat/radium-product-name (off chore/upstream-v2.0.37 at 6c3909482) holds UNCOMMITTED edits written for 'Radium Chat' - a data-folder migration module with 11 unit tests, an NSIS pre-install hook, a launch-at-startup migration command, a contract test, an ADR and doc edits. NONE OF IT HAS BEEN COMPILED OR RUN. It will be re-targeted to 'Radium' and verified from scratch, not trusted as written. THE AGENT CREATED THAT BRANCH WITHOUT ASKING, which the working agreement forbids; recorded here rather than hidden. MEASURED ON THIS PC, not assumed: the data folder C:\Users\Warwick\AppData\Roaming\Atomic Chat\data is 3.4 GB and stores no absolute path to itself (model.yml paths are relative), so a same-volume rename is safe. BOTH settings.json files - %APPDATA%\chat.atomic.app and the legacy %APPDATA%\Atomic-Chat, which wins while it exists - name that path, so changing productName alone moves nothing and the migration must repoint both. The installed app is an MSI (v2.0.23, WiX key {64542677-4056-4D46-BBEE-094163B8EC1A}): the MSI channel upgrades in place because its upgradeCode is pinned, but the NSIS installer finds a previous install by productName and would install side by side without a pre-install hook. A stray, empty %APPDATA%\Radium Chat\data (one 0-byte db file, made by jan-cli) exists - see D26. Launch-at-startup is OFF on this PC today. MEDIA: nothing in this task needs a protected file, and the guard must pass untouched. | 2026-09-13: PR #8 (v2.0.37 sync) and PR #9 (the rename) are MERGED into main (eb28f890d). Open: T21-S14 needs an installed build to log the stray-folder cleanup.</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2529,7 @@
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F25" s="13" t="n"/>
@@ -2549,7 +2551,7 @@
       </c>
       <c r="K25" s="15" t="inlineStr">
         <is>
-          <t>SCOPE MEASURED 2026-09-13, not assumed. Today: web-app/src/components/left-sidebar/NavMain.tsx renders top-level Cloud (route.cloud.index = /cloud/, routes/cloud/index.tsx, 243 lines, the cloud provider registry) and API (route.api.index = /api/, routes/api/index.tsx, 148 lines, the local API server page). Upstream put them there DELIBERATELY in d887d3817 (Mike, 2026-09-03, 'Improve/agent flow #265'): /settings/local-api-server now only redirects to /api, and Settings &gt; Model providers &gt; a provider navigates to /cloud. OTHER PLACES THAT LINK TO THEM and must keep working: containers/DropdownModelProvider.tsx (to /cloud), containers/LocalApiServerStatusRow.tsx (to /api), routes/settings/providers/$providerName.tsx (to /cloud), routes/settings/local-api-server.tsx (redirect to /api). Settings menu: containers/SettingsMenu.tsx. MERGE COST: this reverses an upstream design choice, so NavMain.tsx, SettingsMenu.tsx and constants/routes.ts will conflict on upstream syncs that touch them. They differ from v2.0.37 today by only +18, +6 and +3 lines, so keep the change small and in as few upstream files as possible. MEDIA: none of these files is protected, and Media stays in the sidebar. | CHAT SETTINGS, MEASURED 2026-09-13: that panel is web-app/src/containers/RunSettingsPanel.tsx (446 lines), opened from AgentWorkspaceLayout.tsx via stores/run-settings-panel-store; it has its own tests (containers/RunSettingsPanel.test.tsx). It mixes two kinds of setting: per-ASSISTANT (system prompt, sampling, penalties) and per-MODEL (context size, advanced load options). Settings already has an Assistants page (routes/settings/assistant.tsx, 197 lines) that lists and edits assistants - the obvious neighbour. Not protected; no media file involved.</t>
+          <t>SCOPE MEASURED 2026-09-13, not assumed. Today: web-app/src/components/left-sidebar/NavMain.tsx renders top-level Cloud (route.cloud.index = /cloud/, routes/cloud/index.tsx, 243 lines, the cloud provider registry) and API (route.api.index = /api/, routes/api/index.tsx, 148 lines, the local API server page). Upstream put them there DELIBERATELY in d887d3817 (Mike, 2026-09-03, 'Improve/agent flow #265'): /settings/local-api-server now only redirects to /api, and Settings &gt; Model providers &gt; a provider navigates to /cloud. OTHER PLACES THAT LINK TO THEM and must keep working: containers/DropdownModelProvider.tsx (to /cloud), containers/LocalApiServerStatusRow.tsx (to /api), routes/settings/providers/$providerName.tsx (to /cloud), routes/settings/local-api-server.tsx (redirect to /api). Settings menu: containers/SettingsMenu.tsx. MERGE COST: this reverses an upstream design choice, so NavMain.tsx, SettingsMenu.tsx and constants/routes.ts will conflict on upstream syncs that touch them. They differ from v2.0.37 today by only +18, +6 and +3 lines, so keep the change small and in as few upstream files as possible. MEDIA: none of these files is protected, and Media stays in the sidebar. | CHAT SETTINGS, MEASURED 2026-09-13: that panel is web-app/src/containers/RunSettingsPanel.tsx (446 lines), opened from AgentWorkspaceLayout.tsx via stores/run-settings-panel-store; it has its own tests (containers/RunSettingsPanel.test.tsx). It mixes two kinds of setting: per-ASSISTANT (system prompt, sampling, penalties) and per-MODEL (context size, advanced load options). Settings already has an Assistants page (routes/settings/assistant.tsx, 197 lines) that lists and edits assistants - the obvious neighbour. Not protected; no media file involved. | 2026-09-13: BUILT on feat/api-cloud-chat-in-settings off main (eb28f890d). Settings menu gains Chat, Cloud and API. /settings/api and /settings/cloud render the existing pages inside the Settings frame (new SettingsPageLayout); /api, /cloud (keeping ?provider) and /settings/local-api-server redirect there. Cloud and API left the sidebar. Settings &gt; Chat shows the run settings panel's own controls; the chat's sliders button now opens that page, and the side panel, its store and the model pill's fold-down (which only existed for that panel) are gone.</t>
         </is>
       </c>
     </row>
@@ -2602,7 +2604,7 @@
       </c>
       <c r="K26" s="15" t="inlineStr">
         <is>
-          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision.</t>
+          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision. | 2026-09-13: PR #10 (fix/window-controls, head 229d2352b) now includes main, so its test build has the rename, the T21-S14 fix and the window controls together - run 34791322213. Waiting on: the user installs it and checks T23-S05.</t>
         </is>
       </c>
     </row>
@@ -2629,7 +2631,7 @@
       </c>
       <c r="E27" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F27" s="13" t="n"/>
@@ -2643,7 +2645,11 @@
           <t>Uncensored appears inside the Sort filter menu with the other checkboxes, works the same, and tests cover it.</t>
         </is>
       </c>
-      <c r="I27" s="13" t="n"/>
+      <c r="I27" s="13" t="inlineStr">
+        <is>
+          <t>85f5c0779 (PR #11)</t>
+        </is>
+      </c>
       <c r="J27" s="14" t="inlineStr">
         <is>
           <t>ADDED 2026-09-13 at the user's instruction: "add or move the check button for uncensored into the already made download filter panel".</t>
@@ -2651,7 +2657,7 @@
       </c>
       <c r="K27" s="15" t="inlineStr">
         <is>
-          <t>MEASURED 2026-09-13: web-app/src/containers/hub/HubFilters.tsx renders Uncensored as a standalone checkbox button next to the Sort menu. That menu already holds 'Installed on this device' and 'Only show models that fit' as DropdownMenuCheckboxItems, so Uncensored becomes a third one. State is state.uncensored in lib/hub-filters.ts, already saved - no data change.</t>
+          <t>MEASURED 2026-09-13: web-app/src/containers/hub/HubFilters.tsx renders Uncensored as a standalone checkbox button next to the Sort menu. That menu already holds 'Installed on this device' and 'Only show models that fit' as DropdownMenuCheckboxItems, so Uncensored becomes a third one. State is state.uncensored in lib/hub-filters.ts, already saved - no data change. | 2026-09-13: DONE on feat/uncensored-in-filter-menu off main. Uncensored is a checkbox item in the Sort filter menu, keeps its hover hint and keeps the menu open. PR https://github.com/walladanger/Radium/pull/11.</t>
         </is>
       </c>
     </row>
@@ -2703,6 +2709,51 @@
           <t>WHY, MEASURED 2026-09-13: the only guard today (scripts/verify-selective-v2032.mjs) hash-checks 9 media files and forbids Atomic Code paths and text. The fork differs from upstream v2.0.37 in 447 files, almost all unguarded. The window controls (Task 23) lived in web-app/src/routes/__root.tsx, which was not protected, and their only test rendered the component on its own - so the v2.0.35 merge dropped them and nothing failed. WHY NOT AUTO-STRIP: silently discarding upstream changes to a file also discards its bug and security fixes, and a half-removed change often does not build; the gateway stops and asks instead. BUILD NOTE: writing the .xlsx from a script needs either Python openpyxl (on this PC, not a repo dependency) or a Node library such as exceljs (a NEW dependency - AGENTS.md rule 6 requires the user's ok naming it). Settle in S04, ask first.</t>
         </is>
       </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>Task 26</t>
+        </is>
+      </c>
+      <c r="B29" s="11" t="inlineStr">
+        <is>
+          <t>13 - Media</t>
+        </is>
+      </c>
+      <c r="C29" s="14" t="inlineStr">
+        <is>
+          <t>Get Radium Media generating end to end</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="inlineStr">
+        <is>
+          <t>This PC for images; an NVIDIA 24 GB machine for video</t>
+        </is>
+      </c>
+      <c r="E29" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F29" s="13" t="inlineStr"/>
+      <c r="G29" s="14" t="inlineStr">
+        <is>
+          <t>Nothing for the image path. Video needs suitable hardware.</t>
+        </is>
+      </c>
+      <c r="H29" s="14" t="inlineStr">
+        <is>
+          <t>An image generated from Radium Media on this PC through ComfyUI, saved to the media library; a documented, tested path for video.</t>
+        </is>
+      </c>
+      <c r="I29" s="13" t="inlineStr"/>
+      <c r="J29" s="14" t="inlineStr">
+        <is>
+          <t>ADDED 2026-09-13 after the user asked how to get Radium Media running and whether any model can now be downloaded and used. MEASURED ANSWER: Radium Media does not run media models itself. It talks to an engine through adapters (Radium Media Worker at 127.0.0.1:13420 - not installed on this PC and not published; ComfyUI - two text-to-image workflow templates, uses whatever checkpoints ComfyUI has; OpenAI-compatible images / custom HTTP - declared model gpt-image-1, needs a key and costs money). 'Model agnostic' means the engine is pluggable, not that Radium downloads and runs any media model the way it does chat models. The remote media registry (Task 15) is not implemented and its URL returns 404. No end-to-end generation has ever run. This PC (AMD integrated GPU, 14.8 GB RAM) cannot run Wan 2.2 video (needs a ~24 GB NVIDIA GPU).</t>
+        </is>
+      </c>
+      <c r="K29" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:K40"/>
@@ -2721,7 +2772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I195"/>
+  <dimension ref="A1:I200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9446,7 +9497,7 @@
       </c>
       <c r="E165" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F165" s="13" t="n"/>
@@ -9462,7 +9513,7 @@
       </c>
       <c r="I165" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13: commits 1df96dc89 (rename), a22ac62da (media wording, D25 amendment) and 4402b9749 (isolated guard re-baseline accepting only MediaPreview.tsx), each authorised by the user. Pushed, and PR #9 opened with the user's authorisation: https://github.com/walladanger/Radium/pull/9, base chore/upstream-v2.0.37, 4 commits, mergeable. Stays open until PR #8 merges and #9 is retargeted to main and merged. This tracker update is itself uncommitted until the user says so.</t>
+          <t>2026-09-13: commits 1df96dc89 (rename), a22ac62da (media wording, D25 amendment) and 4402b9749 (isolated guard re-baseline accepting only MediaPreview.tsx), each authorised by the user. Pushed, and PR #9 opened with the user's authorisation: https://github.com/walladanger/Radium/pull/9, base chore/upstream-v2.0.37, 4 commits, mergeable. Stays open until PR #8 merges and #9 is retargeted to main and merged. This tracker update is itself uncommitted until the user says so. | 2026-09-13: PR #9 merged into main at eb28f890d.</t>
         </is>
       </c>
     </row>
@@ -9503,7 +9554,7 @@
       </c>
       <c r="I166" s="15" t="inlineStr">
         <is>
-          <t>FOUND 2026-09-13 on the install test. Expected: after 'Moved the data folder', the cleanup loop in data_migration.rs (lines 141-150 at 4402b9749) deletes any other old default folder that holds no data. Observed: C:\Users\Warwick\AppData\Roaming\Radium Chat\data\db\__status__.db still there, 0 bytes, created and last written 2026-09-11 08:18 - so it was never removed, not removed and recreated. Ruled out: not locked, not read-only (attrs=Archive), owned by the user, and a copy deletes fine. The installed code is identical to the branch, and unit test removes_the_empty_radium_chat_folder_jan_cli_left_behind passes, so the cause is not known yet. HARMLESS in the meantime: no code in the installed build writes to that folder, and removing it by hand loses nothing. | 2026-09-13: FIXED IN CODE, commit 15438a573 on feat/radium-product-name. Cause at that moment still unknown (not locked or read-only afterwards), so the fix is robust rather than a guess: cleanup now runs on every launch while the data lives at the new default, and every old folder is logged as Removed, HoldsData or Failed with the error. Tests first; 18 migration tests pass; clippy clean. Done once an installed build logs 'Removed the empty old data folder ...\Radium Chat\data' on this PC.</t>
+          <t>FOUND 2026-09-13 on the install test. Expected: after 'Moved the data folder', the cleanup loop in data_migration.rs (lines 141-150 at 4402b9749) deletes any other old default folder that holds no data. Observed: C:\Users\Warwick\AppData\Roaming\Radium Chat\data\db\__status__.db still there, 0 bytes, created and last written 2026-09-11 08:18 - so it was never removed, not removed and recreated. Ruled out: not locked, not read-only (attrs=Archive), owned by the user, and a copy deletes fine. The installed code is identical to the branch, and unit test removes_the_empty_radium_chat_folder_jan_cli_left_behind passes, so the cause is not known yet. HARMLESS in the meantime: no code in the installed build writes to that folder, and removing it by hand loses nothing. | 2026-09-13: FIXED IN CODE, commit 15438a573 on feat/radium-product-name. Cause at that moment still unknown (not locked or read-only afterwards), so the fix is robust rather than a guess: cleanup now runs on every launch while the data lives at the new default, and every old folder is logged as Removed, HoldsData or Failed with the error. Tests first; 18 migration tests pass; clippy clean. Done once an installed build logs 'Removed the empty old data folder ...\Radium Chat\data' on this PC. | 2026-09-13: FIXED IN CODE (15438a573 + rustfmt 9db0736fa, merged with PR #9): the cleanup now retries on every launch and logs its outcome. Done once an installed build logs 'Removed the empty old data folder ...Radium Chat\data'.</t>
         </is>
       </c>
     </row>
@@ -9569,7 +9620,7 @@
       </c>
       <c r="E168" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F168" s="13" t="n"/>
@@ -9585,7 +9636,7 @@
       </c>
       <c r="I168" s="15" t="inlineStr">
         <is>
-          <t>Keeps this out of the #8 / #9 stack.</t>
+          <t>Keeps this out of the #8 / #9 stack. | 2026-09-13: Branch feat/api-cloud-chat-in-settings off main eb28f890d, under the user's standing 'just act' instruction.</t>
         </is>
       </c>
     </row>
@@ -9610,7 +9661,7 @@
       </c>
       <c r="E169" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F169" s="13" t="n"/>
@@ -9626,7 +9677,7 @@
       </c>
       <c r="I169" s="15" t="inlineStr">
         <is>
-          <t>Existing tests to extend: routes/api/__tests__, routes/cloud/__tests__, containers/__tests__/SettingsMenu.test.tsx.</t>
+          <t>Existing tests to extend: routes/api/__tests__, routes/cloud/__tests__, containers/__tests__/SettingsMenu.test.tsx. | 2026-09-13: RED first for the right reasons: NavMain still showed Cloud/API; SettingsMenu had no Chat/Cloud/API; /api and /cloud rendered instead of redirecting; local-api-server went to /api; ApiPage had no settings menu; the chat button opened the side panel; the panel always showed a close button.</t>
         </is>
       </c>
     </row>
@@ -9651,7 +9702,7 @@
       </c>
       <c r="E170" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F170" s="13" t="n"/>
@@ -9667,7 +9718,7 @@
       </c>
       <c r="I170" s="15" t="inlineStr">
         <is>
-          <t>Reuse the existing pages - do not rewrite them. | D28 = B: add Settings entries for the pages rendered inside the Settings layout at /settings/api and /settings/cloud.</t>
+          <t>Reuse the existing pages - do not rewrite them. | D28 = B: add Settings entries for the pages rendered inside the Settings layout at /settings/api and /settings/cloud. | 2026-09-13: SettingsMenu: Chat after General; Cloud and API after Media. routes/settings/api.tsx and cloud.tsx reuse ApiPage and CloudPage unchanged apart from the frame.</t>
         </is>
       </c>
     </row>
@@ -9692,7 +9743,7 @@
       </c>
       <c r="E171" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F171" s="13" t="n"/>
@@ -9708,7 +9759,7 @@
       </c>
       <c r="I171" s="15" t="inlineStr">
         <is>
-          <t>Media and the rest of the sidebar stay exactly as they are.</t>
+          <t>Media and the rest of the sidebar stay exactly as they are. | 2026-09-13: NavMain: Cloud and API rows, their icons and refs removed. Media and everything else untouched.</t>
         </is>
       </c>
     </row>
@@ -9733,7 +9784,7 @@
       </c>
       <c r="E172" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F172" s="13" t="n"/>
@@ -9749,7 +9800,7 @@
       </c>
       <c r="I172" s="15" t="inlineStr">
         <is>
-          <t>A link that silently 404s is the likeliest regression. | D28 = B: /api and /cloud must redirect to /settings/api and /settings/cloud.</t>
+          <t>A link that silently 404s is the likeliest regression. | D28 = B: /api and /cloud must redirect to /settings/api and /settings/cloud. | 2026-09-13: Redirects: /api -&gt; /settings/api; /cloud -&gt; /settings/cloud with ?provider; /settings/local-api-server -&gt; /settings/api. Links repointed: LocalApiServerStatusRow, the model picker's gear, the $providerName redirect and the Cloud page's own navigation. routeTree.gen.ts regenerated (additions only).</t>
         </is>
       </c>
     </row>
@@ -9774,7 +9825,7 @@
       </c>
       <c r="E173" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F173" s="13" t="n"/>
@@ -9790,7 +9841,7 @@
       </c>
       <c r="I173" s="15" t="inlineStr">
         <is>
-          <t>New keys need the English default at least.</t>
+          <t>New keys need the English default at least. | 2026-09-13: New key common:chat added to all 14 locales (cloud and api keys already existed everywhere).</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9866,7 @@
       </c>
       <c r="E174" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F174" s="13" t="n"/>
@@ -9831,7 +9882,7 @@
       </c>
       <c r="I174" s="15" t="inlineStr">
         <is>
-          <t>Run cargo and yarn commands directly under Git Bash.</t>
+          <t>Run cargo and yarn commands directly under Git Bash. | 2026-09-13: PASS: web 297 files / 3467 passed / 0 failed; typecheck clean; ESLint 0 errors; test-quality pass (368 files); hardening contracts 40/40; selective media guard verified with NO re-baseline. Code commit 3d197f5e0.</t>
         </is>
       </c>
     </row>
@@ -9856,7 +9907,7 @@
       </c>
       <c r="E175" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F175" s="13" t="n"/>
@@ -9870,7 +9921,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I175" s="15" t="n"/>
+      <c r="I175" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-13: Commit and PR under the standing instruction; a look in the real app comes with the next test build.</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="6" t="inlineStr">
@@ -9934,7 +9989,7 @@
       </c>
       <c r="E177" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F177" s="13" t="n"/>
@@ -9950,7 +10005,7 @@
       </c>
       <c r="I177" s="15" t="inlineStr">
         <is>
-          <t>Per-assistant settings save to the assistant; per-model settings to the model - keep that split. | D29 = new Settings &gt; Chat page reusing RunSettingsPanel.tsx's controls.</t>
+          <t>Per-assistant settings save to the assistant; per-model settings to the model - keep that split. | D29 = new Settings &gt; Chat page reusing RunSettingsPanel.tsx's controls. | 2026-09-13: routes/settings/chat.tsx renders RunSettingsPanel inside SettingsPageLayout. Assistant settings still save to the assistant and model settings to the model - same code.</t>
         </is>
       </c>
     </row>
@@ -9975,7 +10030,7 @@
       </c>
       <c r="E178" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F178" s="13" t="n"/>
@@ -9991,7 +10046,7 @@
       </c>
       <c r="I178" s="15" t="inlineStr">
         <is>
-          <t>D29 = the in-chat panel becomes a shortcut that opens Settings &gt; Chat.</t>
+          <t>D29 = the in-chat panel becomes a shortcut that opens Settings &gt; Chat. | 2026-09-13: AgentWorkspaceLayout: the sliders button navigates to /settings/chat; the right column holds only files. run-settings-panel-store deleted; DropdownModelProvider's compact fold (both side bars open) removed with its test. RunSettingsPanel.onClose is optional.</t>
         </is>
       </c>
     </row>
@@ -10278,7 +10333,7 @@
       </c>
       <c r="I185" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13: commit d692991dd; PR #10 https://github.com/walladanger/Radium/pull/10 into main. Test build run 34790472605 on throwaway branch test/radium-window-controls (rename + fix, never to be merged; its Makefile hardening list lacks the window-controls test because a scripted conflict fix failed - harmless for a build). S05 (see it in a real window) waits for that installer.</t>
+          <t>2026-09-13: commit d692991dd; PR #10 https://github.com/walladanger/Radium/pull/10 into main. Test build run 34790472605 on throwaway branch test/radium-window-controls (rename + fix, never to be merged; its Makefile hardening list lacks the window-controls test because a scripted conflict fix failed - harmless for a build). S05 (see it in a real window) waits for that installer. | 2026-09-13: main merged into fix/window-controls (229d2352b); full test build run 34791322213 started. Merge PR #10 after the user's check on this PC.</t>
         </is>
       </c>
     </row>
@@ -10303,7 +10358,7 @@
       </c>
       <c r="E186" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F186" s="13" t="n"/>
@@ -10319,7 +10374,7 @@
       </c>
       <c r="I186" s="15" t="inlineStr">
         <is>
-          <t>Keep the hover hint (hub:uncensoredHint) somewhere visible, e.g. as the item's description.</t>
+          <t>Keep the hover hint (hub:uncensoredHint) somewhere visible, e.g. as the item's description. | 2026-09-13: HubFilters.tsx: the standalone button became a DropdownMenuCheckboxItem after the fit filter; hint kept as the item's title.</t>
         </is>
       </c>
     </row>
@@ -10344,7 +10399,7 @@
       </c>
       <c r="E187" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F187" s="13" t="n"/>
@@ -10358,7 +10413,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I187" s="15" t="n"/>
+      <c r="I187" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-13: The bar-checkbox test was replaced by two menu tests, both seen RED before the change.</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="6" t="inlineStr">
@@ -10381,7 +10440,7 @@
       </c>
       <c r="E188" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F188" s="13" t="n"/>
@@ -10395,7 +10454,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I188" s="15" t="n"/>
+      <c r="I188" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-13: Hub filter, Hub page and hub-filters tests 65/65, typecheck clean, ESLint clean, test-quality pass. Commit 85f5c0779, PR #11. Authorised by the user's standing instruction 'ok to everything ... just act'.</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="6" t="inlineStr">
@@ -10677,6 +10740,207 @@
       <c r="I195" s="15" t="inlineStr">
         <is>
           <t>This is the proof the gateway works before it is needed for real.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="6" t="inlineStr">
+        <is>
+          <t>T26-S01</t>
+        </is>
+      </c>
+      <c r="B196" s="17" t="inlineStr">
+        <is>
+          <t>Task 26</t>
+        </is>
+      </c>
+      <c r="C196" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D196" s="14" t="inlineStr">
+        <is>
+          <t>Install ComfyUI and one small image checkpoint on this PC</t>
+        </is>
+      </c>
+      <c r="E196" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F196" s="13" t="inlineStr"/>
+      <c r="G196" s="14" t="inlineStr">
+        <is>
+          <t>ComfyUI portable (CPU or DirectML for AMD); an SD 1.5-class checkpoint; start it on 127.0.0.1:8188</t>
+        </is>
+      </c>
+      <c r="H196" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I196" s="15" t="inlineStr">
+        <is>
+          <t>The user's install - Radium does not bundle it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="6" t="inlineStr">
+        <is>
+          <t>T26-S02</t>
+        </is>
+      </c>
+      <c r="B197" s="17" t="inlineStr">
+        <is>
+          <t>Task 26</t>
+        </is>
+      </c>
+      <c r="C197" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D197" s="14" t="inlineStr">
+        <is>
+          <t>Add ComfyUI as a media provider in Settings &gt; Media and generate one image</t>
+        </is>
+      </c>
+      <c r="E197" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F197" s="13" t="inlineStr"/>
+      <c r="G197" s="14" t="inlineStr">
+        <is>
+          <t>Provider type ComfyUI, base URL http://127.0.0.1:8188; pick the checkpoint; generate</t>
+        </is>
+      </c>
+      <c r="H197" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I197" s="15" t="inlineStr">
+        <is>
+          <t>First ever end-to-end run - record what breaks.</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="6" t="inlineStr">
+        <is>
+          <t>T26-S03</t>
+        </is>
+      </c>
+      <c r="B198" s="17" t="inlineStr">
+        <is>
+          <t>Task 26</t>
+        </is>
+      </c>
+      <c r="C198" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D198" s="14" t="inlineStr">
+        <is>
+          <t>Fix what the first run exposes, tests first</t>
+        </is>
+      </c>
+      <c r="E198" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F198" s="13" t="inlineStr"/>
+      <c r="G198" s="14" t="inlineStr">
+        <is>
+          <t>Adapter, polling, saving to the library</t>
+        </is>
+      </c>
+      <c r="H198" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I198" s="15" t="inlineStr"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="6" t="inlineStr">
+        <is>
+          <t>T26-S04</t>
+        </is>
+      </c>
+      <c r="B199" s="17" t="inlineStr">
+        <is>
+          <t>Task 26</t>
+        </is>
+      </c>
+      <c r="C199" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D199" s="14" t="inlineStr">
+        <is>
+          <t>Add a ComfyUI video workflow template (Wan 2.2) behind a hardware check</t>
+        </is>
+      </c>
+      <c r="E199" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F199" s="13" t="inlineStr"/>
+      <c r="G199" s="14" t="inlineStr">
+        <is>
+          <t>comfyWorkflows.ts template + tests; refuse clearly below the VRAM floor</t>
+        </is>
+      </c>
+      <c r="H199" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I199" s="15" t="inlineStr">
+        <is>
+          <t>Only usable on an NVIDIA ~24 GB machine.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="6" t="inlineStr">
+        <is>
+          <t>T26-S05</t>
+        </is>
+      </c>
+      <c r="B200" s="17" t="inlineStr">
+        <is>
+          <t>Task 26</t>
+        </is>
+      </c>
+      <c r="C200" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D200" s="14" t="inlineStr">
+        <is>
+          <t>Decide the Radium Media Worker's future: package it, or retire it in favour of ComfyUI</t>
+        </is>
+      </c>
+      <c r="E200" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F200" s="13" t="inlineStr"/>
+      <c r="G200" s="14" t="inlineStr">
+        <is>
+          <t>New decision on the Decisions sheet</t>
+        </is>
+      </c>
+      <c r="H200" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I200" s="15" t="inlineStr">
+        <is>
+          <t>The worker is not published anywhere today.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): record Task 25, add the Fork features and Upstream impact sheets and D32
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -12,6 +12,8 @@
     <sheet name="Steps" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Decisions" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Evidence" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Fork features" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Upstream impact" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Tasks'!$A$2:$K$40</definedName>
@@ -174,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -228,6 +230,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1070,7 +1073,7 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>2026-09-13 (latest): feat/api-cloud-chat-in-settings (Task 22) off main. Open PRs: #10 fix/window-controls (Task 23), #11 feat/uncensored-in-filter-menu (Task 24). PR #8 and #9 are merged.</t>
+          <t>2026-09-13 (latest): feat/upstream-gateway (Task 25) stacked on feat/api-cloud-chat-in-settings (Task 22, PR #12). Open PRs: #10 window controls, #11 Uncensored filter, #12 Task 22, and the Task 25 PR. PR #8 and #9 merged.</t>
         </is>
       </c>
     </row>
@@ -2706,7 +2709,7 @@
       </c>
       <c r="K28" s="15" t="inlineStr">
         <is>
-          <t>WHY, MEASURED 2026-09-13: the only guard today (scripts/verify-selective-v2032.mjs) hash-checks 9 media files and forbids Atomic Code paths and text. The fork differs from upstream v2.0.37 in 447 files, almost all unguarded. The window controls (Task 23) lived in web-app/src/routes/__root.tsx, which was not protected, and their only test rendered the component on its own - so the v2.0.35 merge dropped them and nothing failed. WHY NOT AUTO-STRIP: silently discarding upstream changes to a file also discards its bug and security fixes, and a half-removed change often does not build; the gateway stops and asks instead. BUILD NOTE: writing the .xlsx from a script needs either Python openpyxl (on this PC, not a repo dependency) or a Node library such as exceljs (a NEW dependency - AGENTS.md rule 6 requires the user's ok naming it). Settle in S04, ask first.</t>
+          <t>WHY, MEASURED 2026-09-13: the only guard today (scripts/verify-selective-v2032.mjs) hash-checks 9 media files and forbids Atomic Code paths and text. The fork differs from upstream v2.0.37 in 447 files, almost all unguarded. The window controls (Task 23) lived in web-app/src/routes/__root.tsx, which was not protected, and their only test rendered the component on its own - so the v2.0.35 merge dropped them and nothing failed. WHY NOT AUTO-STRIP: silently discarding upstream changes to a file also discards its bug and security fixes, and a half-removed change often does not build; the gateway stops and asks instead. BUILD NOTE: writing the .xlsx from a script needs either Python openpyxl (on this PC, not a repo dependency) or a Node library such as exceljs (a NEW dependency - AGENTS.md rule 6 requires the user's ok naming it). Settle in S04, ask first. | 2026-09-13: BUILT on feat/upstream-gateway (stacked on the Task 22 branch). New sheets 'Fork features' (13 features) and 'Upstream impact'. Commands: make upstream-impact (report), python scripts/upstream-gateway-tracker.py export / import (sheets and your decisions), make upstream-gate (refuses until every flagged row is decided), make upstream-post-merge (runs every feature's check). DEMO on the v2.0.37 sync we already did: it flags 4 features - the Radium name CONFLICTS in 3 setup.json files; auto-update, Settings and the Hub filter files are edited - plus 3 conflicting files no feature claims (INDEX.md, proxy.rs, models.ts - models.ts is where the leftover &gt;&gt;&gt;&gt;&gt;&gt;&gt; marker came from). The gate refused until decisions were recorded. Against upstream today: 0 new upstream commits, nothing to decide.</t>
         </is>
       </c>
     </row>
@@ -10522,7 +10525,7 @@
       </c>
       <c r="E190" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F190" s="13" t="n"/>
@@ -10538,7 +10541,7 @@
       </c>
       <c r="I190" s="15" t="inlineStr">
         <is>
-          <t>Flag every row that has no check yet - those are the gaps that let the window controls go.</t>
+          <t>Flag every row that has no check yet - those are the gaps that let the window controls go. | 2026-09-13: docs/upstream-gateway/fork-features.json, mirrored to the 'Fork features' sheet. 13 rows: Radium Media, Media in the sidebar, Atomic Code stays removed, product name, data-folder move, launch at startup, assistant name migration, no auto-update, Windows offline backends, Settings Chat/Cloud/API, Windows window controls (pending PR #10), Uncensored filter (pending PR #11), Windows test build CI (no check yet). tests/fork-features-register.test.mjs keeps every row pointing at real files and tests.</t>
         </is>
       </c>
     </row>
@@ -10563,7 +10566,7 @@
       </c>
       <c r="E191" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F191" s="13" t="n"/>
@@ -10579,7 +10582,7 @@
       </c>
       <c r="I191" s="15" t="inlineStr">
         <is>
-          <t>A check that cannot fail is not a check.</t>
+          <t>A check that cannot fail is not a check. | 2026-09-13: Every live row but one has a check. NEW: a NavMain test that Media stays in the sidebar. Mutation proof: removing the Media row from NavMain.tsx made 'keeps Media as its own sidebar entry' fail; restored with no diff. Remaining gap: windows-test-build-ci (workflow; no local check). All checks run on this branch: all 13 rows' checks pass on this branch (media 404 tests, NavMain 8, product name 8, data-folder migration 18 Rust tests, launch at startup 11, assistant migration 12, no auto-update 6, Windows backends 4, Settings Chat/Cloud/API 67, selective guard verified); pending rows skipped until PR #10/#11 merge. The data-folder check first crashed loading the test binary (0xC0000139) because it lacked --no-default-features --features test-tauri; fixed in the register.</t>
         </is>
       </c>
     </row>
@@ -10604,7 +10607,7 @@
       </c>
       <c r="E192" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F192" s="13" t="n"/>
@@ -10620,7 +10623,7 @@
       </c>
       <c r="I192" s="15" t="inlineStr">
         <is>
-          <t>Ask before adding any dependency (see the task notes).</t>
+          <t>Ask before adding any dependency (see the task notes). | 2026-09-13: scripts/upstream-gateway.mjs impact: git merge-tree trial merge (no branch or file touched), per-feature kind untouched/edited/deleted/conflict, commits, plain-language consequence, recommendation, decisions kept while the upstream commits behind them are unchanged, and conflicts in files no feature claims. Tests drive it against a throwaway repo (tests/upstream-gateway.test.mjs, 7 tests). NO new dependency: node for the gate, openpyxl (already the tracker's tool) for the sheets.</t>
         </is>
       </c>
     </row>
@@ -10645,7 +10648,7 @@
       </c>
       <c r="E193" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F193" s="13" t="n"/>
@@ -10659,7 +10662,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I193" s="15" t="n"/>
+      <c r="I193" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-13: make upstream-gate (exit 1 naming undecided rows, or a stale report) and make upstream-post-merge (runs every feature's checks, names failures). Both tested. Both tests added to make test-hardening-contracts.</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="6" t="inlineStr">
@@ -10682,7 +10689,7 @@
       </c>
       <c r="E194" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F194" s="13" t="n"/>
@@ -10698,7 +10705,7 @@
       </c>
       <c r="I194" s="15" t="inlineStr">
         <is>
-          <t>Keep AGENTS.md under its size limit.</t>
+          <t>Keep AGENTS.md under its size limit. | 2026-09-13: AGENTS.md rule 10 (file kept at 200 lines), DEVELOP.md 'Syncing with upstream', ADR docs/decisions/2026-09-13-gate-every-upstream-sync-on-a-fork-features-impact-report.md with INDEX lines (load-bearing + Other; 252 records).</t>
         </is>
       </c>
     </row>
@@ -10723,7 +10730,7 @@
       </c>
       <c r="E195" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F195" s="13" t="n"/>
@@ -10739,7 +10746,7 @@
       </c>
       <c r="I195" s="15" t="inlineStr">
         <is>
-          <t>This is the proof the gateway works before it is needed for real.</t>
+          <t>This is the proof the gateway works before it is needed for real. | 2026-09-13: Dry run against upstream/main: 0 commits since v2.0.37, nothing flagged. Demo on the v2.0.37 sync shown to the user. The real walk-through happens at the next upstream release.</t>
         </is>
       </c>
     </row>
@@ -10961,7 +10968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12370,6 +12377,43 @@
         </is>
       </c>
       <c r="G38" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>D32</t>
+        </is>
+      </c>
+      <c r="B39" s="14" t="inlineStr">
+        <is>
+          <t>HOW THE GATEWAY STORES THE REGISTER AND YOUR DECISIONS (Task 25). Taken under the user's standing 'just act' instruction.</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>Task 25 S02-S05.</t>
+        </is>
+      </c>
+      <c r="D39" s="14" t="inlineStr">
+        <is>
+          <t>The register and report are JSON files in the repo (read by the gate and by CI, no new dependency); the tracker's two sheets are generated from them and the yellow decision column is imported back. Rejected: making the xlsx the source of truth (the gate would need an Excel library in the repo).</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>Decided by the agent 2026-09-13 under the standing instruction; the user can reverse it.</t>
+        </is>
+      </c>
+      <c r="F39" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
         <is>
           <t>2026-09-13</t>
         </is>
@@ -12891,4 +12935,687 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="25" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C1" s="25" t="inlineStr">
+        <is>
+          <t>What it does for you</t>
+        </is>
+      </c>
+      <c r="D1" s="25" t="inlineStr">
+        <is>
+          <t>Where it lives</t>
+        </is>
+      </c>
+      <c r="E1" s="25" t="inlineStr">
+        <is>
+          <t>The check that proves it works</t>
+        </is>
+      </c>
+      <c r="F1" s="25" t="inlineStr">
+        <is>
+          <t>Decision or record</t>
+        </is>
+      </c>
+      <c r="G1" s="25" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>radium-media</t>
+        </is>
+      </c>
+      <c r="B2" s="24" t="inlineStr">
+        <is>
+          <t>Radium Media</t>
+        </is>
+      </c>
+      <c r="C2" s="24" t="inlineStr">
+        <is>
+          <t>Generate images and video from the Media page through a pluggable engine (Radium Media Worker, ComfyUI or a cloud images API), keep the results in a media library, and store provider keys in the OS keychain.</t>
+        </is>
+      </c>
+      <c r="D2" s="24" t="inlineStr">
+        <is>
+          <t>web-app/src/services/media/**
+web-app/src/services/atomicMedia/**
+web-app/src/containers/media/**
+web-app/src/routes/media.tsx
+web-app/src/routes/media_.library.tsx
+web-app/src/services/media-registry.ts
+web-app/src/locales/*/media.json</t>
+        </is>
+      </c>
+      <c r="E2" s="24" t="inlineStr">
+        <is>
+          <t>npx vitest run src/services/media src/services/atomicMedia src/containers/media
+node --test tests/verify-selective-v2032.test.mjs
+node scripts/verify-selective-v2032.mjs</t>
+        </is>
+      </c>
+      <c r="F2" s="24" t="inlineStr">
+        <is>
+          <t>docs/decisions/2026-09-10-adopt-a-provider-adapter-architecture-for-radium-media.md</t>
+        </is>
+      </c>
+      <c r="G2" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>media-sidebar-entry</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Media in the sidebar</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>A Media row in the left sidebar opens Radium Media. Upstream has no such row.</t>
+        </is>
+      </c>
+      <c r="D3" s="24" t="inlineStr">
+        <is>
+          <t>web-app/src/components/left-sidebar/NavMain.tsx</t>
+        </is>
+      </c>
+      <c r="E3" s="24" t="inlineStr">
+        <is>
+          <t>npx vitest run src/components/left-sidebar/__tests__/NavMain.test.tsx</t>
+        </is>
+      </c>
+      <c r="F3" s="24" t="inlineStr">
+        <is>
+          <t>Task 19 (v2.0.35 sync)</t>
+        </is>
+      </c>
+      <c r="G3" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>atomic-code-removed</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Atomic Code workspace stays removed</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>The unfinished Code workspace and its model router are gone and must not come back with an upstream update.</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>MUST STAY REMOVED: web-app/src/containers/code/**
+web-app/src/routes/code.tsx
+web-app/src/services/model-router/**
+web-app/src/hooks/useModelStrategy.ts</t>
+        </is>
+      </c>
+      <c r="E4" s="24" t="inlineStr">
+        <is>
+          <t>node scripts/verify-selective-v2032.mjs</t>
+        </is>
+      </c>
+      <c r="F4" s="24" t="inlineStr">
+        <is>
+          <t>e0b537747 (PR #3)</t>
+        </is>
+      </c>
+      <c r="G4" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>product-name-radium</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>The product is called Radium</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>The app, window titles, installer, Start menu entry and every visible string say Radium; the installer removes an old Atomic Chat install without touching its data.</t>
+        </is>
+      </c>
+      <c r="D5" s="24" t="inlineStr">
+        <is>
+          <t>src-tauri/tauri.conf.json
+src-tauri/tauri.*.conf.json
+src-tauri/windows/hooks.nsh
+web-app/index.html
+web-app/src/locales/*/*.json</t>
+        </is>
+      </c>
+      <c r="E5" s="24" t="inlineStr">
+        <is>
+          <t>node --test tests/radium-product-name.test.mjs</t>
+        </is>
+      </c>
+      <c r="F5" s="24" t="inlineStr">
+        <is>
+          <t>docs/decisions/2026-09-13-rename-the-product-to-radium-and-move-the-data-folder.md</t>
+        </is>
+      </c>
+      <c r="G5" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>data-folder-migration</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Data folder moves to Radium on first launch</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>Chats, models and settings saved under Atomic Chat move to %APPDATA%\Radium\data once, and empty old folders are tidied on later launches.</t>
+        </is>
+      </c>
+      <c r="D6" s="24" t="inlineStr">
+        <is>
+          <t>src-tauri/src/core/app/data_migration.rs
+src-tauri/src/core/app/mod.rs
+src-tauri/src/lib.rs</t>
+        </is>
+      </c>
+      <c r="E6" s="24" t="inlineStr">
+        <is>
+          <t>cargo test --manifest-path src-tauri/Cargo.toml --no-default-features --features test-tauri --lib data_migration -- --test-threads=1</t>
+        </is>
+      </c>
+      <c r="F6" s="24" t="inlineStr">
+        <is>
+          <t>docs/decisions/2026-09-13-rename-the-product-to-radium-and-move-the-data-folder.md</t>
+        </is>
+      </c>
+      <c r="G6" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>launch-at-startup-rename</t>
+        </is>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Launch at startup survives the rename</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>If Atomic Chat was set to start with the computer, Radium keeps starting with it.</t>
+        </is>
+      </c>
+      <c r="D7" s="24" t="inlineStr">
+        <is>
+          <t>web-app/src/lib/launchAtStartup.ts</t>
+        </is>
+      </c>
+      <c r="E7" s="24" t="inlineStr">
+        <is>
+          <t>npx vitest run src/lib/__tests__/launchAtStartup.test.ts</t>
+        </is>
+      </c>
+      <c r="F7" s="24" t="inlineStr">
+        <is>
+          <t>docs/decisions/2026-09-13-rename-the-product-to-radium-and-move-the-data-folder.md</t>
+        </is>
+      </c>
+      <c r="G7" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>assistant-name-migration</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Saved assistants say Radium</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>The default assistant's name and instructions that said Atomic Chat or Radium Chat are updated to Radium.</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>extensions/assistant-extension/src/**</t>
+        </is>
+      </c>
+      <c r="E8" s="24" t="inlineStr">
+        <is>
+          <t>npx vitest run src/index.test.ts</t>
+        </is>
+      </c>
+      <c r="F8" s="24" t="inlineStr">
+        <is>
+          <t>450100bda</t>
+        </is>
+      </c>
+      <c r="G8" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>no-auto-update</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Radium never auto-updates</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>No update prompt can install upstream's Atomic Chat over Radium.</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>src-tauri/tauri.conf.json
+src-tauri/tauri.*.conf.json
+src-tauri/Cargo.toml
+web-app/package.json
+web-app/src/**/*pdater*</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>node --test tests/no-auto-update.test.mjs</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>docs/decisions/2026-09-12-radium-never-auto-updates.md</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>windows-offline-backends</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Windows installers carry verified engine backends</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>A fresh Windows install can run local models without downloading an engine first.</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>scripts/stage-windows-backends.mjs
+scripts/windows-backend-bundle.json
+.github/workflows/windows-test-build.yml
+src-tauri/resources/backend-packages/**</t>
+        </is>
+      </c>
+      <c r="E10" s="24" t="inlineStr">
+        <is>
+          <t>node --test tests/stage-windows-backends.test.mjs</t>
+        </is>
+      </c>
+      <c r="F10" s="24" t="inlineStr">
+        <is>
+          <t>b0d716a95, 60bc3b914</t>
+        </is>
+      </c>
+      <c r="G10" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
+        <is>
+          <t>settings-chat-cloud-api</t>
+        </is>
+      </c>
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t>Chat, Cloud and API live in Settings</t>
+        </is>
+      </c>
+      <c r="C11" s="24" t="inlineStr">
+        <is>
+          <t>Settings holds the chat's run settings, cloud providers and the local API server; the sidebar no longer lists Cloud or API, and old links still land on the right page.</t>
+        </is>
+      </c>
+      <c r="D11" s="24" t="inlineStr">
+        <is>
+          <t>web-app/src/containers/SettingsMenu.tsx
+web-app/src/containers/SettingsPageLayout.tsx
+web-app/src/containers/AgentWorkspaceLayout.tsx
+web-app/src/containers/RunSettingsPanel.tsx
+web-app/src/routes/settings/chat.tsx
+web-app/src/routes/settings/cloud.tsx
+web-app/src/routes/settings/api.tsx
+web-app/src/routes/api/index.tsx
+web-app/src/routes/cloud/index.tsx
+web-app/src/components/left-sidebar/NavMain.tsx
+web-app/src/constants/routes.ts</t>
+        </is>
+      </c>
+      <c r="E11" s="24" t="inlineStr">
+        <is>
+          <t>npx vitest run src/containers/__tests__/SettingsMenu.test.tsx src/components/left-sidebar/__tests__/NavMain.test.tsx src/routes/settings/__tests__/moved-pages-redirect.test.ts src/routes/api src/routes/cloud src/containers/AgentWorkspaceLayout.test.tsx src/containers/RunSettingsPanel.test.tsx</t>
+        </is>
+      </c>
+      <c r="F11" s="24" t="inlineStr">
+        <is>
+          <t>Task 22, D28 = B and D29 (PR #12)</t>
+        </is>
+      </c>
+      <c r="G11" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>windows-title-bar</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Windows window controls</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>On Windows the app has its own title bar with Minimize, Maximize/Restore and Close, and can be dragged and resized.</t>
+        </is>
+      </c>
+      <c r="D12" s="24" t="inlineStr">
+        <is>
+          <t>web-app/src/components/WindowFrame.tsx
+web-app/src/components/WindowControls.tsx
+web-app/src/lib/window-chrome.ts
+web-app/src/routes/__root.tsx
+web-app/src/index.css
+src-tauri/tauri.windows.conf.json</t>
+        </is>
+      </c>
+      <c r="E12" s="24" t="inlineStr">
+        <is>
+          <t>node --test tests/window-controls.test.mjs
+npx vitest run src/components/__tests__/WindowFrame.test.tsx src/components/__tests__/WindowControls.test.tsx</t>
+        </is>
+      </c>
+      <c r="F12" s="24" t="inlineStr">
+        <is>
+          <t>Task 23, D30 = A (PR #10). Lost once already in the v2.0.35 sync.</t>
+        </is>
+      </c>
+      <c r="G12" s="24" t="inlineStr">
+        <is>
+          <t>Waiting for its PR to merge</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
+        <is>
+          <t>hub-uncensored-in-filter-menu</t>
+        </is>
+      </c>
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t>Uncensored filter in the Hub filter menu</t>
+        </is>
+      </c>
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>The Uncensored checkbox sits inside the Hub's sort and filter menu with the other filters.</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
+        <is>
+          <t>web-app/src/containers/hub/HubFilters.tsx</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
+        <is>
+          <t>npx vitest run src/containers/hub/__tests__/HubFilters.test.tsx</t>
+        </is>
+      </c>
+      <c r="F13" s="24" t="inlineStr">
+        <is>
+          <t>Task 24 (PR #11)</t>
+        </is>
+      </c>
+      <c r="G13" s="24" t="inlineStr">
+        <is>
+          <t>Waiting for its PR to merge</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
+          <t>windows-test-build-ci</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Unsigned Windows test installer from GitHub Actions</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>Every branch can produce a Windows installer to try on this PC before merging.</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>.github/workflows/windows-test-build.yml</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>none - this is a gap</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>d0f56745c, 72bd66144</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>NO CHECK YET</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="50" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="25" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="C1" s="25" t="inlineStr">
+        <is>
+          <t>What upstream does to it</t>
+        </is>
+      </c>
+      <c r="D1" s="25" t="inlineStr">
+        <is>
+          <t>What this means</t>
+        </is>
+      </c>
+      <c r="E1" s="25" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="F1" s="25" t="inlineStr">
+        <is>
+          <t>Upstream commits</t>
+        </is>
+      </c>
+      <c r="G1" s="25" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="H1" s="25" t="inlineStr">
+        <is>
+          <t>Your decision</t>
+        </is>
+      </c>
+      <c r="I1" s="25" t="inlineStr">
+        <is>
+          <t>Decided on</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="24" t="inlineStr"/>
+      <c r="B2" s="24" t="inlineStr">
+        <is>
+          <t>Upstream upstream/main at 7eb04761f; Radium HEAD at 9a3aac704; made 2026-09-14.</t>
+        </is>
+      </c>
+      <c r="C2" s="24" t="n"/>
+      <c r="D2" s="24" t="n"/>
+      <c r="E2" s="24" t="n"/>
+      <c r="F2" s="24" t="n"/>
+      <c r="G2" s="24" t="n"/>
+      <c r="H2" s="24" t="n"/>
+      <c r="I2" s="24" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr"/>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Untouched by this update: Radium Media, Media in the sidebar, Atomic Code workspace stays removed, The product is called Radium, Data folder moves to Radium on first launch, Launch at startup survives the rename, Saved assistants say Radium, Radium never auto-updates, Windows installers carry verified engine backends, Chat, Cloud and API live in Settings, Windows window controls, Uncensored filter in the Hub filter menu, Unsigned Windows test installer from GitHub Actions</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="n"/>
+      <c r="D3" s="24" t="n"/>
+      <c r="E3" s="24" t="n"/>
+      <c r="F3" s="24" t="n"/>
+      <c r="G3" s="24" t="n"/>
+      <c r="H3" s="24" t="n"/>
+      <c r="I3" s="24" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs(tracker): record D27 done (PR #14, green build), the ready test installer and PR #13
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1073,7 +1073,7 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>2026-09-13 (latest): feat/upstream-gateway (Task 25) stacked on feat/api-cloud-chat-in-settings (Task 22, PR #12). Open PRs: #10 window controls, #11 Uncensored filter, #12 Task 22, and the Task 25 PR. PR #8 and #9 merged.</t>
+          <t>2026-09-14 (latest): open PRs #10 window controls, #11 Uncensored filter, #12 Task 22, #13 Task 25 (stacked on #12, carries the tracker), #14 D27 Node 24 actions. Tracker updates go on feat/upstream-gateway until #13 merges.</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-13 (latest): (1) the user installs the test build from run 34791322213 (PR #10) and checks the window bar (T23-S05) and the app log for T21-S14; then merge #10 and #11. (2) Review and merge the Task 22 PR. (3) Task 25 gateway before any upstream sync. (4) Task 26: get Radium Media actually generating.</t>
+          <t>2026-09-14 (latest): (1) USER: install the test build from run 34791322213 and check the window bar (T23-S05); the agent then reads app.log for T21-S14. (2) Merge order: #10 and #11 after that check, then #12, then #13 (retarget to main), then #14 (its build is green). (3) Task 26: the user installs ComfyUI and one image model for the first end-to-end Radium Media run. (4) Next upstream release: run make upstream-impact and walk the user through the Upstream impact sheet.</t>
         </is>
       </c>
     </row>
@@ -2709,7 +2709,7 @@
       </c>
       <c r="K28" s="15" t="inlineStr">
         <is>
-          <t>WHY, MEASURED 2026-09-13: the only guard today (scripts/verify-selective-v2032.mjs) hash-checks 9 media files and forbids Atomic Code paths and text. The fork differs from upstream v2.0.37 in 447 files, almost all unguarded. The window controls (Task 23) lived in web-app/src/routes/__root.tsx, which was not protected, and their only test rendered the component on its own - so the v2.0.35 merge dropped them and nothing failed. WHY NOT AUTO-STRIP: silently discarding upstream changes to a file also discards its bug and security fixes, and a half-removed change often does not build; the gateway stops and asks instead. BUILD NOTE: writing the .xlsx from a script needs either Python openpyxl (on this PC, not a repo dependency) or a Node library such as exceljs (a NEW dependency - AGENTS.md rule 6 requires the user's ok naming it). Settle in S04, ask first. | 2026-09-13: BUILT on feat/upstream-gateway (stacked on the Task 22 branch). New sheets 'Fork features' (13 features) and 'Upstream impact'. Commands: make upstream-impact (report), python scripts/upstream-gateway-tracker.py export / import (sheets and your decisions), make upstream-gate (refuses until every flagged row is decided), make upstream-post-merge (runs every feature's check). DEMO on the v2.0.37 sync we already did: it flags 4 features - the Radium name CONFLICTS in 3 setup.json files; auto-update, Settings and the Hub filter files are edited - plus 3 conflicting files no feature claims (INDEX.md, proxy.rs, models.ts - models.ts is where the leftover &gt;&gt;&gt;&gt;&gt;&gt;&gt; marker came from). The gate refused until decisions were recorded. Against upstream today: 0 new upstream commits, nothing to decide.</t>
+          <t>WHY, MEASURED 2026-09-13: the only guard today (scripts/verify-selective-v2032.mjs) hash-checks 9 media files and forbids Atomic Code paths and text. The fork differs from upstream v2.0.37 in 447 files, almost all unguarded. The window controls (Task 23) lived in web-app/src/routes/__root.tsx, which was not protected, and their only test rendered the component on its own - so the v2.0.35 merge dropped them and nothing failed. WHY NOT AUTO-STRIP: silently discarding upstream changes to a file also discards its bug and security fixes, and a half-removed change often does not build; the gateway stops and asks instead. BUILD NOTE: writing the .xlsx from a script needs either Python openpyxl (on this PC, not a repo dependency) or a Node library such as exceljs (a NEW dependency - AGENTS.md rule 6 requires the user's ok naming it). Settle in S04, ask first. | 2026-09-13: BUILT on feat/upstream-gateway (stacked on the Task 22 branch). New sheets 'Fork features' (13 features) and 'Upstream impact'. Commands: make upstream-impact (report), python scripts/upstream-gateway-tracker.py export / import (sheets and your decisions), make upstream-gate (refuses until every flagged row is decided), make upstream-post-merge (runs every feature's check). DEMO on the v2.0.37 sync we already did: it flags 4 features - the Radium name CONFLICTS in 3 setup.json files; auto-update, Settings and the Hub filter files are edited - plus 3 conflicting files no feature claims (INDEX.md, proxy.rs, models.ts - models.ts is where the leftover &gt;&gt;&gt;&gt;&gt;&gt;&gt; marker came from). The gate refused until decisions were recorded. Against upstream today: 0 new upstream commits, nothing to decide. | 2026-09-14: PR #13 https://github.com/walladanger/Radium/pull/13 (base feat/api-cloud-chat-in-settings - merge #12 first, then retarget). All 12 live rows' checks pass; the data-folder check needed --no-default-features --features test-tauri (first run crashed loading the test binary, 0xC0000139).</t>
         </is>
       </c>
     </row>
@@ -10336,7 +10336,7 @@
       </c>
       <c r="I185" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13: commit d692991dd; PR #10 https://github.com/walladanger/Radium/pull/10 into main. Test build run 34790472605 on throwaway branch test/radium-window-controls (rename + fix, never to be merged; its Makefile hardening list lacks the window-controls test because a scripted conflict fix failed - harmless for a build). S05 (see it in a real window) waits for that installer. | 2026-09-13: main merged into fix/window-controls (229d2352b); full test build run 34791322213 started. Merge PR #10 after the user's check on this PC.</t>
+          <t>2026-09-13: commit d692991dd; PR #10 https://github.com/walladanger/Radium/pull/10 into main. Test build run 34790472605 on throwaway branch test/radium-window-controls (rename + fix, never to be merged; its Makefile hardening list lacks the window-controls test because a scripted conflict fix failed - harmless for a build). S05 (see it in a real window) waits for that installer. | 2026-09-13: main merged into fix/window-controls (229d2352b); full test build run 34791322213 started. Merge PR #10 after the user's check on this PC. | 2026-09-14: test build run 34791322213 (PR #10 head 229d2352b) SUCCEEDED; artifact radium-windows-test-229d2352b..., 1314 MB, expires 2026-09-28. Waiting for the user to install it and check T23-S05, and for the app log line that closes T21-S14.</t>
         </is>
       </c>
     </row>
@@ -12220,17 +12220,17 @@
       </c>
       <c r="E34" s="15" t="inlineStr">
         <is>
-          <t>Agent recommendation, 2026-09-13; the user asked whether it needs updating and was told not yet.</t>
+          <t>Agent recommendation, 2026-09-13; the user asked whether it needs updating and was told not yet. | 2026-09-14: DONE in PR #14 (chore/actions-node24, caa5727ef). windows-test-build.yml only: checkout v5, setup-node v5 (package-manager-cache: false, because v5 would cache Yarn before corepack activates Yarn 4), setup-python v6, cache v5, upload-artifact v6. Test build run 34793572212 on the branch: SUCCESS with NO annotations - the Node 20 warning is gone. release.yml (upstream's, never run by the fork) left alone.</t>
         </is>
       </c>
       <c r="F34" s="13" t="inlineStr">
         <is>
-          <t>Noted</t>
+          <t>Answered</t>
         </is>
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): record the blank-screen fix, D33 header controls and the rename gaps
- T21-S14 done: the stray Radium Chat folder was removed on this PC.
- T21-S16: blank screen from stale extensions.json paths, repaired by hand,
  fixed in PR #15.
- T21-S15: the sidebar wordmark and 'Atomic Bot' strings the rename missed.
- D33: window controls in the page header, no separate bar (PR #10, 7141cef4c).
- Combined test build run 34800010936 (#10 + #11 + #12 + #15).
- Register: windows-title-bar follows the new layout; new pending row
  extensions-follow-data-folder for PR #15.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1040,7 +1040,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1193,11 +1192,10 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): (1) USER: install the test build from run 34791322213 and check the window bar (T23-S05); the agent then reads app.log for T21-S14. (2) Merge order: #10 and #11 after that check, then #12, then #13 (retarget to main), then #14 (its build is green). (3) Task 26: the user installs ComfyUI and one image model for the first end-to-end Radium Media run. (4) Next upstream release: run make upstream-impact and walk the user through the Upstream impact sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
+          <t>2026-09-14 (latest): (1) USER: install the combined build from run 34800010936 (PR #10 new layout + #11 + #12 + #15); check the window controls in the header (T23-S05), Settings &gt; Chat/Cloud/API (Task 22), and that the app opens normally. (2) Merge order after that: #10, #11, #15, #12, then #13 (retarget to main), #14. (3) T21-S15: finish the rename (wordmark, 'Atomic Bot' strings, guard). (4) Task 26 when the user installs ComfyUI.</t>
+        </is>
+      </c>
+    </row>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -2554,7 +2552,7 @@
       </c>
       <c r="K25" s="15" t="inlineStr">
         <is>
-          <t>SCOPE MEASURED 2026-09-13, not assumed. Today: web-app/src/components/left-sidebar/NavMain.tsx renders top-level Cloud (route.cloud.index = /cloud/, routes/cloud/index.tsx, 243 lines, the cloud provider registry) and API (route.api.index = /api/, routes/api/index.tsx, 148 lines, the local API server page). Upstream put them there DELIBERATELY in d887d3817 (Mike, 2026-09-03, 'Improve/agent flow #265'): /settings/local-api-server now only redirects to /api, and Settings &gt; Model providers &gt; a provider navigates to /cloud. OTHER PLACES THAT LINK TO THEM and must keep working: containers/DropdownModelProvider.tsx (to /cloud), containers/LocalApiServerStatusRow.tsx (to /api), routes/settings/providers/$providerName.tsx (to /cloud), routes/settings/local-api-server.tsx (redirect to /api). Settings menu: containers/SettingsMenu.tsx. MERGE COST: this reverses an upstream design choice, so NavMain.tsx, SettingsMenu.tsx and constants/routes.ts will conflict on upstream syncs that touch them. They differ from v2.0.37 today by only +18, +6 and +3 lines, so keep the change small and in as few upstream files as possible. MEDIA: none of these files is protected, and Media stays in the sidebar. | CHAT SETTINGS, MEASURED 2026-09-13: that panel is web-app/src/containers/RunSettingsPanel.tsx (446 lines), opened from AgentWorkspaceLayout.tsx via stores/run-settings-panel-store; it has its own tests (containers/RunSettingsPanel.test.tsx). It mixes two kinds of setting: per-ASSISTANT (system prompt, sampling, penalties) and per-MODEL (context size, advanced load options). Settings already has an Assistants page (routes/settings/assistant.tsx, 197 lines) that lists and edits assistants - the obvious neighbour. Not protected; no media file involved. | 2026-09-13: BUILT on feat/api-cloud-chat-in-settings off main (eb28f890d). Settings menu gains Chat, Cloud and API. /settings/api and /settings/cloud render the existing pages inside the Settings frame (new SettingsPageLayout); /api, /cloud (keeping ?provider) and /settings/local-api-server redirect there. Cloud and API left the sidebar. Settings &gt; Chat shows the run settings panel's own controls; the chat's sliders button now opens that page, and the side panel, its store and the model pill's fold-down (which only existed for that panel) are gone.</t>
+          <t>SCOPE MEASURED 2026-09-13, not assumed. Today: web-app/src/components/left-sidebar/NavMain.tsx renders top-level Cloud (route.cloud.index = /cloud/, routes/cloud/index.tsx, 243 lines, the cloud provider registry) and API (route.api.index = /api/, routes/api/index.tsx, 148 lines, the local API server page). Upstream put them there DELIBERATELY in d887d3817 (Mike, 2026-09-03, 'Improve/agent flow #265'): /settings/local-api-server now only redirects to /api, and Settings &gt; Model providers &gt; a provider navigates to /cloud. OTHER PLACES THAT LINK TO THEM and must keep working: containers/DropdownModelProvider.tsx (to /cloud), containers/LocalApiServerStatusRow.tsx (to /api), routes/settings/providers/$providerName.tsx (to /cloud), routes/settings/local-api-server.tsx (redirect to /api). Settings menu: containers/SettingsMenu.tsx. MERGE COST: this reverses an upstream design choice, so NavMain.tsx, SettingsMenu.tsx and constants/routes.ts will conflict on upstream syncs that touch them. They differ from v2.0.37 today by only +18, +6 and +3 lines, so keep the change small and in as few upstream files as possible. MEDIA: none of these files is protected, and Media stays in the sidebar. | CHAT SETTINGS, MEASURED 2026-09-13: that panel is web-app/src/containers/RunSettingsPanel.tsx (446 lines), opened from AgentWorkspaceLayout.tsx via stores/run-settings-panel-store; it has its own tests (containers/RunSettingsPanel.test.tsx). It mixes two kinds of setting: per-ASSISTANT (system prompt, sampling, penalties) and per-MODEL (context size, advanced load options). Settings already has an Assistants page (routes/settings/assistant.tsx, 197 lines) that lists and edits assistants - the obvious neighbour. Not protected; no media file involved. | 2026-09-13: BUILT on feat/api-cloud-chat-in-settings off main (eb28f890d). Settings menu gains Chat, Cloud and API. /settings/api and /settings/cloud render the existing pages inside the Settings frame (new SettingsPageLayout); /api, /cloud (keeping ?provider) and /settings/local-api-server redirect there. Cloud and API left the sidebar. Settings &gt; Chat shows the run settings panel's own controls; the chat's sliders button now opens that page, and the side panel, its store and the model pill's fold-down (which only existed for that panel) are gone. | 2026-09-14: the user asked again, from the PR #10 test build, for the in-chat settings, Cloud and API to move into Settings. That is exactly PR #12, which the installed build did not contain. It is in combined build run 34800010936.</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2605,7 @@
       </c>
       <c r="K26" s="15" t="inlineStr">
         <is>
-          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision. | 2026-09-13: PR #10 (fix/window-controls, head 229d2352b) now includes main, so its test build has the rename, the T21-S14 fix and the window controls together - run 34791322213. Waiting on: the user installs it and checks T23-S05.</t>
+          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision. | 2026-09-13: PR #10 (fix/window-controls, head 229d2352b) now includes main, so its test build has the rename, the T21-S14 fix and the window controls together - run 34791322213. Waiting on: the user installs it and checks T23-S05. | 2026-09-14: the user asked for the controls in the page header with no separate bar (D33); done in 7141cef4c. PR #10 title and description updated.</t>
         </is>
       </c>
     </row>
@@ -2775,7 +2773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I200"/>
+  <dimension ref="A1:I202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -9541,7 +9539,7 @@
       </c>
       <c r="E166" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F166" s="13" t="n"/>
@@ -9557,7 +9555,7 @@
       </c>
       <c r="I166" s="15" t="inlineStr">
         <is>
-          <t>FOUND 2026-09-13 on the install test. Expected: after 'Moved the data folder', the cleanup loop in data_migration.rs (lines 141-150 at 4402b9749) deletes any other old default folder that holds no data. Observed: C:\Users\Warwick\AppData\Roaming\Radium Chat\data\db\__status__.db still there, 0 bytes, created and last written 2026-09-11 08:18 - so it was never removed, not removed and recreated. Ruled out: not locked, not read-only (attrs=Archive), owned by the user, and a copy deletes fine. The installed code is identical to the branch, and unit test removes_the_empty_radium_chat_folder_jan_cli_left_behind passes, so the cause is not known yet. HARMLESS in the meantime: no code in the installed build writes to that folder, and removing it by hand loses nothing. | 2026-09-13: FIXED IN CODE, commit 15438a573 on feat/radium-product-name. Cause at that moment still unknown (not locked or read-only afterwards), so the fix is robust rather than a guess: cleanup now runs on every launch while the data lives at the new default, and every old folder is logged as Removed, HoldsData or Failed with the error. Tests first; 18 migration tests pass; clippy clean. Done once an installed build logs 'Removed the empty old data folder ...\Radium Chat\data' on this PC. | 2026-09-13: FIXED IN CODE (15438a573 + rustfmt 9db0736fa, merged with PR #9): the cleanup now retries on every launch and logs its outcome. Done once an installed build logs 'Removed the empty old data folder ...Radium Chat\data'.</t>
+          <t>FOUND 2026-09-13 on the install test. Expected: after 'Moved the data folder', the cleanup loop in data_migration.rs (lines 141-150 at 4402b9749) deletes any other old default folder that holds no data. Observed: C:\Users\Warwick\AppData\Roaming\Radium Chat\data\db\__status__.db still there, 0 bytes, created and last written 2026-09-11 08:18 - so it was never removed, not removed and recreated. Ruled out: not locked, not read-only (attrs=Archive), owned by the user, and a copy deletes fine. The installed code is identical to the branch, and unit test removes_the_empty_radium_chat_folder_jan_cli_left_behind passes, so the cause is not known yet. HARMLESS in the meantime: no code in the installed build writes to that folder, and removing it by hand loses nothing. | 2026-09-13: FIXED IN CODE, commit 15438a573 on feat/radium-product-name. Cause at that moment still unknown (not locked or read-only afterwards), so the fix is robust rather than a guess: cleanup now runs on every launch while the data lives at the new default, and every old folder is logged as Removed, HoldsData or Failed with the error. Tests first; 18 migration tests pass; clippy clean. Done once an installed build logs 'Removed the empty old data folder ...\Radium Chat\data' on this PC. | 2026-09-13: FIXED IN CODE (15438a573 + rustfmt 9db0736fa, merged with PR #9): the cleanup now retries on every launch and logs its outcome. Done once an installed build logs 'Removed the empty old data folder ...Radium Chat\data'. | 2026-09-14: DONE, measured on this PC. The PR #10 test build logged 'Removed the empty old data folder C:\Users\Warwick\AppData\Roaming\Radium Chat\data' at 02:24:00 UTC on its second launch; the folder is gone.</t>
         </is>
       </c>
     </row>
@@ -10213,7 +10211,7 @@
       </c>
       <c r="I182" s="15" t="inlineStr">
         <is>
-          <t>D30 = A: re-mount WindowControls and the drag region in __root.tsx; decorations stays false. | 2026-09-13: components/WindowFrame.tsx + lib/window-chrome.ts, wrapped in routes/__root.tsx. FOUND ON THE WAY: 3b147addc's August bar never shortened ~25 full-height layouts (h-svh, min-h-svh, the fixed sidebar), so it would have cut the bottom off every page; index.css now does that inside the frame, and the contract test pins those rules too.</t>
+          <t>D30 = A: re-mount WindowControls and the drag region in __root.tsx; decorations stays false. | 2026-09-13: components/WindowFrame.tsx + lib/window-chrome.ts, wrapped in routes/__root.tsx. FOUND ON THE WAY: 3b147addc's August bar never shortened ~25 full-height layouts (h-svh, min-h-svh, the fixed sidebar), so it would have cut the bottom off every page; index.css now does that inside the frame, and the contract test pins those rules too. | 2026-09-14: LAYOUT REDONE per D33 (commit 7141cef4c on PR #10): no separate bar; controls in the page header row left of the sliders button; HeaderPage is the drag region and keeps 160px clear. Tests red first; web 298 files / 3468 passed; hardening 45/45.</t>
         </is>
       </c>
     </row>
@@ -10254,7 +10252,7 @@
       </c>
       <c r="I183" s="15" t="inlineStr">
         <is>
-          <t>Edge resizing may have gone with the title bar - confirm rather than assume.</t>
+          <t>Edge resizing may have gone with the title bar - confirm rather than assume. | 2026-09-14: first look in a real build (run 34791322213): the buttons worked, but the user rejected the separate title bar (D33). Re-check on the combined build run 34800010936.</t>
         </is>
       </c>
     </row>
@@ -10336,7 +10334,7 @@
       </c>
       <c r="I185" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13: commit d692991dd; PR #10 https://github.com/walladanger/Radium/pull/10 into main. Test build run 34790472605 on throwaway branch test/radium-window-controls (rename + fix, never to be merged; its Makefile hardening list lacks the window-controls test because a scripted conflict fix failed - harmless for a build). S05 (see it in a real window) waits for that installer. | 2026-09-13: main merged into fix/window-controls (229d2352b); full test build run 34791322213 started. Merge PR #10 after the user's check on this PC. | 2026-09-14: test build run 34791322213 (PR #10 head 229d2352b) SUCCEEDED; artifact radium-windows-test-229d2352b..., 1314 MB, expires 2026-09-28. Waiting for the user to install it and check T23-S05, and for the app log line that closes T21-S14.</t>
+          <t>2026-09-13: commit d692991dd; PR #10 https://github.com/walladanger/Radium/pull/10 into main. Test build run 34790472605 on throwaway branch test/radium-window-controls (rename + fix, never to be merged; its Makefile hardening list lacks the window-controls test because a scripted conflict fix failed - harmless for a build). S05 (see it in a real window) waits for that installer. | 2026-09-13: main merged into fix/window-controls (229d2352b); full test build run 34791322213 started. Merge PR #10 after the user's check on this PC. | 2026-09-14: test build run 34791322213 (PR #10 head 229d2352b) SUCCEEDED; artifact radium-windows-test-229d2352b..., 1314 MB, expires 2026-09-28. Waiting for the user to install it and check T23-S05, and for the app log line that closes T21-S14. | 2026-09-14: combined test build run 34800010936 on test/radium-combined-2026-09-14 = PR #10 (new layout) + #11 + #12 + #15.</t>
         </is>
       </c>
     </row>
@@ -10948,6 +10946,88 @@
       <c r="I200" s="15" t="inlineStr">
         <is>
           <t>The worker is not published anywhere today.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="6" t="inlineStr">
+        <is>
+          <t>T21-S15</t>
+        </is>
+      </c>
+      <c r="B201" s="17" t="inlineStr">
+        <is>
+          <t>Task 21</t>
+        </is>
+      </c>
+      <c r="C201" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D201" s="14" t="inlineStr">
+        <is>
+          <t>Finish the rename: the sidebar wordmark and every visible 'Atomic Bot' / 'Atomic Chat' left</t>
+        </is>
+      </c>
+      <c r="E201" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F201" s="13" t="inlineStr"/>
+      <c r="G201" s="14" t="inlineStr">
+        <is>
+          <t>AppLogo.tsx draws 'Atomic Chat' as SVG paths (aria-label too); 'Atomic Bot' remains in 4 locale files x 14 locales (common, mcp-servers, settings, setup) and about 23 hard-coded strings in components (toasts, alt text, sample prompt, security dialog, OpenRouter X-Title). Extend tests/radium-product-name.test.mjs to cover 'Atomic Bot' and component source.</t>
+        </is>
+      </c>
+      <c r="H201" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I201" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: SEEN on the PR #10 test build: the sidebar still shows the Atomic Chat logo. The rename guard only searched locales for 'Atomic Chat'/'Radium Chat', so it missed 'Atomic Bot' and hard-coded strings. KEEP per D24: the 'Atomic Bot V2 VL' Hugging Face model name, AtomicBot-ai links, comments about the migration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="6" t="inlineStr">
+        <is>
+          <t>T21-S16</t>
+        </is>
+      </c>
+      <c r="B202" s="17" t="inlineStr">
+        <is>
+          <t>Task 21</t>
+        </is>
+      </c>
+      <c r="C202" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="D202" s="14" t="inlineStr">
+        <is>
+          <t>Blank screen after the data-folder move: extensions.json kept absolute paths to the old folder</t>
+        </is>
+      </c>
+      <c r="E202" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F202" s="13" t="inlineStr"/>
+      <c r="G202" s="14" t="inlineStr">
+        <is>
+          <t>PR #15 (fix/extensions-after-data-move, b5b01cac2): at startup reinstall the bundled extensions when extensions.json names files outside the current extensions folder, or is missing or unreadable. 4 Rust tests red first, data_migration 18/18, clippy clean.</t>
+        </is>
+      </c>
+      <c r="H202" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I202" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: FOUND on this PC with the PR #10 test build. The move to Radium/data worked, but extensions.json still pointed all 14 url/origin entries at Atomic Chat/data; the version had not changed, so nothing reinstalled, no extension loaded and the window was blank. REPAIRED BY HAND: backup extensions.json.before-path-fix-2026-09-14.bak, paths repointed, relaunch loaded every extension. Done once a build with PR #15 opens normally on a moved folder.</t>
         </is>
       </c>
     </row>
@@ -10968,7 +11048,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G39"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12416,6 +12496,43 @@
       <c r="G39" s="13" t="inlineStr">
         <is>
           <t>2026-09-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t>D33</t>
+        </is>
+      </c>
+      <c r="B40" s="14" t="inlineStr">
+        <is>
+          <t>WHERE DO THE WINDOWS WINDOW CONTROLS GO? (Task 23)</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Task 23 S04-S05.</t>
+        </is>
+      </c>
+      <c r="D40" s="14" t="inlineStr">
+        <is>
+          <t>The user's instruction, not a recommendation.</t>
+        </is>
+      </c>
+      <c r="E40" s="15" t="inlineStr">
+        <is>
+          <t>DECIDED BY THE USER 2026-09-14, from a screenshot of the first test build: 'i don't want that top bar. the windows controls need to move where red is' (the page header row, just left of the sliders button), then 'You can make the apps top space a bit taller but I need or want the windows transport bar'. Implemented as: no separate bar; Minimize, Maximize and Close in the header row; the header row moves the window.</t>
+        </is>
+      </c>
+      <c r="F40" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
         </is>
       </c>
     </row>
@@ -12943,7 +13060,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13197,69 +13314,71 @@
     <row r="7">
       <c r="A7" s="24" t="inlineStr">
         <is>
-          <t>launch-at-startup-rename</t>
+          <t>extensions-follow-data-folder</t>
         </is>
       </c>
       <c r="B7" s="24" t="inlineStr">
         <is>
-          <t>Launch at startup survives the rename</t>
+          <t>Extensions load after the data folder moves</t>
         </is>
       </c>
       <c r="C7" s="24" t="inlineStr">
         <is>
-          <t>If Atomic Chat was set to start with the computer, Radium keeps starting with it.</t>
+          <t>If extensions.json points at an old data folder, or is missing or unreadable, Radium reinstalls its bundled extensions instead of opening to a blank window.</t>
         </is>
       </c>
       <c r="D7" s="24" t="inlineStr">
         <is>
-          <t>web-app/src/lib/launchAtStartup.ts</t>
+          <t>src-tauri/src/core/setup.rs
+src-tauri/src/core/extensions/**
+src-tauri/src/lib.rs</t>
         </is>
       </c>
       <c r="E7" s="24" t="inlineStr">
         <is>
-          <t>npx vitest run src/lib/__tests__/launchAtStartup.test.ts</t>
+          <t>cargo test --manifest-path src-tauri/Cargo.toml --no-default-features --features test-tauri --lib extension_path_tests -- --test-threads=1</t>
         </is>
       </c>
       <c r="F7" s="24" t="inlineStr">
         <is>
-          <t>docs/decisions/2026-09-13-rename-the-product-to-radium-and-move-the-data-folder.md</t>
+          <t>Tracker T21-S16 (PR #15), found on this PC 2026-09-14</t>
         </is>
       </c>
       <c r="G7" s="24" t="inlineStr">
         <is>
-          <t>Checked</t>
+          <t>Waiting for its PR to merge</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="24" t="inlineStr">
         <is>
-          <t>assistant-name-migration</t>
+          <t>launch-at-startup-rename</t>
         </is>
       </c>
       <c r="B8" s="24" t="inlineStr">
         <is>
-          <t>Saved assistants say Radium</t>
+          <t>Launch at startup survives the rename</t>
         </is>
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>The default assistant's name and instructions that said Atomic Chat or Radium Chat are updated to Radium.</t>
+          <t>If Atomic Chat was set to start with the computer, Radium keeps starting with it.</t>
         </is>
       </c>
       <c r="D8" s="24" t="inlineStr">
         <is>
-          <t>extensions/assistant-extension/src/**</t>
+          <t>web-app/src/lib/launchAtStartup.ts</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>npx vitest run src/index.test.ts</t>
+          <t>npx vitest run src/lib/__tests__/launchAtStartup.test.ts</t>
         </is>
       </c>
       <c r="F8" s="24" t="inlineStr">
         <is>
-          <t>450100bda</t>
+          <t>docs/decisions/2026-09-13-rename-the-product-to-radium-and-move-the-data-folder.md</t>
         </is>
       </c>
       <c r="G8" s="24" t="inlineStr">
@@ -13271,20 +13390,57 @@
     <row r="9">
       <c r="A9" s="24" t="inlineStr">
         <is>
+          <t>assistant-name-migration</t>
+        </is>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Saved assistants say Radium</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>The default assistant's name and instructions that said Atomic Chat or Radium Chat are updated to Radium.</t>
+        </is>
+      </c>
+      <c r="D9" s="24" t="inlineStr">
+        <is>
+          <t>extensions/assistant-extension/src/**</t>
+        </is>
+      </c>
+      <c r="E9" s="24" t="inlineStr">
+        <is>
+          <t>npx vitest run src/index.test.ts</t>
+        </is>
+      </c>
+      <c r="F9" s="24" t="inlineStr">
+        <is>
+          <t>450100bda</t>
+        </is>
+      </c>
+      <c r="G9" s="24" t="inlineStr">
+        <is>
+          <t>Checked</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
           <t>no-auto-update</t>
         </is>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>Radium never auto-updates</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>No update prompt can install upstream's Atomic Chat over Radium.</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>src-tauri/tauri.conf.json
 src-tauri/tauri.*.conf.json
@@ -13293,39 +13449,39 @@
 web-app/src/**/*pdater*</t>
         </is>
       </c>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>node --test tests/no-auto-update.test.mjs</t>
         </is>
       </c>
-      <c r="F9" s="24" t="inlineStr">
+      <c r="F10" s="24" t="inlineStr">
         <is>
           <t>docs/decisions/2026-09-12-radium-never-auto-updates.md</t>
         </is>
       </c>
-      <c r="G9" s="24" t="inlineStr">
+      <c r="G10" s="24" t="inlineStr">
         <is>
           <t>Checked</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>windows-offline-backends</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Windows installers carry verified engine backends</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>A fresh Windows install can run local models without downloading an engine first.</t>
         </is>
       </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="D11" s="24" t="inlineStr">
         <is>
           <t>scripts/stage-windows-backends.mjs
 scripts/windows-backend-bundle.json
@@ -13333,39 +13489,39 @@
 src-tauri/resources/backend-packages/**</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr">
         <is>
           <t>node --test tests/stage-windows-backends.test.mjs</t>
         </is>
       </c>
-      <c r="F10" s="24" t="inlineStr">
+      <c r="F11" s="24" t="inlineStr">
         <is>
           <t>b0d716a95, 60bc3b914</t>
         </is>
       </c>
-      <c r="G10" s="24" t="inlineStr">
+      <c r="G11" s="24" t="inlineStr">
         <is>
           <t>Checked</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="24" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>settings-chat-cloud-api</t>
         </is>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>Chat, Cloud and API live in Settings</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>Settings holds the chat's run settings, cloud providers and the local API server; the sidebar no longer lists Cloud or API, and old links still land on the right page.</t>
         </is>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>web-app/src/containers/SettingsMenu.tsx
 web-app/src/containers/SettingsPageLayout.tsx
@@ -13380,94 +13536,57 @@
 web-app/src/constants/routes.ts</t>
         </is>
       </c>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E12" s="24" t="inlineStr">
         <is>
           <t>npx vitest run src/containers/__tests__/SettingsMenu.test.tsx src/components/left-sidebar/__tests__/NavMain.test.tsx src/routes/settings/__tests__/moved-pages-redirect.test.ts src/routes/api src/routes/cloud src/containers/AgentWorkspaceLayout.test.tsx src/containers/RunSettingsPanel.test.tsx</t>
         </is>
       </c>
-      <c r="F11" s="24" t="inlineStr">
+      <c r="F12" s="24" t="inlineStr">
         <is>
           <t>Task 22, D28 = B and D29 (PR #12)</t>
         </is>
       </c>
-      <c r="G11" s="24" t="inlineStr">
+      <c r="G12" s="24" t="inlineStr">
         <is>
           <t>Checked</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="24" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>windows-title-bar</t>
         </is>
       </c>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Windows window controls</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
-        <is>
-          <t>On Windows the app has its own title bar with Minimize, Maximize/Restore and Close, and can be dragged and resized.</t>
-        </is>
-      </c>
-      <c r="D12" s="24" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
+        <is>
+          <t>On Windows the Minimize, Maximize/Restore and Close buttons sit in the page header row (no separate title bar, D33), and the header row moves the window.</t>
+        </is>
+      </c>
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>web-app/src/components/WindowFrame.tsx
 web-app/src/components/WindowControls.tsx
 web-app/src/lib/window-chrome.ts
 web-app/src/routes/__root.tsx
-web-app/src/index.css
-src-tauri/tauri.windows.conf.json</t>
-        </is>
-      </c>
-      <c r="E12" s="24" t="inlineStr">
+src-tauri/tauri.windows.conf.json
+web-app/src/containers/HeaderPage.tsx</t>
+        </is>
+      </c>
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>node --test tests/window-controls.test.mjs
-npx vitest run src/components/__tests__/WindowFrame.test.tsx src/components/__tests__/WindowControls.test.tsx</t>
-        </is>
-      </c>
-      <c r="F12" s="24" t="inlineStr">
-        <is>
-          <t>Task 23, D30 = A (PR #10). Lost once already in the v2.0.35 sync.</t>
-        </is>
-      </c>
-      <c r="G12" s="24" t="inlineStr">
-        <is>
-          <t>Waiting for its PR to merge</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="24" t="inlineStr">
-        <is>
-          <t>hub-uncensored-in-filter-menu</t>
-        </is>
-      </c>
-      <c r="B13" s="24" t="inlineStr">
-        <is>
-          <t>Uncensored filter in the Hub filter menu</t>
-        </is>
-      </c>
-      <c r="C13" s="24" t="inlineStr">
-        <is>
-          <t>The Uncensored checkbox sits inside the Hub's sort and filter menu with the other filters.</t>
-        </is>
-      </c>
-      <c r="D13" s="24" t="inlineStr">
-        <is>
-          <t>web-app/src/containers/hub/HubFilters.tsx</t>
-        </is>
-      </c>
-      <c r="E13" s="24" t="inlineStr">
-        <is>
-          <t>npx vitest run src/containers/hub/__tests__/HubFilters.test.tsx</t>
+npx vitest run src/components/__tests__/WindowFrame.test.tsx src/components/__tests__/WindowControls.test.tsx src/containers/__tests__/HeaderPage.test.tsx</t>
         </is>
       </c>
       <c r="F13" s="24" t="inlineStr">
         <is>
-          <t>Task 24 (PR #11)</t>
+          <t>Task 23, D30 = A, D33 (PR #10). Lost once already in the v2.0.35 sync.</t>
         </is>
       </c>
       <c r="G13" s="24" t="inlineStr">
@@ -13479,35 +13598,72 @@
     <row r="14">
       <c r="A14" s="24" t="inlineStr">
         <is>
+          <t>hub-uncensored-in-filter-menu</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Uncensored filter in the Hub filter menu</t>
+        </is>
+      </c>
+      <c r="C14" s="24" t="inlineStr">
+        <is>
+          <t>The Uncensored checkbox sits inside the Hub's sort and filter menu with the other filters.</t>
+        </is>
+      </c>
+      <c r="D14" s="24" t="inlineStr">
+        <is>
+          <t>web-app/src/containers/hub/HubFilters.tsx</t>
+        </is>
+      </c>
+      <c r="E14" s="24" t="inlineStr">
+        <is>
+          <t>npx vitest run src/containers/hub/__tests__/HubFilters.test.tsx</t>
+        </is>
+      </c>
+      <c r="F14" s="24" t="inlineStr">
+        <is>
+          <t>Task 24 (PR #11)</t>
+        </is>
+      </c>
+      <c r="G14" s="24" t="inlineStr">
+        <is>
+          <t>Waiting for its PR to merge</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="24" t="inlineStr">
+        <is>
           <t>windows-test-build-ci</t>
         </is>
       </c>
-      <c r="B14" s="24" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>Unsigned Windows test installer from GitHub Actions</t>
         </is>
       </c>
-      <c r="C14" s="24" t="inlineStr">
+      <c r="C15" s="24" t="inlineStr">
         <is>
           <t>Every branch can produce a Windows installer to try on this PC before merging.</t>
         </is>
       </c>
-      <c r="D14" s="24" t="inlineStr">
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>.github/workflows/windows-test-build.yml</t>
         </is>
       </c>
-      <c r="E14" s="24" t="inlineStr">
+      <c r="E15" s="24" t="inlineStr">
         <is>
           <t>none - this is a gap</t>
         </is>
       </c>
-      <c r="F14" s="24" t="inlineStr">
+      <c r="F15" s="24" t="inlineStr">
         <is>
           <t>d0f56745c, 72bd66144</t>
         </is>
       </c>
-      <c r="G14" s="24" t="inlineStr">
+      <c r="G15" s="24" t="inlineStr">
         <is>
           <t>NO CHECK YET</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): record PR #16 for the rename follow-up (T21-S15)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1040,6 +1040,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1072,7 +1073,7 @@
       </c>
       <c r="B6" s="22" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): open PRs #10 window controls, #11 Uncensored filter, #12 Task 22, #13 Task 25 (stacked on #12, carries the tracker), #14 D27 Node 24 actions. Tracker updates go on feat/upstream-gateway until #13 merges.</t>
+          <t>2026-09-14 (latest): open PRs #10 window controls (header layout), #11 Uncensored filter, #12 Task 22, #13 Task 25 (stacked on #12, carries the tracker), #14 D27, #15 extensions after data move, #16 finish the rename. Tracker updates go on feat/upstream-gateway until #13 merges.</t>
         </is>
       </c>
     </row>
@@ -1196,6 +1197,7 @@
         </is>
       </c>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -2503,7 +2505,7 @@
       </c>
       <c r="K24" s="15" t="inlineStr">
         <is>
-          <t>2026-09-13 INSTALL TEST ON THIS PC: the rename and data move WORKED on real data - see T21-S12 for the measurements. Open: the user confirming a chat reply, and T21-S14 (the empty Radium Chat folder was not removed). Also recorded: D27, the Node.js 20 deprecation warning in the workflows. | Earlier: 2026-09-13 PROGRESS: S01-S11 Done and verified (see Steps). Open: S12 install test on this PC, S13 commit and PR - both wait for the user. STILL SAYING 'Radium Chat' OR 'Atomic Chat', each deliberate and reported to the user: media wording in MediaPreview.tsx (protected), MediaParamField.tsx, atomicWorker.ts and en/media.json (D25); the entry name Radium writes into Zed and Droid, which their config uses as a lookup key; LICENSE header (legal - user's call); the sidebar wordmark in AppLogo.tsx, drawn as SVG and owned by the separate wordmark task. PRE-EXISTING, found on the way, not fixed: CLI_OWNERSHIP_MARKER is b"Radium Chat" since D13, but the legacy jan binaries it is meant to recognise would contain 'Atomic Chat'; src-tauri/tauri.bundle.windows.nsis.template is not referenced by any build config. | Earlier: 2026-09-13, STATE BEFORE CODE STARTS, stated plainly. DONE: GitHub repo renamed walladanger/Atomic-Chat -&gt; walladanger/Radium, authorised by the user; local origin repointed; PR #8 and Windows test build run 34761971349 followed the rename and old URLs redirect. NOT DONE, DRAFT ONLY: branch feat/radium-product-name (off chore/upstream-v2.0.37 at 6c3909482) holds UNCOMMITTED edits written for 'Radium Chat' - a data-folder migration module with 11 unit tests, an NSIS pre-install hook, a launch-at-startup migration command, a contract test, an ADR and doc edits. NONE OF IT HAS BEEN COMPILED OR RUN. It will be re-targeted to 'Radium' and verified from scratch, not trusted as written. THE AGENT CREATED THAT BRANCH WITHOUT ASKING, which the working agreement forbids; recorded here rather than hidden. MEASURED ON THIS PC, not assumed: the data folder C:\Users\Warwick\AppData\Roaming\Atomic Chat\data is 3.4 GB and stores no absolute path to itself (model.yml paths are relative), so a same-volume rename is safe. BOTH settings.json files - %APPDATA%\chat.atomic.app and the legacy %APPDATA%\Atomic-Chat, which wins while it exists - name that path, so changing productName alone moves nothing and the migration must repoint both. The installed app is an MSI (v2.0.23, WiX key {64542677-4056-4D46-BBEE-094163B8EC1A}): the MSI channel upgrades in place because its upgradeCode is pinned, but the NSIS installer finds a previous install by productName and would install side by side without a pre-install hook. A stray, empty %APPDATA%\Radium Chat\data (one 0-byte db file, made by jan-cli) exists - see D26. Launch-at-startup is OFF on this PC today. MEDIA: nothing in this task needs a protected file, and the guard must pass untouched. | 2026-09-13: PR #8 (v2.0.37 sync) and PR #9 (the rename) are MERGED into main (eb28f890d). Open: T21-S14 needs an installed build to log the stray-folder cleanup.</t>
+          <t>2026-09-13 INSTALL TEST ON THIS PC: the rename and data move WORKED on real data - see T21-S12 for the measurements. Open: the user confirming a chat reply, and T21-S14 (the empty Radium Chat folder was not removed). Also recorded: D27, the Node.js 20 deprecation warning in the workflows. | Earlier: 2026-09-13 PROGRESS: S01-S11 Done and verified (see Steps). Open: S12 install test on this PC, S13 commit and PR - both wait for the user. STILL SAYING 'Radium Chat' OR 'Atomic Chat', each deliberate and reported to the user: media wording in MediaPreview.tsx (protected), MediaParamField.tsx, atomicWorker.ts and en/media.json (D25); the entry name Radium writes into Zed and Droid, which their config uses as a lookup key; LICENSE header (legal - user's call); the sidebar wordmark in AppLogo.tsx, drawn as SVG and owned by the separate wordmark task. PRE-EXISTING, found on the way, not fixed: CLI_OWNERSHIP_MARKER is b"Radium Chat" since D13, but the legacy jan binaries it is meant to recognise would contain 'Atomic Chat'; src-tauri/tauri.bundle.windows.nsis.template is not referenced by any build config. | Earlier: 2026-09-13, STATE BEFORE CODE STARTS, stated plainly. DONE: GitHub repo renamed walladanger/Atomic-Chat -&gt; walladanger/Radium, authorised by the user; local origin repointed; PR #8 and Windows test build run 34761971349 followed the rename and old URLs redirect. NOT DONE, DRAFT ONLY: branch feat/radium-product-name (off chore/upstream-v2.0.37 at 6c3909482) holds UNCOMMITTED edits written for 'Radium Chat' - a data-folder migration module with 11 unit tests, an NSIS pre-install hook, a launch-at-startup migration command, a contract test, an ADR and doc edits. NONE OF IT HAS BEEN COMPILED OR RUN. It will be re-targeted to 'Radium' and verified from scratch, not trusted as written. THE AGENT CREATED THAT BRANCH WITHOUT ASKING, which the working agreement forbids; recorded here rather than hidden. MEASURED ON THIS PC, not assumed: the data folder C:\Users\Warwick\AppData\Roaming\Atomic Chat\data is 3.4 GB and stores no absolute path to itself (model.yml paths are relative), so a same-volume rename is safe. BOTH settings.json files - %APPDATA%\chat.atomic.app and the legacy %APPDATA%\Atomic-Chat, which wins while it exists - name that path, so changing productName alone moves nothing and the migration must repoint both. The installed app is an MSI (v2.0.23, WiX key {64542677-4056-4D46-BBEE-094163B8EC1A}): the MSI channel upgrades in place because its upgradeCode is pinned, but the NSIS installer finds a previous install by productName and would install side by side without a pre-install hook. A stray, empty %APPDATA%\Radium Chat\data (one 0-byte db file, made by jan-cli) exists - see D26. Launch-at-startup is OFF on this PC today. MEDIA: nothing in this task needs a protected file, and the guard must pass untouched. | 2026-09-13: PR #8 (v2.0.37 sync) and PR #9 (the rename) are MERGED into main (eb28f890d). Open: T21-S14 needs an installed build to log the stray-folder cleanup. | 2026-09-14: follow-up PR #16 finishes the rename (T21-S15). Blank-screen fix PR #15 (T21-S16).</t>
         </is>
       </c>
     </row>
@@ -10970,7 +10972,7 @@
       </c>
       <c r="E201" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F201" s="13" t="inlineStr"/>
@@ -10986,7 +10988,7 @@
       </c>
       <c r="I201" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: SEEN on the PR #10 test build: the sidebar still shows the Atomic Chat logo. The rename guard only searched locales for 'Atomic Chat'/'Radium Chat', so it missed 'Atomic Bot' and hard-coded strings. KEEP per D24: the 'Atomic Bot V2 VL' Hugging Face model name, AtomicBot-ai links, comments about the migration.</t>
+          <t>2026-09-14: SEEN on the PR #10 test build: the sidebar still shows the Atomic Chat logo. The rename guard only searched locales for 'Atomic Chat'/'Radium Chat', so it missed 'Atomic Bot' and hard-coded strings. KEEP per D24: the 'Atomic Bot V2 VL' Hugging Face model name, AtomicBot-ai links, comments about the migration. | 2026-09-14: BUILT in PR #16 https://github.com/walladanger/Radium/pull/16 (fix/finish-radium-rename, e9eb8959f). AppLogo wordmark is now the text Radium; 276 'Atomic Bot' locale strings and ten hard-coded strings renamed. KEPT: Atomic Bot V2 VL model name, atomic-chat-cli command, and 'What is Atomic Bot?' in ThreadList.tsx because it recognises welcome threads saved by earlier versions (renaming it would let that thread be deleted during setup - caught before commit). Guard now forbids all three old names in locales and in web-app/src code text; AppLogo test. Both red first. Web 297 files / 3465 passed; typecheck, lint, test-quality, hardening 41/41, media guard all clean. Waiting on: a look at the text wordmark in a real window (next test build).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): every build gets a new version number (rule, D34, Task 27)
The user's standing rule: each build we commit, push and compile carries a new
version. Recorded in the Handover working agreement, with the numbering scheme
as D34 (add one to the last number, 2.0.37 -> 2.0.38) and Task 27 to automate
and enforce it. Every test build so far was 2.0.37.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1019,7 +1019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): (1) USER: install the combined build from run 34800010936 (PR #10 new layout + #11 + #12 + #15); check the window controls in the header (T23-S05), Settings &gt; Chat/Cloud/API (Task 22), and that the app opens normally. (2) Merge order after that: #10, #11, #15, #12, then #13 (retarget to main), #14. (3) T21-S15: finish the rename (wordmark, 'Atomic Bot' strings, guard). (4) Task 26 when the user installs ComfyUI.</t>
+          <t>2026-09-14 (latest): (1) USER: install the combined build from run 34800010936 (still v2.0.37 - built before the version rule) and check the window controls, Settings &gt; Chat/Cloud/API and a normal start. (2) Task 27: version bump script + tests, then the next combined build (with PR #16) as v2.0.38. (3) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16. (4) Task 26 when the user installs ComfyUI.</t>
         </is>
       </c>
     </row>
@@ -1291,6 +1291,18 @@
       <c r="B25" s="22" t="inlineStr">
         <is>
           <t>OBSOLETE as of 2026-09-10 - kept only so the next agent understands why the instruction disappeared. The eleven paths this row used to list are all committed and the working tree is clean. There are currently NO paths that must be left unstaged. Do not reinstate this list without checking git status first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>Every build gets a new version</t>
+        </is>
+      </c>
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>STANDING RULE FROM THE USER, 2026-09-14: "are we updating each edition of the software we create? if not, then we need to. Please create this rule into the excel tracker. Each version of software we create then commit, push and compile a version the version number should also change". Every build of Radium that is committed, pushed and compiled for the user carries a NEW version number, and no two different builds ever share one. Before starting a test or release build: bump the version in the commit that will be built (node scripts/bump-version.mjs once Task 27 lands; until then set src-tauri/tauri.conf.json and web-app/package.json to the same new number), commit, push, then build. Tell the user the new number with the download link. Scheme per D34: add one to the last number (2.0.37 -&gt; 2.0.38 -&gt; 2.0.39). History: before this rule every test build was 2.0.37, so installers could not be told apart and the app's version-triggered extension reinstall never ran (part of the 2026-09-14 blank screen).</t>
         </is>
       </c>
     </row>
@@ -1305,7 +1317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2758,6 +2770,51 @@
       </c>
       <c r="K29" s="15" t="inlineStr"/>
     </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>Task 27</t>
+        </is>
+      </c>
+      <c r="B30" s="11" t="inlineStr">
+        <is>
+          <t>14 - Release hygiene</t>
+        </is>
+      </c>
+      <c r="C30" s="14" t="inlineStr">
+        <is>
+          <t>Every build gets a new version number</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="E30" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F30" s="13" t="inlineStr"/>
+      <c r="G30" s="14" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="H30" s="14" t="inlineStr">
+        <is>
+          <t>Two version files always agree (test); one command bumps both; every test installer's name carries its version; a build whose version was already used by a different commit is refused; the installed app shows the new number.</t>
+        </is>
+      </c>
+      <c r="I30" s="13" t="inlineStr"/>
+      <c r="J30" s="14" t="inlineStr">
+        <is>
+          <t>ADDED 2026-09-14 at the user's instruction: "are we updating each edition of the software we create? if not, then we need to. Please create this rule into the excel tracker. Each version of software we create then commit, push and compile a version the version number should also change". MEASURED: every test build so far (runs 34765539327, 34791322213, 34800010936) was Radium_2.0.37_x64-setup.exe and showed v2.0.37 - the upstream number from the v2.0.37 sync. Nothing in the fork changes the version: only upstream's release.yml sets it from a tag, and windows-test-build.yml never does.</t>
+        </is>
+      </c>
+      <c r="K30" s="15" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A2:K40"/>
   <dataValidations count="1">
@@ -2775,7 +2832,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I202"/>
+  <dimension ref="A1:I208"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11032,6 +11089,240 @@
           <t>2026-09-14: FOUND on this PC with the PR #10 test build. The move to Radium/data worked, but extensions.json still pointed all 14 url/origin entries at Atomic Chat/data; the version had not changed, so nothing reinstalled, no extension loaded and the window was blank. REPAIRED BY HAND: backup extensions.json.before-path-fix-2026-09-14.bak, paths repointed, relaunch loaded every extension. Done once a build with PR #15 opens normally on a moved folder.</t>
         </is>
       </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="6" t="inlineStr">
+        <is>
+          <t>T27-S01</t>
+        </is>
+      </c>
+      <c r="B203" s="17" t="inlineStr">
+        <is>
+          <t>Task 27</t>
+        </is>
+      </c>
+      <c r="C203" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D203" s="14" t="inlineStr">
+        <is>
+          <t>Record the rule (Handover working agreement) and the scheme (D34)</t>
+        </is>
+      </c>
+      <c r="E203" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F203" s="13" t="inlineStr"/>
+      <c r="G203" s="14" t="inlineStr">
+        <is>
+          <t>Tracker Handover sheet row 'Every build gets a new version'; Decisions D34.</t>
+        </is>
+      </c>
+      <c r="H203" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I203" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: done at the user's instruction.</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="6" t="inlineStr">
+        <is>
+          <t>T27-S02</t>
+        </is>
+      </c>
+      <c r="B204" s="17" t="inlineStr">
+        <is>
+          <t>Task 27</t>
+        </is>
+      </c>
+      <c r="C204" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D204" s="14" t="inlineStr">
+        <is>
+          <t>Write the failing tests first</t>
+        </is>
+      </c>
+      <c r="E204" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F204" s="13" t="inlineStr"/>
+      <c r="G204" s="14" t="inlineStr">
+        <is>
+          <t>tests/app-version.test.mjs: tauri.conf.json and web-app/package.json carry the same version; the bump script adds one to the last number in both, in a scratch copy. Run red first.</t>
+        </is>
+      </c>
+      <c r="H204" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I204" s="15" t="inlineStr"/>
+    </row>
+    <row r="205">
+      <c r="A205" s="6" t="inlineStr">
+        <is>
+          <t>T27-S03</t>
+        </is>
+      </c>
+      <c r="B205" s="17" t="inlineStr">
+        <is>
+          <t>Task 27</t>
+        </is>
+      </c>
+      <c r="C205" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D205" s="14" t="inlineStr">
+        <is>
+          <t>scripts/bump-version.mjs and make bump-version</t>
+        </is>
+      </c>
+      <c r="E205" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F205" s="13" t="inlineStr"/>
+      <c r="G205" s="14" t="inlineStr">
+        <is>
+          <t>Reads the current version, adds one to the last number (or takes an explicit version), writes both files, prints the new number.</t>
+        </is>
+      </c>
+      <c r="H205" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I205" s="15" t="inlineStr">
+        <is>
+          <t>No new dependency.</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="6" t="inlineStr">
+        <is>
+          <t>T27-S04</t>
+        </is>
+      </c>
+      <c r="B206" s="17" t="inlineStr">
+        <is>
+          <t>Task 27</t>
+        </is>
+      </c>
+      <c r="C206" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D206" s="14" t="inlineStr">
+        <is>
+          <t>Name the test installer artifact with its version, and refuse a reused version</t>
+        </is>
+      </c>
+      <c r="E206" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F206" s="13" t="inlineStr"/>
+      <c r="G206" s="14" t="inlineStr">
+        <is>
+          <t>windows-test-build.yml: artifact radium-windows-test-&lt;version&gt;-&lt;sha&gt;; a step fails the build when that version was already built from a different commit.</t>
+        </is>
+      </c>
+      <c r="H206" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I206" s="15" t="inlineStr">
+        <is>
+          <t>The refusal is what makes the rule impossible to forget.</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="6" t="inlineStr">
+        <is>
+          <t>T27-S05</t>
+        </is>
+      </c>
+      <c r="B207" s="17" t="inlineStr">
+        <is>
+          <t>Task 27</t>
+        </is>
+      </c>
+      <c r="C207" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D207" s="14" t="inlineStr">
+        <is>
+          <t>Bump to 2.0.38 for the next combined test build (with PR #16) and confirm the app shows it</t>
+        </is>
+      </c>
+      <c r="E207" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F207" s="13" t="inlineStr"/>
+      <c r="G207" s="14" t="inlineStr">
+        <is>
+          <t>node scripts/bump-version.mjs on the build branch, commit, push, build; the sidebar and the installer name show 2.0.38.</t>
+        </is>
+      </c>
+      <c r="H207" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I207" s="15" t="inlineStr"/>
+    </row>
+    <row r="208">
+      <c r="A208" s="6" t="inlineStr">
+        <is>
+          <t>T27-S06</t>
+        </is>
+      </c>
+      <c r="B208" s="17" t="inlineStr">
+        <is>
+          <t>Task 27</t>
+        </is>
+      </c>
+      <c r="C208" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D208" s="14" t="inlineStr">
+        <is>
+          <t>Upstream gateway: flag an upstream version change as a Radium decision</t>
+        </is>
+      </c>
+      <c r="E208" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F208" s="13" t="inlineStr"/>
+      <c r="G208" s="14" t="inlineStr">
+        <is>
+          <t>Fork features row 'radium-version' on the two version files, so a sync that brings upstream's version bump is flagged (normally keep ours).</t>
+        </is>
+      </c>
+      <c r="H208" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I208" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -11050,7 +11341,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G40"/>
+  <dimension ref="A1:G41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12533,6 +12824,43 @@
         </is>
       </c>
       <c r="G40" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>D34</t>
+        </is>
+      </c>
+      <c r="B41" s="14" t="inlineStr">
+        <is>
+          <t>HOW DOES THE VERSION NUMBER CHANGE FOR EACH BUILD? (Task 27)</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>Every build from 2026-09-14 on.</t>
+        </is>
+      </c>
+      <c r="D41" s="14" t="inlineStr">
+        <is>
+          <t>Add one to the last number of the version on every build handed to the user: 2.0.37 -&gt; 2.0.38 -&gt; 2.0.39. It lives in src-tauri/tauri.conf.json (installer and Windows) and web-app/package.json (the v2.0.xx shown in the sidebar); both always change together. The Rust package version (0.6.599) is internal and stays. ALTERNATIVE the user can choose instead: a Radium-only line such as 3.0.1, 3.0.2, ... so Radium numbers never look like upstream Atomic Chat release numbers. Either way each installer counts as newer than the last.</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>THE RULE IS THE USER'S (2026-09-14): "are we updating each edition of the software we create? if not, then we need to. Please create this rule into the excel tracker. Each version of software we create then commit, push and compile a version the version number should also change". The numbering scheme (add one to the last number) was chosen by the agent under the user's standing 'just act' instruction and can be changed by the user at any time.</t>
+        </is>
+      </c>
+      <c r="F41" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G41" s="13" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): Task 27 built in PR #17; register row for version numbering
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1040,7 +1040,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1197,7 +1196,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -2807,13 +2805,21 @@
           <t>Two version files always agree (test); one command bumps both; every test installer's name carries its version; a build whose version was already used by a different commit is refused; the installed app shows the new number.</t>
         </is>
       </c>
-      <c r="I30" s="13" t="inlineStr"/>
+      <c r="I30" s="13" t="inlineStr">
+        <is>
+          <t>4bc6d347b (PR #17)</t>
+        </is>
+      </c>
       <c r="J30" s="14" t="inlineStr">
         <is>
           <t>ADDED 2026-09-14 at the user's instruction: "are we updating each edition of the software we create? if not, then we need to. Please create this rule into the excel tracker. Each version of software we create then commit, push and compile a version the version number should also change". MEASURED: every test build so far (runs 34765539327, 34791322213, 34800010936) was Radium_2.0.37_x64-setup.exe and showed v2.0.37 - the upstream number from the v2.0.37 sync. Nothing in the fork changes the version: only upstream's release.yml sets it from a tag, and windows-test-build.yml never does.</t>
         </is>
       </c>
-      <c r="K30" s="15" t="inlineStr"/>
+      <c r="K30" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: built and verified in PR #17. Next: the first build under the rule, v2.0.38, with #10, #11, #12, #15, #16, #17.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:K40"/>
@@ -11152,7 +11158,7 @@
       </c>
       <c r="E204" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F204" s="13" t="inlineStr"/>
@@ -11166,7 +11172,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I204" s="15" t="inlineStr"/>
+      <c r="I204" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: tests/app-version.test.mjs (5) and tests/build-version.test.mjs (6), both seen failing first because the scripts did not exist; the workflow assertion was seen failing before the workflow change. PR #17 https://github.com/walladanger/Radium/pull/17 (chore/version-every-build, 4bc6d347b). Hardening contracts 51/51, test-quality pass.</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="6" t="inlineStr">
@@ -11189,7 +11199,7 @@
       </c>
       <c r="E205" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F205" s="13" t="inlineStr"/>
@@ -11205,7 +11215,7 @@
       </c>
       <c r="I205" s="15" t="inlineStr">
         <is>
-          <t>No new dependency.</t>
+          <t>No new dependency. | 2026-09-14: scripts/bump-version.mjs + make bump-version: adds one to the last number in both files (VERSION=x.y.z sets a newer one); refuses disagreeing files and backwards numbers; touches only the top-level version line. PR #17 https://github.com/walladanger/Radium/pull/17 (chore/version-every-build, 4bc6d347b). Hardening contracts 51/51, test-quality pass.</t>
         </is>
       </c>
     </row>
@@ -11230,7 +11240,7 @@
       </c>
       <c r="E206" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F206" s="13" t="inlineStr"/>
@@ -11246,7 +11256,7 @@
       </c>
       <c r="I206" s="15" t="inlineStr">
         <is>
-          <t>The refusal is what makes the rule impossible to forget.</t>
+          <t>The refusal is what makes the rule impossible to forget. | 2026-09-14: scripts/check-build-version.mjs + windows-test-build.yml: the check runs right after checkout, the artifact is radium-windows-test-&lt;version&gt;-&lt;sha&gt;, a successful build tags test-build/v&lt;version&gt; (permissions contents: write). Workflow parses as YAML (21 steps). PR #17 https://github.com/walladanger/Radium/pull/17 (chore/version-every-build, 4bc6d347b). Hardening contracts 51/51, test-quality pass.</t>
         </is>
       </c>
     </row>
@@ -11308,7 +11318,7 @@
       </c>
       <c r="E208" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F208" s="13" t="inlineStr"/>
@@ -11322,7 +11332,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I208" s="15" t="inlineStr"/>
+      <c r="I208" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: Fork features row 'radium-version' added (pending until PR #17 merges).</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -13390,7 +13404,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -13996,6 +14010,47 @@
       <c r="G15" s="24" t="inlineStr">
         <is>
           <t>NO CHECK YET</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>radium-version</t>
+        </is>
+      </c>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t>Every build has its own version number</t>
+        </is>
+      </c>
+      <c r="C16" s="24" t="inlineStr">
+        <is>
+          <t>Each Radium installer carries a new version number, and a test build refuses to reuse one (tracker D34).</t>
+        </is>
+      </c>
+      <c r="D16" s="24" t="inlineStr">
+        <is>
+          <t>src-tauri/tauri.conf.json
+web-app/package.json
+scripts/bump-version.mjs
+scripts/check-build-version.mjs
+.github/workflows/windows-test-build.yml</t>
+        </is>
+      </c>
+      <c r="E16" s="24" t="inlineStr">
+        <is>
+          <t>node --test tests/app-version.test.mjs tests/build-version.test.mjs</t>
+        </is>
+      </c>
+      <c r="F16" s="24" t="inlineStr">
+        <is>
+          <t>Tracker D34, Task 27 (PR #17)</t>
+        </is>
+      </c>
+      <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>Waiting for its PR to merge</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): D35 - window controls back in a slim top strip with no line
The user found the header-row controls (D33) overlapping page buttons and
asked to revert just that area to the top strip, shorter and with no line.
D35 supersedes D33; PR #10 commit ea8707641; test build v2.0.39 run
34843302629. Register row windows-title-bar follows the strip again.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -2617,7 +2617,7 @@
       </c>
       <c r="K26" s="15" t="inlineStr">
         <is>
-          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision. | 2026-09-13: PR #10 (fix/window-controls, head 229d2352b) now includes main, so its test build has the rename, the T21-S14 fix and the window controls together - run 34791322213. Waiting on: the user installs it and checks T23-S05. | 2026-09-14: the user asked for the controls in the page header with no separate bar (D33); done in 7141cef4c. PR #10 title and description updated.</t>
+          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision. | 2026-09-13: PR #10 (fix/window-controls, head 229d2352b) now includes main, so its test build has the rename, the T21-S14 fix and the window controls together - run 34791322213. Waiting on: the user installs it and checks T23-S05. | 2026-09-14: the user asked for the controls in the page header with no separate bar (D33); done in 7141cef4c. PR #10 title and description updated. | 2026-09-14: D35 - back to a slim top strip with no line (commit ea8707641); v2.0.39 test build run 34843302629.</t>
         </is>
       </c>
     </row>
@@ -10276,7 +10276,7 @@
       </c>
       <c r="I182" s="15" t="inlineStr">
         <is>
-          <t>D30 = A: re-mount WindowControls and the drag region in __root.tsx; decorations stays false. | 2026-09-13: components/WindowFrame.tsx + lib/window-chrome.ts, wrapped in routes/__root.tsx. FOUND ON THE WAY: 3b147addc's August bar never shortened ~25 full-height layouts (h-svh, min-h-svh, the fixed sidebar), so it would have cut the bottom off every page; index.css now does that inside the frame, and the contract test pins those rules too. | 2026-09-14: LAYOUT REDONE per D33 (commit 7141cef4c on PR #10): no separate bar; controls in the page header row left of the sliders button; HeaderPage is the drag region and keeps 160px clear. Tests red first; web 298 files / 3468 passed; hardening 45/45.</t>
+          <t>D30 = A: re-mount WindowControls and the drag region in __root.tsx; decorations stays false. | 2026-09-13: components/WindowFrame.tsx + lib/window-chrome.ts, wrapped in routes/__root.tsx. FOUND ON THE WAY: 3b147addc's August bar never shortened ~25 full-height layouts (h-svh, min-h-svh, the fixed sidebar), so it would have cut the bottom off every page; index.css now does that inside the frame, and the contract test pins those rules too. | 2026-09-14: LAYOUT REDONE per D33 (commit 7141cef4c on PR #10): no separate bar; controls in the page header row left of the sliders button; HeaderPage is the drag region and keeps 160px clear. Tests red first; web 298 files / 3468 passed; hardening 45/45. | 2026-09-14: LAYOUT PER D35 (commit ea8707641 on PR #10): the top strip is back, 2rem tall with no line under it; HeaderPage is main's again. Tests red first (contract 5/5, component 6/6 after), hardening 45/45.</t>
         </is>
       </c>
     </row>
@@ -10317,7 +10317,7 @@
       </c>
       <c r="I183" s="15" t="inlineStr">
         <is>
-          <t>Edge resizing may have gone with the title bar - confirm rather than assume. | 2026-09-14: first look in a real build (run 34791322213): the buttons worked, but the user rejected the separate title bar (D33). Re-check on the combined build run 34800010936.</t>
+          <t>Edge resizing may have gone with the title bar - confirm rather than assume. | 2026-09-14: first look in a real build (run 34791322213): the buttons worked, but the user rejected the separate title bar (D33). Re-check on the combined build run 34800010936. | 2026-09-14: on the header-layout build the user saw the controls overlap the Hub's 'Open on Web' button and asked for the slim strip (D35). Re-check on test build v2.0.39, run 34843302629.</t>
         </is>
       </c>
     </row>
@@ -11281,7 +11281,7 @@
       </c>
       <c r="E207" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F207" s="13" t="inlineStr"/>
@@ -11295,7 +11295,11 @@
           <t>This PC</t>
         </is>
       </c>
-      <c r="I207" s="15" t="inlineStr"/>
+      <c r="I207" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: v2.0.38 was the first build under the rule (run 34841320635): still building when this was recorded; its version check step passed on the runner. The user then asked for the D35 window strip, so the next build is v2.0.39 (run 34843302629).</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="6" t="inlineStr">
@@ -11355,7 +11359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12829,7 +12833,7 @@
       </c>
       <c r="E40" s="15" t="inlineStr">
         <is>
-          <t>DECIDED BY THE USER 2026-09-14, from a screenshot of the first test build: 'i don't want that top bar. the windows controls need to move where red is' (the page header row, just left of the sliders button), then 'You can make the apps top space a bit taller but I need or want the windows transport bar'. Implemented as: no separate bar; Minimize, Maximize and Close in the header row; the header row moves the window.</t>
+          <t>DECIDED BY THE USER 2026-09-14, from a screenshot of the first test build: 'i don't want that top bar. the windows controls need to move where red is' (the page header row, just left of the sliders button), then 'You can make the apps top space a bit taller but I need or want the windows transport bar'. Implemented as: no separate bar; Minimize, Maximize and Close in the header row; the header row moves the window. | SUPERSEDED BY D35 on 2026-09-14: in a real build the header position overlapped page buttons (the Hub's 'Open on Web'); the user chose the slim top strip instead.</t>
         </is>
       </c>
       <c r="F40" s="13" t="inlineStr">
@@ -12875,6 +12879,43 @@
         </is>
       </c>
       <c r="G41" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="inlineStr">
+        <is>
+          <t>D35</t>
+        </is>
+      </c>
+      <c r="B42" s="14" t="inlineStr">
+        <is>
+          <t>WINDOWS WINDOW CONTROLS: BACK TO A TOP STRIP (Task 23). Supersedes D33.</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>Task 23 S04-S05.</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="inlineStr">
+        <is>
+          <t>The user's instruction, not a recommendation.</t>
+        </is>
+      </c>
+      <c r="E42" s="15" t="inlineStr">
+        <is>
+          <t>DECIDED BY THE USER 2026-09-14, after using the build with the controls in the page header (D33): "My main concern is the placement of the windows controls. Looking at the screenshot provided you can see there is some over lap of the controls and the UI. ... I don't think we need such a vertically tall space JUST for the windows controls. Unless you have a better idea I would like to revert JUST THIS ONE AREA AND NOTHING ELSE to how it was in the screenshot (with the red highlight) but reduce the vertical space assigned for the windows controls." Earlier the same day the user had also asked for the line under the strip to be erased. Implemented as: the top strip from the first PR #10 build, 2rem (32px) tall instead of 2.5rem, with no line under it; HeaderPage back to main's version. Nothing else changed. D33 is superseded.</t>
+        </is>
+      </c>
+      <c r="F42" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G42" s="13" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
@@ -13909,7 +13950,7 @@
       </c>
       <c r="C13" s="24" t="inlineStr">
         <is>
-          <t>On Windows the Minimize, Maximize/Restore and Close buttons sit in the page header row (no separate title bar, D33), and the header row moves the window.</t>
+          <t>On Windows a slim 32px strip along the top of the window holds the window's title and the Minimize, Maximize/Restore and Close buttons, with no line under it (D35); the strip moves the window.</t>
         </is>
       </c>
       <c r="D13" s="24" t="inlineStr">
@@ -13918,19 +13959,19 @@
 web-app/src/components/WindowControls.tsx
 web-app/src/lib/window-chrome.ts
 web-app/src/routes/__root.tsx
-src-tauri/tauri.windows.conf.json
-web-app/src/containers/HeaderPage.tsx</t>
+web-app/src/index.css
+src-tauri/tauri.windows.conf.json</t>
         </is>
       </c>
       <c r="E13" s="24" t="inlineStr">
         <is>
           <t>node --test tests/window-controls.test.mjs
-npx vitest run src/components/__tests__/WindowFrame.test.tsx src/components/__tests__/WindowControls.test.tsx src/containers/__tests__/HeaderPage.test.tsx</t>
+npx vitest run src/components/__tests__/WindowFrame.test.tsx src/components/__tests__/WindowControls.test.tsx</t>
         </is>
       </c>
       <c r="F13" s="24" t="inlineStr">
         <is>
-          <t>Task 23, D30 = A, D33 (PR #10). Lost once already in the v2.0.35 sync.</t>
+          <t>Task 23, D30 = A, D35 (supersedes D33) (PR #10). Lost once already in the v2.0.35 sync.</t>
         </is>
       </c>
       <c r="G13" s="24" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): Task 28 - review skills and MCP connectors before use (D36)
The user asked what protects against harmful skills and MCP servers, and for a
screen that shows what one can do before it is used. Records what exists today
(per-action approval, shell hard blocks, skill import checks, per-tool MCP
switches), the gaps (MCP actions auto-approved by default, self-declared
read-only hints, no review when a skill or connector is added, no scanner), and
the plan: a plain-language review screen, re-review on change, a safer MCP
default, and labelled warnings.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1040,6 +1040,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1192,10 +1193,11 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): (1) USER: install the combined build from run 34800010936 (still v2.0.37 - built before the version rule) and check the window controls, Settings &gt; Chat/Cloud/API and a normal start. (2) Task 27: version bump script + tests, then the next combined build (with PR #16) as v2.0.38. (3) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16. (4) Task 26 when the user installs ComfyUI.</t>
-        </is>
-      </c>
-    </row>
+          <t>2026-09-14 (latest): (1) USER: install test build v2.0.39 (slim window strip, D35) when run 34843302629 finishes. (2) Task 28: review-before-use screens for skills and MCP connectors, re-review on change, safer MCP default, warnings - tests first. (3) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #17. (4) Task 26 when the user installs ComfyUI.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -1315,7 +1317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2821,6 +2823,51 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="B31" s="11" t="inlineStr">
+        <is>
+          <t>15 - Safety</t>
+        </is>
+      </c>
+      <c r="C31" s="14" t="inlineStr">
+        <is>
+          <t>Review before use: a clear permissions screen for skills and MCP connectors, plus safer defaults</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="inlineStr">
+        <is>
+          <t>Laptop, then this PC</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F31" s="13" t="inlineStr"/>
+      <c r="G31" s="14" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="H31" s="14" t="inlineStr">
+        <is>
+          <t>No skill or connector is used until the user has seen, in plain language, what it can do and has allowed it; changed contents ask again; MCP actions that can change things ask by default; suspicious patterns are shown as warnings; tests cover each.</t>
+        </is>
+      </c>
+      <c r="I31" s="13" t="inlineStr"/>
+      <c r="J31" s="14" t="inlineStr">
+        <is>
+          <t>ADDED 2026-09-14 at the user's request: "what can we do against malicious code are actions in regards to skills and MCP's? is there some sort of auto checker anti virus for MCP's and skills? at the very least can we create a pop window or user verifiable before proceeding pop up screen that clearly lists what the skill or mcp can do or has access to before actually using it?" MEASURED ON MAIN 2026-09-14. WHAT EXISTS: (1) Per-action approval for the agent's own tools: a dialog shows the tool, the reason, a preview of the arguments and the files it touches, with Deny / Approve once / Always allow (ADRs 2026-07-16, 2026-07-23; AgentApprovalDialog.tsx). Reading inside the workspace needs no approval; writing, deleting, leaving the workspace and flagged shell commands do. (2) A shell guard hard-blocks the worst commands (e.g. 'rm -rf /', formatting a disk) even when approvals are skipped, and asks before sudo, chmod, curl, wget, shutdown (shell_guard.rs). (3) Skill import checks: SKILL.md must parse, name/description required, unknown header fields and symlinks refused, prompt-injection-looking catalog text refused (authoring.rs, manifest.rs). Skills can declare 'dangerous', 'requires_tools', 'requires_scripts', but these are only passed to the AI as text. (4) Per-tool on/off switches for each MCP connector (ADR 2026-09-02). GAPS: (a) 'Allow all MCP permissions' defaults to ON, and a one-time migration forced it ON for every existing user (useToolApproval.ts), so MCP tools that can change things run without asking. (b) Whether an MCP tool counts as read-only comes from the server's own readOnlyHint - a malicious server can simply claim it. (c) A new skill or connector is usable as soon as it is added: nothing shows the user what it asks for, and nothing asks again when its contents change. (d) There is no scanner. None can prove a skill (plain instructions) or an MCP server (someone else's program or web service) is safe; pattern checks can only warn.</t>
+        </is>
+      </c>
+      <c r="K31" s="15" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A2:K40"/>
   <dataValidations count="1">
@@ -2838,7 +2885,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I208"/>
+  <dimension ref="A1:I216"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11341,6 +11388,326 @@
           <t>2026-09-14: Fork features row 'radium-version' added (pending until PR #17 merges).</t>
         </is>
       </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="6" t="inlineStr">
+        <is>
+          <t>T28-S01</t>
+        </is>
+      </c>
+      <c r="B209" s="17" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="C209" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="D209" s="14" t="inlineStr">
+        <is>
+          <t>Record the findings and the approach (D36)</t>
+        </is>
+      </c>
+      <c r="E209" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F209" s="13" t="inlineStr"/>
+      <c r="G209" s="14" t="inlineStr">
+        <is>
+          <t>Tasks sheet Task 28 notes; Decisions D36.</t>
+        </is>
+      </c>
+      <c r="H209" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I209" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: done.</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="6" t="inlineStr">
+        <is>
+          <t>T28-S02</t>
+        </is>
+      </c>
+      <c r="B210" s="17" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="C210" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="D210" s="14" t="inlineStr">
+        <is>
+          <t>Write the failing tests first</t>
+        </is>
+      </c>
+      <c r="E210" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F210" s="13" t="inlineStr"/>
+      <c r="G210" s="14" t="inlineStr">
+        <is>
+          <t>Frontend: a skill or connector that has not been reviewed cannot be switched on or used; the review screen lists its permissions in plain words; Allow enables it, Cancel leaves it off; a changed skill/server asks again. Backend: an unreviewed skill is not offered to the AI; the MCP default asks.</t>
+        </is>
+      </c>
+      <c r="H210" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I210" s="15" t="inlineStr">
+        <is>
+          <t>Run red first, for the right reason.</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="6" t="inlineStr">
+        <is>
+          <t>T28-S03</t>
+        </is>
+      </c>
+      <c r="B211" s="17" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="C211" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="D211" s="14" t="inlineStr">
+        <is>
+          <t>Skill review screen</t>
+        </is>
+      </c>
+      <c r="E211" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F211" s="13" t="inlineStr"/>
+      <c r="G211" s="14" t="inlineStr">
+        <is>
+          <t>Shown when a skill is added, uploaded, or first switched on: name, where it came from, what it asks the AI to use in plain words (run commands, read/write files, internet...), 'marked dangerous', bundled scripts, platforms, and the first lines of its instructions. Buttons: Allow / Cancel. The 18 bundled starter skills count as reviewed at install.</t>
+        </is>
+      </c>
+      <c r="H211" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I211" s="15" t="inlineStr">
+        <is>
+          <t>Plain language, not tool ids.</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="6" t="inlineStr">
+        <is>
+          <t>T28-S04</t>
+        </is>
+      </c>
+      <c r="B212" s="17" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="C212" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="D212" s="14" t="inlineStr">
+        <is>
+          <t>Connector (MCP) review screen</t>
+        </is>
+      </c>
+      <c r="E212" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F212" s="13" t="inlineStr"/>
+      <c r="G212" s="14" t="inlineStr">
+        <is>
+          <t>Shown when a connector is added, imported or first switched on: the program it runs or the web address it talks to, the keys/secrets it receives, and its tools split into 'only reads' and 'can change things' - with a note that the server labels its own tools. Buttons: Allow / Cancel.</t>
+        </is>
+      </c>
+      <c r="H212" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I212" s="15" t="inlineStr"/>
+    </row>
+    <row r="213">
+      <c r="A213" s="6" t="inlineStr">
+        <is>
+          <t>T28-S05</t>
+        </is>
+      </c>
+      <c r="B213" s="17" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="C213" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="D213" s="14" t="inlineStr">
+        <is>
+          <t>Ask again when a skill or connector changes</t>
+        </is>
+      </c>
+      <c r="E213" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F213" s="13" t="inlineStr"/>
+      <c r="G213" s="14" t="inlineStr">
+        <is>
+          <t>Store a fingerprint of what was allowed (the SKILL.md and scripts; the connector's command/URL, arguments and tool list). A different fingerprint turns it off until reviewed again.</t>
+        </is>
+      </c>
+      <c r="H213" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I213" s="15" t="inlineStr">
+        <is>
+          <t>The same idea as 'Always allow' fingerprints in ADR 2026-07-23.</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="6" t="inlineStr">
+        <is>
+          <t>T28-S06</t>
+        </is>
+      </c>
+      <c r="B214" s="17" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="C214" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="D214" s="14" t="inlineStr">
+        <is>
+          <t>Safer default for MCP actions</t>
+        </is>
+      </c>
+      <c r="E214" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F214" s="13" t="inlineStr"/>
+      <c r="G214" s="14" t="inlineStr">
+        <is>
+          <t>New installs: 'Allow all MCP permissions' starts OFF, so tools that can change things ask each time (the existing approval dialog). Existing installs: say so once and let the user choose, rather than silently flipping it.</t>
+        </is>
+      </c>
+      <c r="H214" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I214" s="15" t="inlineStr">
+        <is>
+          <t>Reverses the forced-ON migration in useToolApproval.ts; an ADR records it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="6" t="inlineStr">
+        <is>
+          <t>T28-S07</t>
+        </is>
+      </c>
+      <c r="B215" s="17" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="C215" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="D215" s="14" t="inlineStr">
+        <is>
+          <t>Warning checks (not a guarantee)</t>
+        </is>
+      </c>
+      <c r="E215" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F215" s="13" t="inlineStr"/>
+      <c r="G215" s="14" t="inlineStr">
+        <is>
+          <t>Flag on the review screen, in plain words: commands that download and run code (curl|sh, iwr|iex), deleting outside the workspace, reading key/credential locations, long encoded blobs, instructions to hide actions or send data elsewhere; connectors that run an unpinned package ('npx -y name' without a version) or talk to plain http.</t>
+        </is>
+      </c>
+      <c r="H215" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I215" s="15" t="inlineStr">
+        <is>
+          <t>Warnings only; the screen says a clean check does not prove safety.</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="6" t="inlineStr">
+        <is>
+          <t>T28-S08</t>
+        </is>
+      </c>
+      <c r="B216" s="17" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="C216" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D216" s="14" t="inlineStr">
+        <is>
+          <t>Verify, commit, PR, and try it on this PC</t>
+        </is>
+      </c>
+      <c r="E216" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F216" s="13" t="inlineStr"/>
+      <c r="G216" s="14" t="inlineStr">
+        <is>
+          <t>Web and Rust tests, typecheck, lint, test-quality, hardening contracts; a Fork features register row; commit, PR, a new-version test build (Task 27 rule) and a look on this PC.</t>
+        </is>
+      </c>
+      <c r="H216" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I216" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -11359,7 +11726,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -12916,6 +13283,43 @@
         </is>
       </c>
       <c r="G42" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>D36</t>
+        </is>
+      </c>
+      <c r="B43" s="14" t="inlineStr">
+        <is>
+          <t>HOW DO WE PROTECT AGAINST HARMFUL SKILLS AND MCP CONNECTORS? (Task 28)</t>
+        </is>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>Task 28.</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="inlineStr">
+        <is>
+          <t>No product can reliably scan skills or MCP servers for malice, so the protection is: (1) a plain-language review screen before a skill or connector can be used, listing what it can do and access, with Allow / Cancel - the user's request; (2) ask again whenever its contents change; (3) MCP actions that can change things ask each time by default (today they are auto-approved); (4) pattern-based warnings on the review screen, clearly labelled as warnings, not a guarantee. The existing per-action approval dialog and shell hard-blocks stay as the last line of defence.</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>REQUESTED BY THE USER 2026-09-14: "what can we do against malicious code are actions in regards to skills and MCP's? is there some sort of auto checker anti virus for MCP's and skills? at the very least can we create a pop window or user verifiable before proceeding pop up screen that clearly lists what the skill or mcp can do or has access to before actually using it?". Point (1) is the user's request. Points (2)-(4) were added by the agent under the user's standing 'just act' instruction; (3) changes a default, so existing users are told once and choose. The user can drop any of them.</t>
+        </is>
+      </c>
+      <c r="F43" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G43" s="13" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): Task 28 gains a Preview option on the review screen (D36 amended)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1040,7 +1040,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1197,7 +1196,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18">
       <c r="A18" s="20" t="inlineStr">
         <is>
@@ -2866,7 +2864,11 @@
           <t>ADDED 2026-09-14 at the user's request: "what can we do against malicious code are actions in regards to skills and MCP's? is there some sort of auto checker anti virus for MCP's and skills? at the very least can we create a pop window or user verifiable before proceeding pop up screen that clearly lists what the skill or mcp can do or has access to before actually using it?" MEASURED ON MAIN 2026-09-14. WHAT EXISTS: (1) Per-action approval for the agent's own tools: a dialog shows the tool, the reason, a preview of the arguments and the files it touches, with Deny / Approve once / Always allow (ADRs 2026-07-16, 2026-07-23; AgentApprovalDialog.tsx). Reading inside the workspace needs no approval; writing, deleting, leaving the workspace and flagged shell commands do. (2) A shell guard hard-blocks the worst commands (e.g. 'rm -rf /', formatting a disk) even when approvals are skipped, and asks before sudo, chmod, curl, wget, shutdown (shell_guard.rs). (3) Skill import checks: SKILL.md must parse, name/description required, unknown header fields and symlinks refused, prompt-injection-looking catalog text refused (authoring.rs, manifest.rs). Skills can declare 'dangerous', 'requires_tools', 'requires_scripts', but these are only passed to the AI as text. (4) Per-tool on/off switches for each MCP connector (ADR 2026-09-02). GAPS: (a) 'Allow all MCP permissions' defaults to ON, and a one-time migration forced it ON for every existing user (useToolApproval.ts), so MCP tools that can change things run without asking. (b) Whether an MCP tool counts as read-only comes from the server's own readOnlyHint - a malicious server can simply claim it. (c) A new skill or connector is usable as soon as it is added: nothing shows the user what it asks for, and nothing asks again when its contents change. (d) There is no scanner. None can prove a skill (plain instructions) or an MCP server (someone else's program or web service) is safe; pattern checks can only warn.</t>
         </is>
       </c>
-      <c r="K31" s="15" t="inlineStr"/>
+      <c r="K31" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: the user asked for a Preview option alongside Allow / Cancel (see D36 amendment) and to build Task 28.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A2:K40"/>
@@ -11508,7 +11510,7 @@
       </c>
       <c r="I211" s="15" t="inlineStr">
         <is>
-          <t>Plain language, not tool ids.</t>
+          <t>Plain language, not tool ids. | 2026-09-14: add Preview (full instructions, scripts, what-could-go-wrong list) per the D36 amendment.</t>
         </is>
       </c>
     </row>
@@ -11547,7 +11549,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I212" s="15" t="inlineStr"/>
+      <c r="I212" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: add Preview (look-only start that lists the connector's real tools, then stops) per the D36 amendment.</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="6" t="inlineStr">
@@ -13311,7 +13317,7 @@
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>REQUESTED BY THE USER 2026-09-14: "what can we do against malicious code are actions in regards to skills and MCP's? is there some sort of auto checker anti virus for MCP's and skills? at the very least can we create a pop window or user verifiable before proceeding pop up screen that clearly lists what the skill or mcp can do or has access to before actually using it?". Point (1) is the user's request. Points (2)-(4) were added by the agent under the user's standing 'just act' instruction; (3) changes a default, so existing users are told once and choose. The user can drop any of them.</t>
+          <t>REQUESTED BY THE USER 2026-09-14: "what can we do against malicious code are actions in regards to skills and MCP's? is there some sort of auto checker anti virus for MCP's and skills? at the very least can we create a pop window or user verifiable before proceeding pop up screen that clearly lists what the skill or mcp can do or has access to before actually using it?". Point (1) is the user's request. Points (2)-(4) were added by the agent under the user's standing 'just act' instruction; (3) changes a default, so existing users are told once and choose. The user can drop any of them. | AMENDED BY THE USER 2026-09-14: "task 28 1. allow and cancel. can we create a "preview" option to? not sure what this would do, maybe predict or list the potential bad things or just "things" . failing that, just build task 28". PREVIEW (added at the user's request): a third button beside Allow / Cancel that changes nothing and uses nothing. Skill: shows the full SKILL.md instructions and the contents of any bundled scripts, plus a plain-language 'what could go wrong' list derived from what it asks for (e.g. runs commands -&gt; could install software or delete files; you are still asked before risky commands) and the warning checks. Connector: starts it briefly in look-only mode to list every tool it really offers (name, description, whether it says it only reads) - nothing is callable by the AI - then stops it; for a remote connector it shows the address it talks to. No AI 'prediction' step: a model reading an untrusted skill could itself be misled by it, so the preview is built from facts, not guesses.</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): Task 28 built (PR #18), skills off by default (D38), the Radium logo (Task 29, D37), v2.0.40
- Task 28: built and in PR #18. The user's amendments are recorded on D36:
  every skill and plugin, bundled or from Anthropic, goes through
  Allow / Preview / Cancel; and, after testing, Preview lists all tools at
  once and explains the command and what could go wrong. Steps S02-S05 and
  S07 done, S08 in progress, new S09 (skills off by default). S06 (safer MCP
  default) is still to do.
- D38: every skill is off by default (the user's instruction).
- Task 29 and D37: the user's Radium logo replaces the Atomic mark everywhere
  (PR #19, on #16).
- Task 27: T27-S05 done - v2.0.38 and v2.0.39 passed the version check and
  were tagged; v2.0.40 is the next combined build.
- Handover: install v2.0.40 and what to check; merge order.
- Fork features register: review-before-use and radium-logo rows.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1040,6 +1040,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -1192,7 +1193,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): (1) USER: install test build v2.0.39 (slim window strip, D35) when run 34843302629 finishes. (2) Task 28: review-before-use screens for skills and MCP connectors, re-review on change, safer MCP default, warnings - tests first. (3) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #17. (4) Task 26 when the user installs ComfyUI.</t>
+          <t>2026-09-14 (latest): (1) USER: install test build v2.0.40 when run 34861656623 finishes - it has everything so far: slim window strip (#10), Uncensored in the filter menu (#11), API/Cloud/run settings in Settings (#12), extensions fix (#15), rename (#16), version rule (#17), review before use with skills off by default (#18) and the Radium logo (#19). Check: connectors and skills ask for review (Preview lists tools and explains the command), the Radium logo on the taskbar/installer/sidebar, no Cloud or API in the sidebar. (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 28 left: T28-S06 safer MCP default (Allow all MCP permissions off for new installs). (4) Task 26 when the user installs ComfyUI.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2817,7 +2818,7 @@
       </c>
       <c r="K30" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: built and verified in PR #17. Next: the first build under the rule, v2.0.38, with #10, #11, #12, #15, #16, #17.</t>
+          <t>2026-09-14: built and verified in PR #17. Next: the first build under the rule, v2.0.38, with #10, #11, #12, #15, #16, #17. | 2026-09-14: the rule is working. v2.0.38 (run 34841320635) and v2.0.39 (run 34843302629) each passed the version check and were tagged; v2.0.40 (run 34861656623) is the combined build with Task 28 and the logo.</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2859,11 @@
           <t>No skill or connector is used until the user has seen, in plain language, what it can do and has allowed it; changed contents ask again; MCP actions that can change things ask by default; suspicious patterns are shown as warnings; tests cover each.</t>
         </is>
       </c>
-      <c r="I31" s="13" t="inlineStr"/>
+      <c r="I31" s="13" t="inlineStr">
+        <is>
+          <t>fb9b5b196, fd2133e47, 055f7c4d6 (PR #18)</t>
+        </is>
+      </c>
       <c r="J31" s="14" t="inlineStr">
         <is>
           <t>ADDED 2026-09-14 at the user's request: "what can we do against malicious code are actions in regards to skills and MCP's? is there some sort of auto checker anti virus for MCP's and skills? at the very least can we create a pop window or user verifiable before proceeding pop up screen that clearly lists what the skill or mcp can do or has access to before actually using it?" MEASURED ON MAIN 2026-09-14. WHAT EXISTS: (1) Per-action approval for the agent's own tools: a dialog shows the tool, the reason, a preview of the arguments and the files it touches, with Deny / Approve once / Always allow (ADRs 2026-07-16, 2026-07-23; AgentApprovalDialog.tsx). Reading inside the workspace needs no approval; writing, deleting, leaving the workspace and flagged shell commands do. (2) A shell guard hard-blocks the worst commands (e.g. 'rm -rf /', formatting a disk) even when approvals are skipped, and asks before sudo, chmod, curl, wget, shutdown (shell_guard.rs). (3) Skill import checks: SKILL.md must parse, name/description required, unknown header fields and symlinks refused, prompt-injection-looking catalog text refused (authoring.rs, manifest.rs). Skills can declare 'dangerous', 'requires_tools', 'requires_scripts', but these are only passed to the AI as text. (4) Per-tool on/off switches for each MCP connector (ADR 2026-09-02). GAPS: (a) 'Allow all MCP permissions' defaults to ON, and a one-time migration forced it ON for every existing user (useToolApproval.ts), so MCP tools that can change things run without asking. (b) Whether an MCP tool counts as read-only comes from the server's own readOnlyHint - a malicious server can simply claim it. (c) A new skill or connector is usable as soon as it is added: nothing shows the user what it asks for, and nothing asks again when its contents change. (d) There is no scanner. None can prove a skill (plain instructions) or an MCP server (someone else's program or web service) is safe; pattern checks can only warn.</t>
@@ -2866,7 +2871,60 @@
       </c>
       <c r="K31" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: the user asked for a Preview option alongside Allow / Cancel (see D36 amendment) and to build Task 28.</t>
+          <t>2026-09-14: the user asked for a Preview option alongside Allow / Cancel (see D36 amendment) and to build Task 28. | 2026-09-14: BUILT (PR #18). Skills: the core fingerprints every file of a skill and only offers it to the AI once the user allowed it as it is now; review screen with what it can do, warnings and Preview (full instructions and scripts). Connectors: the core refuses to start any connector the user has not allowed as it is now (checked in start_mcp_server, so launch, every switch and sign-in retries are covered); one review screen for the Connectors page, chat connectors menu, web search button and browser button. AMENDED BY THE USER: every skill and plugin, bundled with Radium or from Anthropic included, goes through Allow / Preview / Cancel - no exemptions, no auto-allow for skills written in Radium. After trying it on this PC the user asked for Preview to list all tools straight away and for more detail about the command and what could go wrong - both done: each part of the command explained, a 'what could go wrong' list from the settings, each tool's inputs, what it says about itself and clues from its name. The user also asked that every skill is off by default (D38) - done. Still to do: T28-S06 safer MCP default.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>Task 29</t>
+        </is>
+      </c>
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>11 - Brand</t>
+        </is>
+      </c>
+      <c r="C32" s="14" t="inlineStr">
+        <is>
+          <t>The new Radium logo everywhere</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Laptop, then this PC</t>
+        </is>
+      </c>
+      <c r="E32" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="14" t="inlineStr">
+        <is>
+          <t>#16 (merge first).</t>
+        </is>
+      </c>
+      <c r="H32" s="14" t="inlineStr">
+        <is>
+          <t>The Radium logo is the app, taskbar, Start menu and installer icon and shows in the sidebar, setup, loading screen and avatars, in full colour; no Atomic mark is left.</t>
+        </is>
+      </c>
+      <c r="I32" s="13" t="inlineStr">
+        <is>
+          <t>351150e46 (PR #19)</t>
+        </is>
+      </c>
+      <c r="J32" s="14" t="inlineStr">
+        <is>
+          <t>ADDED 2026-09-14 at the user's instruction: "Relace the Atomic logo wherever it still exists. Replace the app logo, any setup pages, everything. Replace it with the one I just uploaded and resize to an appropriate size. We still need to update the logo and old atomic name still showing on the main chat page."</t>
+        </is>
+      </c>
+      <c r="K32" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: the logo came from C:\Users\Warwick\Downloads\Radium LOGO.jpg (2048x2048). Trimmed to its rounded tile with transparent corners: 1024x1024 app icon source (src-tauri/icons/icon.png, the only tracked icon; tauri icon generates the rest) and 512x512 web logo images. The inverting/tinting that suited the old black-and-white mark is removed everywhere. The 'Atomic Chat' name still on the main chat page in the tested build was the sidebar wordmark, replaced by #16, which was not in that build. Left alone: the macOS tray template (must be a one-colour silhouette) and other products' names (Atomic Mail, Atomic Agent, AtomicChat model mirrors).</t>
         </is>
       </c>
     </row>
@@ -2887,7 +2945,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I216"/>
+  <dimension ref="A1:I221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11330,7 +11388,7 @@
       </c>
       <c r="E207" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F207" s="13" t="inlineStr"/>
@@ -11346,7 +11404,7 @@
       </c>
       <c r="I207" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: v2.0.38 was the first build under the rule (run 34841320635): still building when this was recorded; its version check step passed on the runner. The user then asked for the D35 window strip, so the next build is v2.0.39 (run 34843302629).</t>
+          <t>2026-09-14: v2.0.38 was the first build under the rule (run 34841320635): still building when this was recorded; its version check step passed on the runner. The user then asked for the D35 window strip, so the next build is v2.0.39 (run 34843302629). | 2026-09-14: DONE. v2.0.38 (run 34841320635) and v2.0.39 (run 34843302629) passed the version check step and were tagged test-build/v2.0.38 and test-build/v2.0.39. Next build v2.0.40 (run 34861656623).</t>
         </is>
       </c>
     </row>
@@ -11453,7 +11511,7 @@
       </c>
       <c r="E210" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F210" s="13" t="inlineStr"/>
@@ -11469,7 +11527,7 @@
       </c>
       <c r="I210" s="15" t="inlineStr">
         <is>
-          <t>Run red first, for the right reason.</t>
+          <t>Run red first, for the right reason. | 2026-09-14: done - tests written first and seen failing for the right reason for each part (Rust registry and connector reviews, web dialogs, pages, queue and host).</t>
         </is>
       </c>
     </row>
@@ -11494,7 +11552,7 @@
       </c>
       <c r="E211" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F211" s="13" t="inlineStr"/>
@@ -11510,7 +11568,7 @@
       </c>
       <c r="I211" s="15" t="inlineStr">
         <is>
-          <t>Plain language, not tool ids. | 2026-09-14: add Preview (full instructions, scripts, what-could-go-wrong list) per the D36 amendment.</t>
+          <t>Plain language, not tool ids. | 2026-09-14: add Preview (full instructions, scripts, what-could-go-wrong list) per the D36 amendment. | 2026-09-14: done (fb9b5b196). Shown when a skill is switched on unreviewed and straight after it is uploaded or written; bundled skills included (user's amendment).</t>
         </is>
       </c>
     </row>
@@ -11535,7 +11593,7 @@
       </c>
       <c r="E212" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F212" s="13" t="inlineStr"/>
@@ -11551,7 +11609,7 @@
       </c>
       <c r="I212" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: add Preview (look-only start that lists the connector's real tools, then stops) per the D36 amendment.</t>
+          <t>2026-09-14: add Preview (look-only start that lists the connector's real tools, then stops) per the D36 amendment. | 2026-09-14: done (fd2133e47, 055f7c4d6). One host dialog for every place a connector is switched on; Preview lists tools at once and explains the command and what could go wrong (user's request after testing).</t>
         </is>
       </c>
     </row>
@@ -11576,7 +11634,7 @@
       </c>
       <c r="E213" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F213" s="13" t="inlineStr"/>
@@ -11592,7 +11650,7 @@
       </c>
       <c r="I213" s="15" t="inlineStr">
         <is>
-          <t>The same idea as 'Always allow' fingerprints in ADR 2026-07-23.</t>
+          <t>The same idea as 'Always allow' fingerprints in ADR 2026-07-23. | 2026-09-14: done. Skills: SHA-256 of every file (.reviewed.json). Connectors: fingerprint of type, address, command, arguments, folder, key and header names (mcp_reviewed.json); key values and on/off do not ask again.</t>
         </is>
       </c>
     </row>
@@ -11658,7 +11716,7 @@
       </c>
       <c r="E215" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F215" s="13" t="inlineStr"/>
@@ -11674,7 +11732,7 @@
       </c>
       <c r="I215" s="15" t="inlineStr">
         <is>
-          <t>Warnings only; the screen says a clean check does not prove safety.</t>
+          <t>Warnings only; the screen says a clean check does not prove safety. | 2026-09-14: done. Pattern warnings with the text that raised them; the screen says a clean check is not a guarantee.</t>
         </is>
       </c>
     </row>
@@ -11699,7 +11757,7 @@
       </c>
       <c r="E216" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F216" s="13" t="inlineStr"/>
@@ -11713,7 +11771,226 @@
           <t>This PC</t>
         </is>
       </c>
-      <c r="I216" s="15" t="inlineStr"/>
+      <c r="I216" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: PR #18. Rust 856 tests, clippy, rustfmt; web 302 files / 3527 tests, typecheck, lint, test-quality, hardening 40/40, media guard. Tried on this PC in a dev build (Exa refused at launch until reviewed; serper review and Preview shown). Combined build v2.0.40 (run 34861656623) for the user to install.</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="6" t="inlineStr">
+        <is>
+          <t>T28-S09</t>
+        </is>
+      </c>
+      <c r="B217" s="17" t="inlineStr">
+        <is>
+          <t>Task 28</t>
+        </is>
+      </c>
+      <c r="C217" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D217" s="14" t="inlineStr">
+        <is>
+          <t>Every skill starts switched off</t>
+        </is>
+      </c>
+      <c r="E217" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F217" s="13" t="n"/>
+      <c r="G217" s="14" t="inlineStr">
+        <is>
+          <t>A skill shows as on only once the user has allowed it as it is now; a changed skill shows as off again (registry test every_skill_starts_switched_off_until_the_user_allows_it).</t>
+        </is>
+      </c>
+      <c r="H217" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I217" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: the user's instruction (D38); done in 055f7c4d6.</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="6" t="inlineStr">
+        <is>
+          <t>T29-S01</t>
+        </is>
+      </c>
+      <c r="B218" s="17" t="inlineStr">
+        <is>
+          <t>Task 29</t>
+        </is>
+      </c>
+      <c r="C218" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D218" s="14" t="inlineStr">
+        <is>
+          <t>Prepare the logo images</t>
+        </is>
+      </c>
+      <c r="E218" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F218" s="13" t="n"/>
+      <c r="G218" s="14" t="inlineStr">
+        <is>
+          <t>Trim the uploaded logo to its tile with transparent corners; 1024x1024 icon source and 512x512 web images; generate all app icons with tauri icon to check.</t>
+        </is>
+      </c>
+      <c r="H218" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I218" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: done; 128x128 and 32x32 icons checked by eye.</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="6" t="inlineStr">
+        <is>
+          <t>T29-S02</t>
+        </is>
+      </c>
+      <c r="B219" s="17" t="inlineStr">
+        <is>
+          <t>Task 29</t>
+        </is>
+      </c>
+      <c r="C219" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D219" s="14" t="inlineStr">
+        <is>
+          <t>Write the failing tests first</t>
+        </is>
+      </c>
+      <c r="E219" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F219" s="13" t="n"/>
+      <c r="G219" s="14" t="inlineStr">
+        <is>
+          <t>node --test tests/radium-logo.test.mjs (icon size and transparency, every logo image replaced, no screen inverts it); AppLogo test for the colour logo.</t>
+        </is>
+      </c>
+      <c r="H219" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I219" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: seen failing before the change (2 contract checks, 1 AppLogo test).</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="6" t="inlineStr">
+        <is>
+          <t>T29-S03</t>
+        </is>
+      </c>
+      <c r="B220" s="17" t="inlineStr">
+        <is>
+          <t>Task 29</t>
+        </is>
+      </c>
+      <c r="C220" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D220" s="14" t="inlineStr">
+        <is>
+          <t>Replace the logo everywhere</t>
+        </is>
+      </c>
+      <c r="E220" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F220" s="13" t="n"/>
+      <c r="G220" s="14" t="inlineStr">
+        <is>
+          <t>Icon source, web logo images, sidebar, setup screen, loading screen, avatars, diagram error, vision prompt.</t>
+        </is>
+      </c>
+      <c r="H220" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I220" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: 351150e46 (PR #19, on #16). Web 297 files / 3466 tests, typecheck, lint, test-quality, hardening 44/44.</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="6" t="inlineStr">
+        <is>
+          <t>T29-S04</t>
+        </is>
+      </c>
+      <c r="B221" s="17" t="inlineStr">
+        <is>
+          <t>Task 29</t>
+        </is>
+      </c>
+      <c r="C221" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D221" s="14" t="inlineStr">
+        <is>
+          <t>Check it on this PC</t>
+        </is>
+      </c>
+      <c r="E221" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F221" s="13" t="n"/>
+      <c r="G221" s="14" t="inlineStr">
+        <is>
+          <t>Install v2.0.40: taskbar, Start menu, installer, window and sidebar show the Radium logo; no Atomic name on the main chat page.</t>
+        </is>
+      </c>
+      <c r="H221" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I221" s="15" t="inlineStr">
+        <is>
+          <t>Combined build v2.0.40, run 34861656623.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -11732,7 +12009,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13317,7 +13594,7 @@
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>REQUESTED BY THE USER 2026-09-14: "what can we do against malicious code are actions in regards to skills and MCP's? is there some sort of auto checker anti virus for MCP's and skills? at the very least can we create a pop window or user verifiable before proceeding pop up screen that clearly lists what the skill or mcp can do or has access to before actually using it?". Point (1) is the user's request. Points (2)-(4) were added by the agent under the user's standing 'just act' instruction; (3) changes a default, so existing users are told once and choose. The user can drop any of them. | AMENDED BY THE USER 2026-09-14: "task 28 1. allow and cancel. can we create a "preview" option to? not sure what this would do, maybe predict or list the potential bad things or just "things" . failing that, just build task 28". PREVIEW (added at the user's request): a third button beside Allow / Cancel that changes nothing and uses nothing. Skill: shows the full SKILL.md instructions and the contents of any bundled scripts, plus a plain-language 'what could go wrong' list derived from what it asks for (e.g. runs commands -&gt; could install software or delete files; you are still asked before risky commands) and the warning checks. Connector: starts it briefly in look-only mode to list every tool it really offers (name, description, whether it says it only reads) - nothing is callable by the AI - then stops it; for a remote connector it shows the address it talks to. No AI 'prediction' step: a model reading an untrusted skill could itself be misled by it, so the preview is built from facts, not guesses.</t>
+          <t>REQUESTED BY THE USER 2026-09-14: "what can we do against malicious code are actions in regards to skills and MCP's? is there some sort of auto checker anti virus for MCP's and skills? at the very least can we create a pop window or user verifiable before proceeding pop up screen that clearly lists what the skill or mcp can do or has access to before actually using it?". Point (1) is the user's request. Points (2)-(4) were added by the agent under the user's standing 'just act' instruction; (3) changes a default, so existing users are told once and choose. The user can drop any of them. | AMENDED BY THE USER 2026-09-14: "task 28 1. allow and cancel. can we create a "preview" option to? not sure what this would do, maybe predict or list the potential bad things or just "things" . failing that, just build task 28". PREVIEW (added at the user's request): a third button beside Allow / Cancel that changes nothing and uses nothing. Skill: shows the full SKILL.md instructions and the contents of any bundled scripts, plus a plain-language 'what could go wrong' list derived from what it asks for (e.g. runs commands -&gt; could install software or delete files; you are still asked before risky commands) and the warning checks. Connector: starts it briefly in look-only mode to list every tool it really offers (name, description, whether it says it only reads) - nothing is callable by the AI - then stops it; for a remote connector it shows the address it talks to. No AI 'prediction' step: a model reading an untrusted skill could itself be misled by it, so the preview is built from facts, not guesses. | AMENDED BY THE USER 2026-09-14: "we need to put the preview and allow and cancel options on every skill and every plug in. doesn't matter if it's been bundled with Radium or comes from Anthropic themselves. This system of Allow, Preview and cancel needs to be backed into Radium. If the user is able to connect to new mcp's or download and upload skills the the review process or the ability to review the mcp or skill to create the "preview" of that skill or mcp needs to happen to every one that gets imported or uploaded to Radium" - so no skill or connector is exempt, and enforcement is in the core, not just the screen. AMENDED BY THE USER 2026-09-14 after testing: "In preview mode, list all the tools as default. Can we also go into more detail about the commands it runs and any potential issues that may happen?" - Preview now lists every tool at once (starting a local program briefly) and explains each part of the command, what could go wrong, and each tool's inputs and labels.</t>
         </is>
       </c>
       <c r="F43" s="13" t="inlineStr">
@@ -13326,6 +13603,80 @@
         </is>
       </c>
       <c r="G43" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>D37</t>
+        </is>
+      </c>
+      <c r="B44" s="14" t="inlineStr">
+        <is>
+          <t>WHICH LOGO DOES RADIUM USE? (Task 29)</t>
+        </is>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>Task 29.</t>
+        </is>
+      </c>
+      <c r="D44" s="14" t="inlineStr">
+        <is>
+          <t>The user's instruction, not a recommendation.</t>
+        </is>
+      </c>
+      <c r="E44" s="15" t="inlineStr">
+        <is>
+          <t>DECIDED BY THE USER 2026-09-14: "Relace the Atomic logo wherever it still exists. Replace the app logo, any setup pages, everything. Replace it with the one I just uploaded and resize to an appropriate size." The uploaded 'R' tile (Downloads\Radium LOGO.jpg) is the logo everywhere; it is shown in full colour, never inverted.</t>
+        </is>
+      </c>
+      <c r="F44" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G44" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>D38</t>
+        </is>
+      </c>
+      <c r="B45" s="14" t="inlineStr">
+        <is>
+          <t>WHAT IS A SKILL'S DEFAULT STATE? (Task 28)</t>
+        </is>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>Task 28.</t>
+        </is>
+      </c>
+      <c r="D45" s="14" t="inlineStr">
+        <is>
+          <t>The user's instruction, not a recommendation.</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>DECIDED BY THE USER 2026-09-14: "All skills should automatically be set to off for it's default state." Every skill, bundled or added, shows as off until the user has allowed it (Allow on its review); a skill that changes shows as off again.</t>
+        </is>
+      </c>
+      <c r="F45" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G45" s="13" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
@@ -13855,7 +14206,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -14500,6 +14851,104 @@
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
+        <is>
+          <t>Waiting for its PR to merge</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="24" t="inlineStr">
+        <is>
+          <t>review-before-use</t>
+        </is>
+      </c>
+      <c r="B17" s="24" t="inlineStr">
+        <is>
+          <t>Review before use for every skill and connector</t>
+        </is>
+      </c>
+      <c r="C17" s="24" t="inlineStr">
+        <is>
+          <t>No skill or MCP connector is used until you have seen what it can do and chosen Allow (with Preview and Cancel); it asks again when it changes, and every skill starts switched off (tracker D36, D38).</t>
+        </is>
+      </c>
+      <c r="D17" s="24" t="inlineStr">
+        <is>
+          <t>src-tauri/src/core/mcp/review.rs
+src-tauri/src/core/mcp/helpers.rs
+src-tauri/src/core/agent/skills/registry.rs
+src-tauri/src/core/agent/skills/commands.rs
+web-app/src/lib/review-before-use.ts
+web-app/src/containers/SkillReviewDialog.tsx
+web-app/src/containers/ConnectorReviewDialog.tsx
+web-app/src/containers/dialogs/ConnectorReviewHost.tsx
+web-app/src/hooks/useConnectorReview.ts
+web-app/src/routes/connectors/index.tsx
+web-app/src/routes/skills/index.tsx
+web-app/src/locales/en/review.json</t>
+        </is>
+      </c>
+      <c r="E17" s="24" t="inlineStr">
+        <is>
+          <t>cargo test --no-default-features --features test-tauri --lib -- core::mcp core::agent::skills
+npx vitest run src/lib/__tests__/review-before-use.test.ts src/containers/__tests__/SkillReviewDialog.test.tsx src/containers/__tests__/ConnectorReviewDialog.test.tsx src/containers/dialogs/__tests__/ConnectorReviewHost.test.tsx src/hooks/__tests__/useConnectorReview.test.ts src/routes/skills/__tests__/SkillsPage.review.test.tsx src/routes/connectors/__tests__/index.test.tsx</t>
+        </is>
+      </c>
+      <c r="F17" s="24" t="inlineStr">
+        <is>
+          <t>Tracker D36, D38, Task 28 (PR #18)</t>
+        </is>
+      </c>
+      <c r="G17" s="24" t="inlineStr">
+        <is>
+          <t>Waiting for its PR to merge</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>radium-logo</t>
+        </is>
+      </c>
+      <c r="B18" s="24" t="inlineStr">
+        <is>
+          <t>The Radium logo</t>
+        </is>
+      </c>
+      <c r="C18" s="24" t="inlineStr">
+        <is>
+          <t>The Radium 'R' logo is the app and installer icon and appears in the sidebar, setup and loading screens and chat avatars, shown in full colour (tracker D37).</t>
+        </is>
+      </c>
+      <c r="D18" s="24" t="inlineStr">
+        <is>
+          <t>src-tauri/icons/icon.png
+web-app/public/images/transparent-logo.png
+web-app/public/images/atomic-chat-logo.png
+web-app/public/images/logo.png
+web-app/public/images/logo-app.png
+web-app/src/components/AppLogo.tsx
+web-app/src/containers/SetupBackendStep.tsx
+web-app/src/containers/AvatarEmoji.tsx
+web-app/src/components/MermaidError.tsx
+web-app/src/containers/PromptVisionModel.tsx
+web-app/src/loader.css
+web-app/index.html</t>
+        </is>
+      </c>
+      <c r="E18" s="24" t="inlineStr">
+        <is>
+          <t>node --test tests/radium-logo.test.mjs
+npx vitest run src/components/__tests__/AppLogo.test.tsx</t>
+        </is>
+      </c>
+      <c r="F18" s="24" t="inlineStr">
+        <is>
+          <t>Tracker D37, Task 29 (PR #19)</t>
+        </is>
+      </c>
+      <c r="G18" s="24" t="inlineStr">
         <is>
           <t>Waiting for its PR to merge</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): v2.0.40 failed its typecheck, #18 fixed, v2.0.41 built
- v2.0.40 (run 34861656623) failed at tsc -b: two typing mistakes in #18. The
  local check had run tsc -p ., which checks no files; the working rule is now
  tsc -b, as the build runs it. Fixed in #18 (32eda45c9, bbb08f727).
- v2.0.41 (run 34871145162) built successfully with #10, #11, #12, #15, #16,
  #17, #18 and #19. Full web suite on the combined code: 305 files, 3539 tests.
- Handover: install v2.0.41 and what to check; merge order unchanged.
- Evidence: local typecheck now matches the build.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): (1) USER: install test build v2.0.40 when run 34861656623 finishes - it has everything so far: slim window strip (#10), Uncensored in the filter menu (#11), API/Cloud/run settings in Settings (#12), extensions fix (#15), rename (#16), version rule (#17), review before use with skills off by default (#18) and the Radium logo (#19). Check: connectors and skills ask for review (Preview lists tools and explains the command), the Radium logo on the taskbar/installer/sidebar, no Cloud or API in the sidebar. (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 28 left: T28-S06 safer MCP default (Allow all MCP permissions off for new installs). (4) Task 26 when the user installs ComfyUI.</t>
+          <t>2026-09-14 (latest): (1) USER: install test build v2.0.41 (run 34871145162) - BUILT SUCCESSFULLY 2026-09-14 (16:51-17:28 UTC); the installer is the run's artifact, ready for the user to install. It has everything so far: slim window strip (#10), Uncensored in the filter menu (#11), API/Cloud/run settings in Settings (#12), extensions fix (#15), rename (#16), version rule (#17), review before use with skills off by default (#18) and the Radium logo (#19). v2.0.40 did not build (typecheck mistakes in #18, now fixed). Check: connectors and skills ask for review (Preview lists tools and explains the command), every skill starts off, the Radium logo on the taskbar/installer/sidebar, no Cloud or API in the sidebar. (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 28 left: T28-S06 safer MCP default. (4) Task 26 when the user installs ComfyUI. (5) Working rule learned: check the web app with 'tsc -b' (as the build does), not 'tsc -p .'.</t>
         </is>
       </c>
     </row>
@@ -2817,7 +2817,7 @@
       </c>
       <c r="K30" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: built and verified in PR #17. Next: the first build under the rule, v2.0.38, with #10, #11, #12, #15, #16, #17. | 2026-09-14: the rule is working. v2.0.38 (run 34841320635) and v2.0.39 (run 34843302629) each passed the version check and were tagged; v2.0.40 (run 34861656623) is the combined build with Task 28 and the logo.</t>
+          <t>2026-09-14: built and verified in PR #17. Next: the first build under the rule, v2.0.38, with #10, #11, #12, #15, #16, #17. | 2026-09-14: the rule is working. v2.0.38 (run 34841320635) and v2.0.39 (run 34843302629) each passed the version check and were tagged; v2.0.40 (run 34861656623) is the combined build with Task 28 and the logo. | 2026-09-14: v2.0.40 failed its typecheck, so the rebuild took a new number, v2.0.41 (run 34871145162), as the rule requires: BUILT SUCCESSFULLY 2026-09-14 (16:51-17:28 UTC); the installer is the run's artifact, ready for the user to install.</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2860,7 @@
       </c>
       <c r="I31" s="13" t="inlineStr">
         <is>
-          <t>fb9b5b196, fd2133e47, 055f7c4d6 (PR #18)</t>
+          <t>fb9b5b196, fd2133e47, 055f7c4d6, 32eda45c9, bbb08f727 (PR #18)</t>
         </is>
       </c>
       <c r="J31" s="14" t="inlineStr">
@@ -2870,7 +2870,7 @@
       </c>
       <c r="K31" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: the user asked for a Preview option alongside Allow / Cancel (see D36 amendment) and to build Task 28. | 2026-09-14: BUILT (PR #18). Skills: the core fingerprints every file of a skill and only offers it to the AI once the user allowed it as it is now; review screen with what it can do, warnings and Preview (full instructions and scripts). Connectors: the core refuses to start any connector the user has not allowed as it is now (checked in start_mcp_server, so launch, every switch and sign-in retries are covered); one review screen for the Connectors page, chat connectors menu, web search button and browser button. AMENDED BY THE USER: every skill and plugin, bundled with Radium or from Anthropic included, goes through Allow / Preview / Cancel - no exemptions, no auto-allow for skills written in Radium. After trying it on this PC the user asked for Preview to list all tools straight away and for more detail about the command and what could go wrong - both done: each part of the command explained, a 'what could go wrong' list from the settings, each tool's inputs, what it says about itself and clues from its name. The user also asked that every skill is off by default (D38) - done. Still to do: T28-S06 safer MCP default.</t>
+          <t>2026-09-14: the user asked for a Preview option alongside Allow / Cancel (see D36 amendment) and to build Task 28. | 2026-09-14: BUILT (PR #18). Skills: the core fingerprints every file of a skill and only offers it to the AI once the user allowed it as it is now; review screen with what it can do, warnings and Preview (full instructions and scripts). Connectors: the core refuses to start any connector the user has not allowed as it is now (checked in start_mcp_server, so launch, every switch and sign-in retries are covered); one review screen for the Connectors page, chat connectors menu, web search button and browser button. AMENDED BY THE USER: every skill and plugin, bundled with Radium or from Anthropic included, goes through Allow / Preview / Cancel - no exemptions, no auto-allow for skills written in Radium. After trying it on this PC the user asked for Preview to list all tools straight away and for more detail about the command and what could go wrong - both done: each part of the command explained, a 'what could go wrong' list from the settings, each tool's inputs, what it says about itself and clues from its name. The user also asked that every skill is off by default (D38) - done. Still to do: T28-S06 safer MCP default. | 2026-09-14: v2.0.40 (run 34861656623) FAILED at 'Build unsigned Windows app': the strict typecheck (tsc -b) rejected two mistakes in #18 - DefaultMCPService's three new review functions took no parameters, so the desktop versions (name, config) did not match them, and the Connectors page passed a caught error (unknown) as the error message. CAUSE OF THE MISS: the local check ran 'tsc -p .' against web-app/tsconfig.json, which lists no files and so checked nothing; the build runs 'tsc -b'. From now on the local check is 'tsc -b', as the build runs it. FIXED in #18: 32eda45c9 (types) and bbb08f727 (the first fix left unused parameters that lint rejected; the fallback functions now log their inputs like the rest of the file). Rebuilt as v2.0.41 (run 34871145162): BUILT SUCCESSFULLY 2026-09-14 (16:51-17:28 UTC); the installer is the run's artifact, ready for the user to install.</t>
         </is>
       </c>
     </row>
@@ -11772,7 +11772,7 @@
       </c>
       <c r="I216" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: PR #18. Rust 856 tests, clippy, rustfmt; web 302 files / 3527 tests, typecheck, lint, test-quality, hardening 40/40, media guard. Tried on this PC in a dev build (Exa refused at launch until reviewed; serper review and Preview shown). Combined build v2.0.40 (run 34861656623) for the user to install.</t>
+          <t>2026-09-14: PR #18. Rust 856 tests, clippy, rustfmt; web 302 files / 3527 tests, typecheck, lint, test-quality, hardening 40/40, media guard. Tried on this PC in a dev build (Exa refused at launch until reviewed; serper review and Preview shown). Combined build v2.0.40 (run 34861656623) for the user to install. | 2026-09-14: v2.0.40 (run 34861656623) FAILED at 'Build unsigned Windows app': the strict typecheck (tsc -b) rejected two mistakes in #18 - DefaultMCPService's three new review functions took no parameters, so the desktop versions (name, config) did not match them, and the Connectors page passed a caught error (unknown) as the error message. CAUSE OF THE MISS: the local check ran 'tsc -p .' against web-app/tsconfig.json, which lists no files and so checked nothing; the build runs 'tsc -b'. From now on the local check is 'tsc -b', as the build runs it. FIXED in #18: 32eda45c9 (types) and bbb08f727 (the first fix left unused parameters that lint rejected; the fallback functions now log their inputs like the rest of the file). v2.0.41 (run 34871145162): BUILT SUCCESSFULLY 2026-09-14 (16:51-17:28 UTC); the installer is the run's artifact, ready for the user to install. Web suite on the combined 2.0.41 code: 305 test files, 3539 tests passed (11 skipped); test-quality guard and selective media guard passed; strict typecheck (tsc -b), whole-app lint (0 errors) and 60 of 60 hardening contracts passed before the push.</t>
         </is>
       </c>
     </row>
@@ -11987,7 +11987,7 @@
       </c>
       <c r="I221" s="15" t="inlineStr">
         <is>
-          <t>Combined build v2.0.40, run 34861656623.</t>
+          <t>Combined build v2.0.40, run 34861656623. | 2026-09-14: v2.0.40 did not build (Task 28 typecheck, not the logo); install v2.0.41 (run 34871145162) instead: BUILT SUCCESSFULLY 2026-09-14 (16:51-17:28 UTC); the installer is the run's artifact, ready for the user to install.</t>
         </is>
       </c>
     </row>
@@ -13697,7 +13697,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -14186,6 +14186,41 @@
       <c r="D15" t="inlineStr">
         <is>
           <t>Task 1 code complete through T01-S05; commit (T01-S06) not yet authorised.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Local typecheck matches the build (tsc -b)</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>web-app (npx tsc -b)</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Captured</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Tracker Task 28 notes; #18 commits 32eda45c9, bbb08f727</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>v2.0.40 failed because 'tsc -p .' checks no files (tsconfig.json has files: []). tsc -b passed on #18 and on the combined 2.0.41 code before it was pushed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): Task 30 built-in media engine (D39, D40); installer and uninstaller logo (T29-S05)
- Task 30: Radium gets its own media engine (stable-diffusion.cpp with CUDA,
  Vulkan and CPU builds and a model catalog), while ComfyUI and cloud
  providers stay available through an Image provider drop-down, with more
  providers added and CUDA checked on the dual-3090 desktop. Steps S01-S12.
  Task 26 (ComfyUI set-up) is superseded as the out-of-the-box path.
- D39 and D40 record the user's decisions in their own words.
- T29-S05, from the user's screenshot of the Radium Uninstall window: the
  installer and uninstaller windows' title-bar icon and header image must show
  the Radium logo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): (1) USER: install test build v2.0.41 (run 34871145162) - BUILT SUCCESSFULLY 2026-09-14 (16:51-17:28 UTC); the installer is the run's artifact, ready for the user to install. It has everything so far: slim window strip (#10), Uncensored in the filter menu (#11), API/Cloud/run settings in Settings (#12), extensions fix (#15), rename (#16), version rule (#17), review before use with skills off by default (#18) and the Radium logo (#19). v2.0.40 did not build (typecheck mistakes in #18, now fixed). Check: connectors and skills ask for review (Preview lists tools and explains the command), every skill starts off, the Radium logo on the taskbar/installer/sidebar, no Cloud or API in the sidebar. (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 28 left: T28-S06 safer MCP default. (4) Task 26 when the user installs ComfyUI. (5) Working rule learned: check the web app with 'tsc -b' (as the build does), not 'tsc -p .'.</t>
+          <t>2026-09-14 (latest): (1) USER: install test build v2.0.41 (run 34871145162) - BUILT SUCCESSFULLY 2026-09-14 (16:51-17:28 UTC); the installer is the run's artifact, ready for the user to install. It has everything so far: slim window strip (#10), Uncensored in the filter menu (#11), API/Cloud/run settings in Settings (#12), extensions fix (#15), rename (#16), version rule (#17), review before use with skills off by default (#18) and the Radium logo (#19). v2.0.40 did not build (typecheck mistakes in #18, now fixed). Check: connectors and skills ask for review (Preview lists tools and explains the command), every skill starts off, the Radium logo on the taskbar/installer/sidebar, no Cloud or API in the sidebar. (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 28 left: T28-S06 safer MCP default. (4) Task 26 when the user installs ComfyUI. (5) Working rule learned: check the web app with 'tsc -b' (as the build does), not 'tsc -p .'. | 2026-09-14 (later): Task 30 started - built-in media engine and Image provider choice (D39, D40); plan on feat/builtin-media-engine. First: S01 proof image on this PC. Task 29 gained T29-S05: the installer and uninstaller windows' title-bar icon and header image must show the Radium logo (user's screenshot).</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K32"/>
+  <dimension ref="A1:K33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2766,7 +2766,11 @@
           <t>ADDED 2026-09-13 after the user asked how to get Radium Media running and whether any model can now be downloaded and used. MEASURED ANSWER: Radium Media does not run media models itself. It talks to an engine through adapters (Radium Media Worker at 127.0.0.1:13420 - not installed on this PC and not published; ComfyUI - two text-to-image workflow templates, uses whatever checkpoints ComfyUI has; OpenAI-compatible images / custom HTTP - declared model gpt-image-1, needs a key and costs money). 'Model agnostic' means the engine is pluggable, not that Radium downloads and runs any media model the way it does chat models. The remote media registry (Task 15) is not implemented and its URL returns 404. No end-to-end generation has ever run. This PC (AMD integrated GPU, 14.8 GB RAM) cannot run Wan 2.2 video (needs a ~24 GB NVIDIA GPU).</t>
         </is>
       </c>
-      <c r="K29" s="15" t="inlineStr"/>
+      <c r="K29" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: SUPERSEDED as the out-of-the-box path by Task 30 (built-in engine), at the user's request. ComfyUI stays available as one provider in the Image provider choice.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -2923,7 +2927,60 @@
       </c>
       <c r="K32" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: the logo came from C:\Users\Warwick\Downloads\Radium LOGO.jpg (2048x2048). Trimmed to its rounded tile with transparent corners: 1024x1024 app icon source (src-tauri/icons/icon.png, the only tracked icon; tauri icon generates the rest) and 512x512 web logo images. The inverting/tinting that suited the old black-and-white mark is removed everywhere. The 'Atomic Chat' name still on the main chat page in the tested build was the sidebar wordmark, replaced by #16, which was not in that build. Left alone: the macOS tray template (must be a one-colour silhouette) and other products' names (Atomic Mail, Atomic Agent, AtomicChat model mirrors).</t>
+          <t>2026-09-14: the logo came from C:\Users\Warwick\Downloads\Radium LOGO.jpg (2048x2048). Trimmed to its rounded tile with transparent corners: 1024x1024 app icon source (src-tauri/icons/icon.png, the only tracked icon; tauri icon generates the rest) and 512x512 web logo images. The inverting/tinting that suited the old black-and-white mark is removed everywhere. The 'Atomic Chat' name still on the main chat page in the tested build was the sidebar wordmark, replaced by #16, which was not in that build. Left alone: the macOS tray template (must be a one-colour silhouette) and other products' names (Atomic Mail, Atomic Agent, AtomicChat model mirrors). | 2026-09-14: THE USER ASKED (screenshot of the Radium Uninstall window, two places circled): "add to the tracker sheet to add the radium logo in the two places ive circled in red". The two places are the Windows installer/uninstaller window's title-bar icon (top left) and its header image (top right). The screenshot is the uninstaller of a build made before #19, so it still shows the Atomic mark. Both come from the app's Windows icon (icon.ico), which the build generates from src-tauri/icons/icon.png - now the Radium logo - so they should show the Radium logo from v2.0.41 on. To be checked, not assumed (T29-S05); if the header image turns out to come from a separate NSIS setting, set it explicitly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="B33" s="11" t="inlineStr">
+        <is>
+          <t>13 - Media</t>
+        </is>
+      </c>
+      <c r="C33" s="14" t="inlineStr">
+        <is>
+          <t>Built-in media engine and an image provider choice</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Laptop, this PC, then the dual-3090 desktop</t>
+        </is>
+      </c>
+      <c r="E33" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F33" s="13" t="n"/>
+      <c r="G33" s="14" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="H33" s="14" t="inlineStr">
+        <is>
+          <t>Installing Radium is enough to generate images: a built-in engine (stable-diffusion.cpp) with CUDA / Vulkan / CPU builds and a model catalog; an Image provider drop-down on the Media page listing Built-in, ComfyUI, cloud and other providers; CUDA verified on the dual-3090 desktop.</t>
+        </is>
+      </c>
+      <c r="I33" s="13" t="inlineStr">
+        <is>
+          <t>391956131 (plan)</t>
+        </is>
+      </c>
+      <c r="J33" s="14" t="inlineStr">
+        <is>
+          <t>ADDED 2026-09-14 at the user's request. The user asked how the Media page works and whether ComfyUI is required: "my initial plan was fir everything to be self contained". Answer measured from the code: Media has no engine of its own; it talks to a Radium Media Worker that is not in this repository, not published and not installed, to ComfyUI (user-installed) or to paid online services; nothing has ever generated end to end. The user said "build it" to a built-in engine, and added: "i still want the option to connect to comfyUI and the cloud and the local option ... Something like image processing provider with a drop down menu listing those providers I just listed and any other ones we can roll up into this" and "we need CUDA and Nvidia for when I get back to my dual 3090 desktop". Plan: docs/superpowers/plans/2026-09-14-builtin-media-engine.md (branch feat/builtin-media-engine).</t>
+        </is>
+      </c>
+      <c r="K33" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: S01 proof started. The user approved downloading sd-master-42d6c0a-bin-win-vulkan-x64.zip (37.3 MB), sd-master-42d6c0a-bin-win-cpu-x64.zip (23.2 MB) and stable-diffusion-v1-5-pruned-emaonly-Q8_0.gguf (1.68 GB) for a test on this PC, checked against the SHA-256 published by GitHub and Hugging Face. This PC: AMD Ryzen 7 7735U with Radeon graphics (Vulkan present), 14.8 GB RAM, 64.6 GB free. Reuse found: the core download manager already verifies size and SHA-256 with progress and cancel; tauri-plugin-hardware already detects NVIDIA / AMD / Intel GPUs (not in test builds); the core already has a decompress command used for llama.cpp backends.</t>
         </is>
       </c>
     </row>
@@ -2944,7 +3001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I221"/>
+  <dimension ref="A1:I234"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -11990,6 +12047,517 @@
           <t>Combined build v2.0.40, run 34861656623. | 2026-09-14: v2.0.40 did not build (Task 28 typecheck, not the logo); install v2.0.41 (run 34871145162) instead: BUILT SUCCESSFULLY 2026-09-14 (16:51-17:28 UTC); the installer is the run's artifact, ready for the user to install.</t>
         </is>
       </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="6" t="inlineStr">
+        <is>
+          <t>T29-S05</t>
+        </is>
+      </c>
+      <c r="B222" s="17" t="inlineStr">
+        <is>
+          <t>Task 29</t>
+        </is>
+      </c>
+      <c r="C222" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D222" s="14" t="inlineStr">
+        <is>
+          <t>Installer and uninstaller windows show the Radium logo</t>
+        </is>
+      </c>
+      <c r="E222" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F222" s="13" t="n"/>
+      <c r="G222" s="14" t="inlineStr">
+        <is>
+          <t>Install and uninstall v2.0.41 (or later): the title-bar icon (top left) and the header image (top right) of both the installer and the uninstaller windows show the Radium logo, not the Atomic mark. If either still shows the old mark, set the NSIS installer icon / header image explicitly in src-tauri/tauri.windows.conf.json and add a hardening check.</t>
+        </is>
+      </c>
+      <c r="H222" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I222" s="15" t="inlineStr">
+        <is>
+          <t>ADDED 2026-09-14 at the user's request, from a screenshot of the Radium Uninstall window with both places circled in red.</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="6" t="inlineStr">
+        <is>
+          <t>T30-S01</t>
+        </is>
+      </c>
+      <c r="B223" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C223" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D223" s="14" t="inlineStr">
+        <is>
+          <t>Proof on this PC</t>
+        </is>
+      </c>
+      <c r="E223" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F223" s="13" t="n"/>
+      <c r="G223" s="14" t="inlineStr">
+        <is>
+          <t>The pinned Vulkan build generates one SD 1.5 image; record time and memory.</t>
+        </is>
+      </c>
+      <c r="H223" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I223" s="15" t="inlineStr"/>
+    </row>
+    <row r="224">
+      <c r="A224" s="6" t="inlineStr">
+        <is>
+          <t>T30-S02</t>
+        </is>
+      </c>
+      <c r="B224" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C224" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D224" s="14" t="inlineStr">
+        <is>
+          <t>Engine variants</t>
+        </is>
+      </c>
+      <c r="E224" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F224" s="13" t="n"/>
+      <c r="G224" s="14" t="inlineStr">
+        <is>
+          <t>Choose CUDA / Vulkan / CPU from detected GPUs; pinned release manifest with SHA-256.</t>
+        </is>
+      </c>
+      <c r="H224" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I224" s="15" t="inlineStr"/>
+    </row>
+    <row r="225">
+      <c r="A225" s="6" t="inlineStr">
+        <is>
+          <t>T30-S03</t>
+        </is>
+      </c>
+      <c r="B225" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C225" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D225" s="14" t="inlineStr">
+        <is>
+          <t>Engine install</t>
+        </is>
+      </c>
+      <c r="E225" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F225" s="13" t="n"/>
+      <c r="G225" s="14" t="inlineStr">
+        <is>
+          <t>Download, verify, unpack into &lt;data&gt;/media/engine/&lt;release&gt;/&lt;variant&gt;; a bad checksum is refused.</t>
+        </is>
+      </c>
+      <c r="H225" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I225" s="15" t="inlineStr"/>
+    </row>
+    <row r="226">
+      <c r="A226" s="6" t="inlineStr">
+        <is>
+          <t>T30-S04</t>
+        </is>
+      </c>
+      <c r="B226" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C226" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D226" s="14" t="inlineStr">
+        <is>
+          <t>Model catalog and model install</t>
+        </is>
+      </c>
+      <c r="E226" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F226" s="13" t="n"/>
+      <c r="G226" s="14" t="inlineStr">
+        <is>
+          <t>Catalog with size, licence, source, SHA-256 and hardware needs; install with progress, cancel and checksum.</t>
+        </is>
+      </c>
+      <c r="H226" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I226" s="15" t="inlineStr"/>
+    </row>
+    <row r="227">
+      <c r="A227" s="6" t="inlineStr">
+        <is>
+          <t>T30-S05</t>
+        </is>
+      </c>
+      <c r="B227" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C227" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D227" s="14" t="inlineStr">
+        <is>
+          <t>Job runner</t>
+        </is>
+      </c>
+      <c r="E227" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F227" s="13" t="n"/>
+      <c r="G227" s="14" t="inlineStr">
+        <is>
+          <t>Build engine arguments from the contract's params, parse progress, cancel, write output into the media folder.</t>
+        </is>
+      </c>
+      <c r="H227" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I227" s="15" t="inlineStr"/>
+    </row>
+    <row r="228">
+      <c r="A228" s="6" t="inlineStr">
+        <is>
+          <t>T30-S06</t>
+        </is>
+      </c>
+      <c r="B228" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C228" s="6" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D228" s="14" t="inlineStr">
+        <is>
+          <t>builtin-engine adapter</t>
+        </is>
+      </c>
+      <c r="E228" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F228" s="13" t="n"/>
+      <c r="G228" s="14" t="inlineStr">
+        <is>
+          <t>Implements the media contract and passes the shared conformance suite unmodified; baseline provider for new users.</t>
+        </is>
+      </c>
+      <c r="H228" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I228" s="15" t="inlineStr"/>
+    </row>
+    <row r="229">
+      <c r="A229" s="6" t="inlineStr">
+        <is>
+          <t>T30-S07</t>
+        </is>
+      </c>
+      <c r="B229" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C229" s="6" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D229" s="14" t="inlineStr">
+        <is>
+          <t>Image provider drop-down</t>
+        </is>
+      </c>
+      <c r="E229" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F229" s="13" t="n"/>
+      <c r="G229" s="14" t="inlineStr">
+        <is>
+          <t>Media page lists every enabled provider; Settings lists the built-in provider first.</t>
+        </is>
+      </c>
+      <c r="H229" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I229" s="15" t="inlineStr"/>
+    </row>
+    <row r="230">
+      <c r="A230" s="6" t="inlineStr">
+        <is>
+          <t>T30-S08</t>
+        </is>
+      </c>
+      <c r="B230" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C230" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D230" s="14" t="inlineStr">
+        <is>
+          <t>First image from the Media page</t>
+        </is>
+      </c>
+      <c r="E230" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F230" s="13" t="n"/>
+      <c r="G230" s="14" t="inlineStr">
+        <is>
+          <t>End to end on this PC.</t>
+        </is>
+      </c>
+      <c r="H230" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I230" s="15" t="inlineStr"/>
+    </row>
+    <row r="231">
+      <c r="A231" s="6" t="inlineStr">
+        <is>
+          <t>T30-S09</t>
+        </is>
+      </c>
+      <c r="B231" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C231" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D231" s="14" t="inlineStr">
+        <is>
+          <t>Automatic1111 / Forge adapter</t>
+        </is>
+      </c>
+      <c r="E231" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F231" s="13" t="n"/>
+      <c r="G231" s="14" t="inlineStr">
+        <is>
+          <t>Passes the conformance suite.</t>
+        </is>
+      </c>
+      <c r="H231" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I231" s="15" t="inlineStr"/>
+    </row>
+    <row r="232">
+      <c r="A232" s="6" t="inlineStr">
+        <is>
+          <t>T30-S10</t>
+        </is>
+      </c>
+      <c r="B232" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C232" s="6" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D232" s="14" t="inlineStr">
+        <is>
+          <t>Stability AI, Replicate and fal.ai adapters</t>
+        </is>
+      </c>
+      <c r="E232" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F232" s="13" t="n"/>
+      <c r="G232" s="14" t="inlineStr">
+        <is>
+          <t>Each passes the conformance suite; keys in the OS credential store.</t>
+        </is>
+      </c>
+      <c r="H232" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I232" s="15" t="inlineStr"/>
+    </row>
+    <row r="233">
+      <c r="A233" s="6" t="inlineStr">
+        <is>
+          <t>T30-S11</t>
+        </is>
+      </c>
+      <c r="B233" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C233" s="6" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="D233" s="14" t="inlineStr">
+        <is>
+          <t>CUDA on the dual-3090 desktop</t>
+        </is>
+      </c>
+      <c r="E233" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F233" s="13" t="n"/>
+      <c r="G233" s="14" t="inlineStr">
+        <is>
+          <t>Install the CUDA build, generate, run two jobs on two GPUs; test splitting one job before promising it.</t>
+        </is>
+      </c>
+      <c r="H233" s="6" t="inlineStr">
+        <is>
+          <t>Desktop</t>
+        </is>
+      </c>
+      <c r="I233" s="15" t="inlineStr"/>
+    </row>
+    <row r="234">
+      <c r="A234" s="6" t="inlineStr">
+        <is>
+          <t>T30-S12</t>
+        </is>
+      </c>
+      <c r="B234" s="17" t="inlineStr">
+        <is>
+          <t>Task 30</t>
+        </is>
+      </c>
+      <c r="C234" s="6" t="inlineStr">
+        <is>
+          <t>12</t>
+        </is>
+      </c>
+      <c r="D234" s="14" t="inlineStr">
+        <is>
+          <t>Verify, commit, PR and test build</t>
+        </is>
+      </c>
+      <c r="E234" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F234" s="13" t="n"/>
+      <c r="G234" s="14" t="inlineStr">
+        <is>
+          <t>Web tsc -b, lint, vitest, test-quality; Rust tests, clippy, rustfmt; hardening; media guard; fork features rows; version-bumped build.</t>
+        </is>
+      </c>
+      <c r="H234" s="6" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="I234" s="15" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -12008,7 +12576,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13676,6 +14244,80 @@
         </is>
       </c>
       <c r="G45" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t>D39</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>SHOULD MEDIA HAVE ITS OWN ENGINE? (Task 30)</t>
+        </is>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>Task 30.</t>
+        </is>
+      </c>
+      <c r="D46" s="14" t="inlineStr">
+        <is>
+          <t>Bundle stable-diffusion.cpp (MIT), the image and video counterpart of llama.cpp that Chat already uses: installing Radium becomes enough; CUDA for NVIDIA, Vulkan for AMD/Intel, CPU fallback; pinned builds with checksums; the engine runs only while a job runs.</t>
+        </is>
+      </c>
+      <c r="E46" s="15" t="inlineStr">
+        <is>
+          <t>DECIDED BY THE USER 2026-09-14: "build it", after asking "do have to use comfyui? my initial plan was fir everything to be self contained" and being shown this recommendation. Supersedes the 2026-08-24 plan's rule that the media worker stays an external localhost service, and settles D12's open question about bundling an engine.</t>
+        </is>
+      </c>
+      <c r="F46" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G46" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>D40</t>
+        </is>
+      </c>
+      <c r="B47" s="14" t="inlineStr">
+        <is>
+          <t>HOW DOES THE USER CHOOSE WHERE IMAGES ARE MADE? (Task 30)</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>Task 30 S07, S09, S10.</t>
+        </is>
+      </c>
+      <c r="D47" s="14" t="inlineStr">
+        <is>
+          <t>The user's instruction, not a recommendation.</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>DECIDED BY THE USER 2026-09-14: "i still want the option to connect to comfyUI and the cloud and the local option. Also we need CUDA and Nvidia for when I get back to my dual 3090 desktop. Something like image processing provider with a drop down menu listing those providers I just listed and any other ones we can roll up into this". An Image provider drop-down lists Built-in, ComfyUI and cloud providers; Automatic1111/Forge, Stability AI, Replicate and fal.ai are added as further providers.</t>
+        </is>
+      </c>
+      <c r="F47" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G47" s="13" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): window buttons on every page and scroll bar arrows (Task 23), TurboQuant (Task 31, D41), first built-in media image (T30-S01), v2.0.42
- Task 23: the user found Minimize/Maximize/Close dead on some pages and asked
  for scroll bar arrows. Cause: notifications, the model picker drop-down and
  the full-screen image viewer were drawn over the window strip; the scroll
  bar lost its styling to a Firefox-only rule. Fixed in #10 (185f8317f,
  8d43c3f1d); new steps T23-S06 and T23-S07; check in v2.0.42.
- Task 31 and D41 (open): TurboQuant is not missing - fresh installs get it
  switched off by design and the CPU build is recommended on PCs with only
  built-in graphics. Whether to change either is the user's call.
- T30-S01 done: the built-in engine made its first image on this PC (84 s).
- Handover: install v2.0.42 and what to check.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): (1) USER: install test build v2.0.41 (run 34871145162) - BUILT SUCCESSFULLY 2026-09-14 (16:51-17:28 UTC); the installer is the run's artifact, ready for the user to install. It has everything so far: slim window strip (#10), Uncensored in the filter menu (#11), API/Cloud/run settings in Settings (#12), extensions fix (#15), rename (#16), version rule (#17), review before use with skills off by default (#18) and the Radium logo (#19). v2.0.40 did not build (typecheck mistakes in #18, now fixed). Check: connectors and skills ask for review (Preview lists tools and explains the command), every skill starts off, the Radium logo on the taskbar/installer/sidebar, no Cloud or API in the sidebar. (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 28 left: T28-S06 safer MCP default. (4) Task 26 when the user installs ComfyUI. (5) Working rule learned: check the web app with 'tsc -b' (as the build does), not 'tsc -p .'. | 2026-09-14 (later): Task 30 started - built-in media engine and Image provider choice (D39, D40); plan on feat/builtin-media-engine. First: S01 proof image on this PC. Task 29 gained T29-S05: the installer and uninstaller windows' title-bar icon and header image must show the Radium logo (user's screenshot).</t>
+          <t>2026-09-14 (latest): (1) USER: install test build v2.0.42 (run 34908571614) - v2.0.41 plus the window fixes: Minimize/Maximize/Close work on every page (including with a notification showing, the model picker open or an image open full-screen) and the scroll bar keeps an up and a down arrow. Also check T29-S05 (installer/uninstaller logo). (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 30 built-in media engine: S01 proof done (84 s image on this PC); next S02 engine variants, tests first, on feat/builtin-media-engine. (4) Task 31 TurboQuant: D41 open (default on? GPU on built-in graphics?). (5) Task 28 S06 safer MCP default. (6) Working rule: check the web app with tsc -b, as the build does.</t>
         </is>
       </c>
     </row>
@@ -1315,7 +1315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K33"/>
+  <dimension ref="A1:K34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2607,7 +2607,7 @@
       </c>
       <c r="I26" s="13" t="inlineStr">
         <is>
-          <t>d692991dd (PR #10)</t>
+          <t>d692991dd, ea8707641, 8d43c3f1d, 185f8317f (PR #10)</t>
         </is>
       </c>
       <c r="J26" s="14" t="inlineStr">
@@ -2617,7 +2617,7 @@
       </c>
       <c r="K26" s="15" t="inlineStr">
         <is>
-          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision. | 2026-09-13: PR #10 (fix/window-controls, head 229d2352b) now includes main, so its test build has the rename, the T21-S14 fix and the window controls together - run 34791322213. Waiting on: the user installs it and checks T23-S05. | 2026-09-14: the user asked for the controls in the page header with no separate bar (D33); done in 7141cef4c. PR #10 title and description updated. | 2026-09-14: D35 - back to a slim top strip with no line (commit ea8707641); v2.0.39 test build run 34843302629.</t>
+          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision. | 2026-09-13: PR #10 (fix/window-controls, head 229d2352b) now includes main, so its test build has the rename, the T21-S14 fix and the window controls together - run 34791322213. Waiting on: the user installs it and checks T23-S05. | 2026-09-14: the user asked for the controls in the page header with no separate bar (D33); done in 7141cef4c. PR #10 title and description updated. | 2026-09-14: D35 - back to a slim top strip with no line (commit ea8707641); v2.0.39 test build run 34843302629. | 2026-09-14: THE USER REPORTED (testing v2.0.41): "Some of the windows controls (minimize, close etc) isnt working on some pages. It works fine on the main page but not every page. Please make sure every page and window that has windows controls operates as it should and the transport bar (running vertically up the right side of the window has an arrow on top and bottom that is always available to be used". CAUSE FOUND IN THE CODE (computer control was off, so not reproduced by clicking): anything drawn over the 32px strip swallows its clicks - notifications (sonner toaster, z-index 999999999, placed 8px from the top, right over Close and Maximize), the model picker drop-down (z-index 9999) and the full-screen image viewer (z-index 100); the strip was z-index 60. FIXED 185f8317f: strip z-index 2147483646 (only the print-only artifact region is higher); notifications start 40px from the top where Radium draws its own buttons; a hardening check fails if anything gets a higher z-index than the strip. SCROLL BAR FIXED 8d43c3f1d: WebView2 (Chromium) ignored all ::-webkit-scrollbar styling because scrollbar-width / scrollbar-color were set on every element (meant for Firefox), so there were no arrows; now up/down arrows at both ends, a 14px bar, and the two properties apply only in Firefox. Pop-out windows (chat threads, logs, system monitor) keep the native title bar and nothing disables their buttons. In combined build v2.0.42.</t>
         </is>
       </c>
     </row>
@@ -2980,7 +2980,56 @@
       </c>
       <c r="K33" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: S01 proof started. The user approved downloading sd-master-42d6c0a-bin-win-vulkan-x64.zip (37.3 MB), sd-master-42d6c0a-bin-win-cpu-x64.zip (23.2 MB) and stable-diffusion-v1-5-pruned-emaonly-Q8_0.gguf (1.68 GB) for a test on this PC, checked against the SHA-256 published by GitHub and Hugging Face. This PC: AMD Ryzen 7 7735U with Radeon graphics (Vulkan present), 14.8 GB RAM, 64.6 GB free. Reuse found: the core download manager already verifies size and SHA-256 with progress and cancel; tauri-plugin-hardware already detects NVIDIA / AMD / Intel GPUs (not in test builds); the core already has a decompress command used for llama.cpp backends.</t>
+          <t>2026-09-14: S01 proof started. The user approved downloading sd-master-42d6c0a-bin-win-vulkan-x64.zip (37.3 MB), sd-master-42d6c0a-bin-win-cpu-x64.zip (23.2 MB) and stable-diffusion-v1-5-pruned-emaonly-Q8_0.gguf (1.68 GB) for a test on this PC, checked against the SHA-256 published by GitHub and Hugging Face. This PC: AMD Ryzen 7 7735U with Radeon graphics (Vulkan present), 14.8 GB RAM, 64.6 GB free. Reuse found: the core download manager already verifies size and SHA-256 with progress and cancel; tauri-plugin-hardware already detects NVIDIA / AMD / Intel GPUs (not in test builds); the core already has a decompress command used for llama.cpp backends. | 2026-09-14: S01 proof DONE - first image from the built-in engine on this PC in 84 s (see T30-S01).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t>Task 31</t>
+        </is>
+      </c>
+      <c r="B34" s="11" t="inlineStr">
+        <is>
+          <t>13 - Engines</t>
+        </is>
+      </c>
+      <c r="C34" s="14" t="inlineStr">
+        <is>
+          <t>Why TurboQuant looks unavailable, and whether it should be on by default</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="E34" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F34" s="13" t="n"/>
+      <c r="G34" s="14" t="inlineStr">
+        <is>
+          <t>D41 (open).</t>
+        </is>
+      </c>
+      <c r="H34" s="14" t="inlineStr">
+        <is>
+          <t>The user can use the TurboQuant llama.cpp provider, with the best build for their hardware, without hunting for a hidden switch.</t>
+        </is>
+      </c>
+      <c r="I34" s="13" t="n"/>
+      <c r="J34" s="14" t="inlineStr">
+        <is>
+          <t>ADDED 2026-09-14 at the user's request (screenshot: Settings, Model Providers, 'llama.cpp turboquant' listed under '1 disabled', 'windows-x64-cpu is the recommended backend'): "I cant use turboquant? can you look into this?"</t>
+        </is>
+      </c>
+      <c r="K34" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: MEASURED. (1) It is not missing: TurboQuant builds exist for Windows (windows-x64-cpu, cuda-12.4, cuda-13.3, vulkan; release b10269-1.4.0). (2) It is switched OFF on purpose for fresh installs: web-app/src/lib/turboquantDefaultMigration.ts freezes a per-profile flag at first launch - existing profiles keep it on, fresh installs get it off; it can be turned on with the switch in Settings &gt; Model Providers &gt; llama.cpp turboquant. The user reinstalled, so the profile counted as fresh. (3) The recommended build is CPU on this PC by design: the llama.cpp extension skips Vulkan when the only GPU is integrated (integratedGpuOnly in extensions/llamacpp-extension/src/index.ts), and this PC has only the Radeon graphics built into the Ryzen 7 7735U. Open question for the user: D41.</t>
         </is>
       </c>
     </row>
@@ -10480,7 +10529,7 @@
       </c>
       <c r="I183" s="15" t="inlineStr">
         <is>
-          <t>Edge resizing may have gone with the title bar - confirm rather than assume. | 2026-09-14: first look in a real build (run 34791322213): the buttons worked, but the user rejected the separate title bar (D33). Re-check on the combined build run 34800010936. | 2026-09-14: on the header-layout build the user saw the controls overlap the Hub's 'Open on Web' button and asked for the slim strip (D35). Re-check on test build v2.0.39, run 34843302629.</t>
+          <t>Edge resizing may have gone with the title bar - confirm rather than assume. | 2026-09-14: first look in a real build (run 34791322213): the buttons worked, but the user rejected the separate title bar (D33). Re-check on the combined build run 34800010936. | 2026-09-14: on the header-layout build the user saw the controls overlap the Hub's 'Open on Web' button and asked for the slim strip (D35). Re-check on test build v2.0.39, run 34843302629. | 2026-09-14: check again in v2.0.42 (run 34908571614) on every page, with a notification showing, with the model picker open and with an image open full-screen.</t>
         </is>
       </c>
     </row>
@@ -12114,7 +12163,7 @@
       </c>
       <c r="E223" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F223" s="13" t="n"/>
@@ -12128,7 +12177,11 @@
           <t>This PC</t>
         </is>
       </c>
-      <c r="I223" s="15" t="inlineStr"/>
+      <c r="I223" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: DONE. stable-diffusion.cpp master-866-42d6c0a (Vulkan build, SHA-256 verified) generated a 512x512 Stable Diffusion 1.5 (Q8_0 GGUF, SHA-256 verified) image on this PC's AMD Radeon graphics: 84 s in total (73 s sampling at ~3.5 s per step, 8.5 s decoding), 1.68 GB of model weights on the GPU. Image sent to the user. Engine facts for later steps: the release ships sd-cli.exe and sd-server.exe (a server that keeps a model loaded between images); --backend 'diffusion=cuda0&amp;cuda1' with --split-mode splits one job across two NVIDIA GPUs (to test on the dual-3090 desktop, S11); --max-vram / --auto-fit fit a model to the memory available; checksums for every build (CPU, Vulkan, CUDA 12 + runtime, ROCm, Linux, macOS) are published on the release.</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="6" t="inlineStr">
@@ -12576,7 +12629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G47"/>
+  <dimension ref="A1:G48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14322,6 +14375,39 @@
           <t>2026-09-14</t>
         </is>
       </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
+          <t>D41</t>
+        </is>
+      </c>
+      <c r="B48" s="14" t="inlineStr">
+        <is>
+          <t>SHOULD TURBOQUANT BE ON BY DEFAULT, AND USE THE GPU ON PCs WITH ONLY BUILT-IN GRAPHICS? (Task 31)</t>
+        </is>
+      </c>
+      <c r="C48" s="12" t="inlineStr">
+        <is>
+          <t>Task 31.</t>
+        </is>
+      </c>
+      <c r="D48" s="14" t="inlineStr">
+        <is>
+          <t>Two separate choices. (a) Default ON for fresh installs as well as existing ones, since the user wants to use it (a small change to turboquantDefaultMigration; existing fresh-install profiles such as this PC would be switched on once). (b) Keep recommending the CPU build where the only GPU is built-in graphics until it is measured on this PC: on shared-memory graphics the Vulkan build can be slower than CPU for generating text, so compare both before changing the rule.</t>
+        </is>
+      </c>
+      <c r="E48" s="15" t="inlineStr">
+        <is>
+          <t>RAISED 2026-09-14. The immediate answer given to the user: switch it on in Settings &gt; Model Providers &gt; llama.cpp turboquant; the CPU recommendation is by design on built-in graphics.</t>
+        </is>
+      </c>
+      <c r="F48" s="13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="G48" s="13" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
docs(tracker): v2.0.42 built; built-in media engine S02-S04 done
- v2.0.42 (run 34908571614) built successfully with the window fixes.
- Task 30: S02 engine build choice (5af4ca5fe), S03 install plan (0ceb4b8a0)
  and S04 model catalog (e7d57716c) done, tests first. Next: S05 job runner.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): (1) USER: install test build v2.0.42 (run 34908571614) - v2.0.41 plus the window fixes: Minimize/Maximize/Close work on every page (including with a notification showing, the model picker open or an image open full-screen) and the scroll bar keeps an up and a down arrow. Also check T29-S05 (installer/uninstaller logo). (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 30 built-in media engine: S01 proof done (84 s image on this PC); next S02 engine variants, tests first, on feat/builtin-media-engine. (4) Task 31 TurboQuant: D41 open (default on? GPU on built-in graphics?). (5) Task 28 S06 safer MCP default. (6) Working rule: check the web app with tsc -b, as the build does.</t>
+          <t>2026-09-14 (latest): (1) USER: install test build v2.0.42 (run 34908571614, BUILT) - v2.0.41 plus the window fixes: Minimize/Maximize/Close work on every page (including with a notification showing, the model picker open or an image open full-screen) and the scroll bar keeps an up and a down arrow. Also check T29-S05 (installer/uninstaller logo). (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 30 built-in media engine: S01-S04 done (proof image, engine build choice, install plan, model catalog); next S05 job runner, tests first, on feat/builtin-media-engine. (4) Task 31 TurboQuant: D41 open (default on? GPU on built-in graphics?). (5) Task 28 S06 safer MCP default. (6) Working rule: check the web app with tsc -b, as the build does.</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="K26" s="15" t="inlineStr">
         <is>
-          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision. | 2026-09-13: PR #10 (fix/window-controls, head 229d2352b) now includes main, so its test build has the rename, the T21-S14 fix and the window controls together - run 34791322213. Waiting on: the user installs it and checks T23-S05. | 2026-09-14: the user asked for the controls in the page header with no separate bar (D33); done in 7141cef4c. PR #10 title and description updated. | 2026-09-14: D35 - back to a slim top strip with no line (commit ea8707641); v2.0.39 test build run 34843302629. | 2026-09-14: THE USER REPORTED (testing v2.0.41): "Some of the windows controls (minimize, close etc) isnt working on some pages. It works fine on the main page but not every page. Please make sure every page and window that has windows controls operates as it should and the transport bar (running vertically up the right side of the window has an arrow on top and bottom that is always available to be used". CAUSE FOUND IN THE CODE (computer control was off, so not reproduced by clicking): anything drawn over the 32px strip swallows its clicks - notifications (sonner toaster, z-index 999999999, placed 8px from the top, right over Close and Maximize), the model picker drop-down (z-index 9999) and the full-screen image viewer (z-index 100); the strip was z-index 60. FIXED 185f8317f: strip z-index 2147483646 (only the print-only artifact region is higher); notifications start 40px from the top where Radium draws its own buttons; a hardening check fails if anything gets a higher z-index than the strip. SCROLL BAR FIXED 8d43c3f1d: WebView2 (Chromium) ignored all ::-webkit-scrollbar styling because scrollbar-width / scrollbar-color were set on every element (meant for Firefox), so there were no arrows; now up/down arrows at both ends, a 14px bar, and the two properties apply only in Firefox. Pop-out windows (chat threads, logs, system monitor) keep the native title bar and nothing disables their buttons. In combined build v2.0.42.</t>
+          <t>ROOT CAUSE, MEASURED 2026-09-13: the fork turned Windows' standard title bar OFF (81b393691, 2026-08-24, decorations false in src-tauri/tauri.windows.conf.json) and drew its own caption buttons instead (3b147addc, 2026-08-24, &lt;WindowControls /&gt; plus a drag region in web-app/src/routes/__root.tsx). The v2.0.35 sync merge c81c4ea98 (2026-09-11, an AI session) resolved __root.tsx by taking upstream's version, which has no WindowControls, and so silently removed them - while decorations stayed false. Upstream itself uses decorations TRUE. Result: since PR #4 merged into main on 2026-09-12 no build has any window buttons, including the Radium test install. The component and its test (components/__tests__/WindowControls.test.tsx) still exist; the test renders the component alone, so it kept passing. The merge commit message does not mention __root.tsx - the loss was not noticed, not a decision. | 2026-09-13: PR #10 (fix/window-controls, head 229d2352b) now includes main, so its test build has the rename, the T21-S14 fix and the window controls together - run 34791322213. Waiting on: the user installs it and checks T23-S05. | 2026-09-14: the user asked for the controls in the page header with no separate bar (D33); done in 7141cef4c. PR #10 title and description updated. | 2026-09-14: D35 - back to a slim top strip with no line (commit ea8707641); v2.0.39 test build run 34843302629. | 2026-09-14: THE USER REPORTED (testing v2.0.41): "Some of the windows controls (minimize, close etc) isnt working on some pages. It works fine on the main page but not every page. Please make sure every page and window that has windows controls operates as it should and the transport bar (running vertically up the right side of the window has an arrow on top and bottom that is always available to be used". CAUSE FOUND IN THE CODE (computer control was off, so not reproduced by clicking): anything drawn over the 32px strip swallows its clicks - notifications (sonner toaster, z-index 999999999, placed 8px from the top, right over Close and Maximize), the model picker drop-down (z-index 9999) and the full-screen image viewer (z-index 100); the strip was z-index 60. FIXED 185f8317f: strip z-index 2147483646 (only the print-only artifact region is higher); notifications start 40px from the top where Radium draws its own buttons; a hardening check fails if anything gets a higher z-index than the strip. SCROLL BAR FIXED 8d43c3f1d: WebView2 (Chromium) ignored all ::-webkit-scrollbar styling because scrollbar-width / scrollbar-color were set on every element (meant for Firefox), so there were no arrows; now up/down arrows at both ends, a 14px bar, and the two properties apply only in Firefox. Pop-out windows (chat threads, logs, system monitor) keep the native title bar and nothing disables their buttons. In combined build v2.0.42. | 2026-09-14: v2.0.42 (run 34908571614) BUILT SUCCESSFULLY with both window fixes; the user was notified to install it.</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="I33" s="13" t="inlineStr">
         <is>
-          <t>391956131 (plan)</t>
+          <t>391956131 (plan), 5af4ca5fe, 0ceb4b8a0, e7d57716c</t>
         </is>
       </c>
       <c r="J33" s="14" t="inlineStr">
@@ -2980,7 +2980,7 @@
       </c>
       <c r="K33" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: S01 proof started. The user approved downloading sd-master-42d6c0a-bin-win-vulkan-x64.zip (37.3 MB), sd-master-42d6c0a-bin-win-cpu-x64.zip (23.2 MB) and stable-diffusion-v1-5-pruned-emaonly-Q8_0.gguf (1.68 GB) for a test on this PC, checked against the SHA-256 published by GitHub and Hugging Face. This PC: AMD Ryzen 7 7735U with Radeon graphics (Vulkan present), 14.8 GB RAM, 64.6 GB free. Reuse found: the core download manager already verifies size and SHA-256 with progress and cancel; tauri-plugin-hardware already detects NVIDIA / AMD / Intel GPUs (not in test builds); the core already has a decompress command used for llama.cpp backends. | 2026-09-14: S01 proof DONE - first image from the built-in engine on this PC in 84 s (see T30-S01).</t>
+          <t>2026-09-14: S01 proof started. The user approved downloading sd-master-42d6c0a-bin-win-vulkan-x64.zip (37.3 MB), sd-master-42d6c0a-bin-win-cpu-x64.zip (23.2 MB) and stable-diffusion-v1-5-pruned-emaonly-Q8_0.gguf (1.68 GB) for a test on this PC, checked against the SHA-256 published by GitHub and Hugging Face. This PC: AMD Ryzen 7 7735U with Radeon graphics (Vulkan present), 14.8 GB RAM, 64.6 GB free. Reuse found: the core download manager already verifies size and SHA-256 with progress and cancel; tauri-plugin-hardware already detects NVIDIA / AMD / Intel GPUs (not in test builds); the core already has a decompress command used for llama.cpp backends. | 2026-09-14: S01 proof DONE - first image from the built-in engine on this PC in 84 s (see T30-S01). | 2026-09-14: S02-S04 done on feat/builtin-media-engine (engine build choice, install plan, model catalog). Next: S05 job runner.</t>
         </is>
       </c>
     </row>
@@ -12206,7 +12206,7 @@
       </c>
       <c r="E224" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F224" s="13" t="n"/>
@@ -12220,7 +12220,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I224" s="15" t="inlineStr"/>
+      <c r="I224" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: DONE 5af4ca5fe. Engine build chosen per computer, pinned to release master-866-42d6c0a with exact sizes and SHA-256: NVIDIA with CUDA driver -&gt; CUDA 12 build + CUDA runtime (CUDA wins beside other graphics); AMD/Intel or NVIDIA without CUDA -&gt; Vulkan, including built-in graphics; none -&gt; CPU; Linux Vulkan/CPU; Apple silicon Metal. 7 tests, red first.</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="6" t="inlineStr">
@@ -12245,7 +12249,7 @@
       </c>
       <c r="E225" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F225" s="13" t="n"/>
@@ -12259,7 +12263,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I225" s="15" t="inlineStr"/>
+      <c r="I225" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: DONE 0ceb4b8a0. Install plan: engine unpacks into media/engine/&lt;release&gt;/&lt;build&gt;; archives saved to media/engine/&lt;release&gt;/downloads/ in the existing download manager's form (size + SHA-256 enforced); CUDA downloads both archives into one install; installed only when the sd-cli program file is there. Reuses the existing download manager and decompress (zip) command. 5 tests, red first.</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="6" t="inlineStr">
@@ -12284,7 +12292,7 @@
       </c>
       <c r="E226" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F226" s="13" t="n"/>
@@ -12298,7 +12306,11 @@
           <t>Laptop</t>
         </is>
       </c>
-      <c r="I226" s="15" t="inlineStr"/>
+      <c r="I226" s="15" t="inlineStr">
+        <is>
+          <t>2026-09-14: DONE e7d57716c. Model catalog pinned to Hugging Face commits with sizes, SHA-256 and licences: Stable Diffusion 1.5 (the file verified on the laptop), SDXL 1.0 Q4_0 + MIT fp16-fix VAE (~8 GB), FLUX.1 schnell Q4_0 with VAE and both text encoders from one open Apache-2.0 repository (the official VAE is gated) (~12 GB), Wan 2.2 TI2V 5B video with its VAE and umt5 encoder (~12 GB). Every part saved in media/models/&lt;model&gt;/; installed only when every part is complete. 4 tests, red first; media tests 25/25; clippy clean.</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs(tracker): installer and uninstaller icon found and fixed (T29-S05), v2.0.43
The circled icons were NSIS's default, in every installer including v2.0.42,
because no installer icon was set. Fixed in #19 (8f0746133); combined test
build v2.0.43.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>2026-09-14 (latest): (1) USER: install test build v2.0.42 (run 34908571614, BUILT) - v2.0.41 plus the window fixes: Minimize/Maximize/Close work on every page (including with a notification showing, the model picker open or an image open full-screen) and the scroll bar keeps an up and a down arrow. Also check T29-S05 (installer/uninstaller logo). (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 30 built-in media engine: S01-S04 done (proof image, engine build choice, install plan, model catalog); next S05 job runner, tests first, on feat/builtin-media-engine. (4) Task 31 TurboQuant: D41 open (default on? GPU on built-in graphics?). (5) Task 28 S06 safer MCP default. (6) Working rule: check the web app with tsc -b, as the build does.</t>
+          <t>2026-09-14 (latest): (1) USER: install test build v2.0.43 (run 34916954195) - v2.0.42 plus the Radium icon on the installer and uninstaller (T29-S05); v2.0.42 (run 34908571614) is - v2.0.41 plus the window fixes: Minimize/Maximize/Close work on every page (including with a notification showing, the model picker open or an image open full-screen) and the scroll bar keeps an up and a down arrow. Also check T29-S05 (installer/uninstaller logo). (2) Merge order after the user's check: #10, #11, #15, #12, #13 (retarget to main), #14, #16, #19 (after #16; retarget to main), #17, #18. (3) Task 30 built-in media engine: S01-S04 done (proof image, engine build choice, install plan, model catalog); next S05 job runner, tests first, on feat/builtin-media-engine. (4) Task 31 TurboQuant: D41 open (default on? GPU on built-in graphics?). (5) Task 28 S06 safer MCP default. (6) Working rule: check the web app with tsc -b, as the build does.</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="I32" s="13" t="inlineStr">
         <is>
-          <t>351150e46 (PR #19)</t>
+          <t>351150e46, 8f0746133 (PR #19)</t>
         </is>
       </c>
       <c r="J32" s="14" t="inlineStr">
@@ -2927,7 +2927,7 @@
       </c>
       <c r="K32" s="15" t="inlineStr">
         <is>
-          <t>2026-09-14: the logo came from C:\Users\Warwick\Downloads\Radium LOGO.jpg (2048x2048). Trimmed to its rounded tile with transparent corners: 1024x1024 app icon source (src-tauri/icons/icon.png, the only tracked icon; tauri icon generates the rest) and 512x512 web logo images. The inverting/tinting that suited the old black-and-white mark is removed everywhere. The 'Atomic Chat' name still on the main chat page in the tested build was the sidebar wordmark, replaced by #16, which was not in that build. Left alone: the macOS tray template (must be a one-colour silhouette) and other products' names (Atomic Mail, Atomic Agent, AtomicChat model mirrors). | 2026-09-14: THE USER ASKED (screenshot of the Radium Uninstall window, two places circled): "add to the tracker sheet to add the radium logo in the two places ive circled in red". The two places are the Windows installer/uninstaller window's title-bar icon (top left) and its header image (top right). The screenshot is the uninstaller of a build made before #19, so it still shows the Atomic mark. Both come from the app's Windows icon (icon.ico), which the build generates from src-tauri/icons/icon.png - now the Radium logo - so they should show the Radium logo from v2.0.41 on. To be checked, not assumed (T29-S05); if the header image turns out to come from a separate NSIS setting, set it explicitly.</t>
+          <t>2026-09-14: the logo came from C:\Users\Warwick\Downloads\Radium LOGO.jpg (2048x2048). Trimmed to its rounded tile with transparent corners: 1024x1024 app icon source (src-tauri/icons/icon.png, the only tracked icon; tauri icon generates the rest) and 512x512 web logo images. The inverting/tinting that suited the old black-and-white mark is removed everywhere. The 'Atomic Chat' name still on the main chat page in the tested build was the sidebar wordmark, replaced by #16, which was not in that build. Left alone: the macOS tray template (must be a one-colour silhouette) and other products' names (Atomic Mail, Atomic Agent, AtomicChat model mirrors). | 2026-09-14: THE USER ASKED (screenshot of the Radium Uninstall window, two places circled): "add to the tracker sheet to add the radium logo in the two places ive circled in red". The two places are the Windows installer/uninstaller window's title-bar icon (top left) and its header image (top right). The screenshot is the uninstaller of a build made before #19, so it still shows the Atomic mark. Both come from the app's Windows icon (icon.ico), which the build generates from src-tauri/icons/icon.png - now the Radium logo - so they should show the Radium logo from v2.0.41 on. To be checked, not assumed (T29-S05); if the header image turns out to come from a separate NSIS setting, set it explicitly. | 2026-09-14: installer and uninstaller icon fixed (T29-S05, 8f0746133); in v2.0.43.</t>
         </is>
       </c>
     </row>
@@ -12120,7 +12120,7 @@
       </c>
       <c r="E222" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F222" s="13" t="n"/>
@@ -12136,7 +12136,7 @@
       </c>
       <c r="I222" s="15" t="inlineStr">
         <is>
-          <t>ADDED 2026-09-14 at the user's request, from a screenshot of the Radium Uninstall window with both places circled in red.</t>
+          <t>ADDED 2026-09-14 at the user's request, from a screenshot of the Radium Uninstall window with both places circled in red. | 2026-09-14: FOUND AND FIXED. The two circled places (title-bar icon and header icon of the Radium Uninstall window) were NSIS's own default icon, not the Atomic mark - the installer used it too in every build, including v2.0.42 (checked by extracting the icon from the downloaded Radium_2.0.42_x64-setup.exe and comparing it with the old Atomic.Chat_2.0.37_x64-setup.exe: identical NSIS default). Cause: bundle.windows.nsis.installerIcon was never set. Fix 8f0746133 (PR #19): installerIcon = icons/icon.ico in tauri.conf.json and tauri.windows.conf.json, the icon the build generates from the Radium logo; tests/radium-logo.test.mjs checks both (red first; hardening 45/45). Combined build v2.0.43 (run 34916954195). The user checks it after installing v2.0.43: installer and uninstaller windows show the Radium logo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): window buttons with pop-ups open (T23-S08), models folder (Task 32, D42), settings audit (Task 33)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1315,7 +1315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K34"/>
+  <dimension ref="A1:K36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3033,6 +3033,92 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>Task 32</t>
+        </is>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>13 - Engines</t>
+        </is>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>Choose where models are saved and loaded (Models folder)</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="inlineStr">
+        <is>
+          <t>Laptop, then this PC</t>
+        </is>
+      </c>
+      <c r="E35" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F35" s="13" t="n"/>
+      <c r="G35" s="14" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="H35" s="14" t="inlineStr">
+        <is>
+          <t>A folder the user picks on the Models page receives every downloaded model, the models already downloaded can move into it, and Radium loads models from there. Checked in a test build.</t>
+        </is>
+      </c>
+      <c r="I35" s="13" t="inlineStr">
+        <is>
+          <t>27549a3d8 (PR #20)</t>
+        </is>
+      </c>
+      <c r="J35" s="14" t="n"/>
+      <c r="K35" s="15" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t>Task 33</t>
+        </is>
+      </c>
+      <c r="B36" s="11" t="inlineStr">
+        <is>
+          <t>15 - Quality</t>
+        </is>
+      </c>
+      <c r="C36" s="14" t="inlineStr">
+        <is>
+          <t>Check every setting, switch and button does what it says</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="inlineStr">
+        <is>
+          <t>Laptop, then this PC</t>
+        </is>
+      </c>
+      <c r="E36" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F36" s="13" t="n"/>
+      <c r="G36" s="14" t="inlineStr">
+        <is>
+          <t>Computer control for Radium (declined 2026-09-14), or the user clicking through the checklist.</t>
+        </is>
+      </c>
+      <c r="H36" s="14" t="inlineStr">
+        <is>
+          <t>Every settings control is wired to something that uses it (static audit), and each page is clicked through in a test build.</t>
+        </is>
+      </c>
+      <c r="I36" s="13" t="n"/>
+      <c r="J36" s="14" t="n"/>
+      <c r="K36" s="15" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A2:K40"/>
   <dataValidations count="1">
@@ -3050,7 +3136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I234"/>
+  <dimension ref="A1:I242"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -12623,6 +12709,342 @@
         </is>
       </c>
       <c r="I234" s="15" t="inlineStr"/>
+    </row>
+    <row r="235">
+      <c r="A235" s="6" t="inlineStr">
+        <is>
+          <t>T23-S08</t>
+        </is>
+      </c>
+      <c r="B235" s="17" t="inlineStr">
+        <is>
+          <t>Task 23</t>
+        </is>
+      </c>
+      <c r="C235" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D235" s="14" t="inlineStr">
+        <is>
+          <t>Window buttons keep working while a pop-up or drop-down menu is open</t>
+        </is>
+      </c>
+      <c r="E235" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F235" s="13" t="n"/>
+      <c r="G235" s="14" t="inlineStr">
+        <is>
+          <t>Pop-ups and menus set pointer-events: none on &lt;body&gt;; the strip switches clicks back on. WindowFrame.test.tsx clicks the buttons with a pop-up and with a menu open (both failed before).</t>
+        </is>
+      </c>
+      <c r="H235" s="6" t="inlineStr">
+        <is>
+          <t>web-app/src/components/WindowFrame.tsx</t>
+        </is>
+      </c>
+      <c r="I235" s="15" t="inlineStr">
+        <is>
+          <t>b5bf16d5d (PR #10). Needs a check in the next test build.</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="6" t="inlineStr">
+        <is>
+          <t>T32-S01</t>
+        </is>
+      </c>
+      <c r="B236" s="17" t="inlineStr">
+        <is>
+          <t>Task 32</t>
+        </is>
+      </c>
+      <c r="C236" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D236" s="14" t="inlineStr">
+        <is>
+          <t>One Rust redirect for the models folder</t>
+        </is>
+      </c>
+      <c r="E236" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F236" s="13" t="n"/>
+      <c r="G236" s="14" t="inlineStr">
+        <is>
+          <t>core::app::models_folder: resolve_path, join_path, read/write_yaml, rm and the downloader follow the chosen folder. 13 unit + 5 file command tests + a real download test.</t>
+        </is>
+      </c>
+      <c r="H236" s="6" t="inlineStr">
+        <is>
+          <t>src-tauri/src/core/app/models_folder.rs</t>
+        </is>
+      </c>
+      <c r="I236" s="15" t="inlineStr">
+        <is>
+          <t>27549a3d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="6" t="inlineStr">
+        <is>
+          <t>T32-S02</t>
+        </is>
+      </c>
+      <c r="B237" s="17" t="inlineStr">
+        <is>
+          <t>Task 32</t>
+        </is>
+      </c>
+      <c r="C237" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D237" s="14" t="inlineStr">
+        <is>
+          <t>Move the models already downloaded</t>
+        </is>
+      </c>
+      <c r="E237" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F237" s="13" t="n"/>
+      <c r="G237" s="14" t="inlineStr">
+        <is>
+          <t>Rename on one drive; copy, size check, then remove across drives; never overwrite; refused while a download runs.</t>
+        </is>
+      </c>
+      <c r="H237" s="6" t="inlineStr">
+        <is>
+          <t>src-tauri/src/core/app/models_folder.rs</t>
+        </is>
+      </c>
+      <c r="I237" s="15" t="inlineStr">
+        <is>
+          <t>27549a3d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="6" t="inlineStr">
+        <is>
+          <t>T32-S03</t>
+        </is>
+      </c>
+      <c r="B238" s="17" t="inlineStr">
+        <is>
+          <t>Task 32</t>
+        </is>
+      </c>
+      <c r="C238" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D238" s="14" t="inlineStr">
+        <is>
+          <t>Models page: Models folder button and panel</t>
+        </is>
+      </c>
+      <c r="E238" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F238" s="13" t="n"/>
+      <c r="G238" s="14" t="inlineStr">
+        <is>
+          <t>ModelsFolderDialog.test.tsx (6): choose, move or leave, default, partial failure, refusal.</t>
+        </is>
+      </c>
+      <c r="H238" s="6" t="inlineStr">
+        <is>
+          <t>web-app/src/containers/hub/ModelsFolderDialog.tsx</t>
+        </is>
+      </c>
+      <c r="I238" s="15" t="inlineStr">
+        <is>
+          <t>27549a3d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="6" t="inlineStr">
+        <is>
+          <t>T32-S04</t>
+        </is>
+      </c>
+      <c r="B239" s="17" t="inlineStr">
+        <is>
+          <t>Task 32</t>
+        </is>
+      </c>
+      <c r="C239" s="6" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D239" s="14" t="inlineStr">
+        <is>
+          <t>Command-line tool follows the models folder</t>
+        </is>
+      </c>
+      <c r="E239" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F239" s="13" t="n"/>
+      <c r="G239" s="14" t="inlineStr">
+        <is>
+          <t>cli::models_in_a_chosen_folder_are_found_and_resolved.</t>
+        </is>
+      </c>
+      <c r="H239" s="6" t="inlineStr">
+        <is>
+          <t>src-tauri/src/core/cli/mod.rs</t>
+        </is>
+      </c>
+      <c r="I239" s="15" t="inlineStr">
+        <is>
+          <t>27549a3d8</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="6" t="inlineStr">
+        <is>
+          <t>T32-S05</t>
+        </is>
+      </c>
+      <c r="B240" s="17" t="inlineStr">
+        <is>
+          <t>Task 32</t>
+        </is>
+      </c>
+      <c r="C240" s="6" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D240" s="14" t="inlineStr">
+        <is>
+          <t>Check in a test build: pick a folder on another drive, download, move, load</t>
+        </is>
+      </c>
+      <c r="E240" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F240" s="13" t="n"/>
+      <c r="G240" s="14" t="inlineStr">
+        <is>
+          <t>A model downloads into the chosen folder, existing models move, a moved model loads and chats.</t>
+        </is>
+      </c>
+      <c r="H240" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I240" s="15" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="6" t="inlineStr">
+        <is>
+          <t>T33-S01</t>
+        </is>
+      </c>
+      <c r="B241" s="17" t="inlineStr">
+        <is>
+          <t>Task 33</t>
+        </is>
+      </c>
+      <c r="C241" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D241" s="14" t="inlineStr">
+        <is>
+          <t>Static audit: every settings control has a handler and every setting is used</t>
+        </is>
+      </c>
+      <c r="E241" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F241" s="13" t="n"/>
+      <c r="G241" s="14" t="inlineStr">
+        <is>
+          <t>No dead controls found: 9 flagged buttons all open menus or pop-ups; attachment settings reach the attachments engine; every llama.cpp setting becomes a server start option except timeout, llamacpp_env and auto_unload, which the engine reads at start. One stored value with no control (Vulkan enabled) is unused.</t>
+        </is>
+      </c>
+      <c r="H241" s="6" t="inlineStr">
+        <is>
+          <t>scratchpad settings-audit.mjs</t>
+        </is>
+      </c>
+      <c r="I241" s="15" t="n"/>
+    </row>
+    <row r="242">
+      <c r="A242" s="6" t="inlineStr">
+        <is>
+          <t>T33-S02</t>
+        </is>
+      </c>
+      <c r="B242" s="17" t="inlineStr">
+        <is>
+          <t>Task 33</t>
+        </is>
+      </c>
+      <c r="C242" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D242" s="14" t="inlineStr">
+        <is>
+          <t>Click through every page and window in a test build</t>
+        </is>
+      </c>
+      <c r="E242" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F242" s="13" t="n"/>
+      <c r="G242" s="14" t="inlineStr">
+        <is>
+          <t>Window buttons, each switch, slider, drop-down and button; record anything that does nothing.</t>
+        </is>
+      </c>
+      <c r="H242" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I242" s="15" t="inlineStr">
+        <is>
+          <t>Needs computer control for Radium, or the user.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -12641,7 +13063,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14420,6 +14842,43 @@
         </is>
       </c>
       <c r="G48" s="13" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>D42</t>
+        </is>
+      </c>
+      <c r="B49" s="14" t="inlineStr">
+        <is>
+          <t>WHERE ARE MODELS SAVED AND LOADED FROM? (Task 32)</t>
+        </is>
+      </c>
+      <c r="C49" s="12" t="inlineStr">
+        <is>
+          <t>Task 32.</t>
+        </is>
+      </c>
+      <c r="D49" s="14" t="inlineStr">
+        <is>
+          <t>The user's instruction, not a recommendation.</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>DECIDED BY THE USER 2026-09-14: "on the models page a simple settings and file system to create and forward every downloaded model to a user defined folder. Then user can select this folder as the default save and read space for models"</t>
+        </is>
+      </c>
+      <c r="F49" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G49" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
docs(tracker): hover line and glow on anything pressable (Task 34, D43), in test build 2.0.45
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
+++ b/docs/superpowers/plans/2026-09-08-model-agnostic-atomic-media-platform-tracker.xlsx
@@ -1315,7 +1315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K36"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3119,6 +3119,51 @@
       <c r="J36" s="14" t="n"/>
       <c r="K36" s="15" t="n"/>
     </row>
+    <row r="37">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>Task 34</t>
+        </is>
+      </c>
+      <c r="B37" s="11" t="inlineStr">
+        <is>
+          <t>11 - Brand</t>
+        </is>
+      </c>
+      <c r="C37" s="14" t="inlineStr">
+        <is>
+          <t>A line and glow around anything you can press, on hover</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="inlineStr">
+        <is>
+          <t>Laptop, then this PC</t>
+        </is>
+      </c>
+      <c r="E37" s="13" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F37" s="13" t="n"/>
+      <c r="G37" s="14" t="inlineStr">
+        <is>
+          <t>Nothing.</t>
+        </is>
+      </c>
+      <c r="H37" s="14" t="inlineStr">
+        <is>
+          <t>Hovering any button, link, menu item, switch, tab, slider or clickable card shows a 1.33px line and a strong glow, white in the dark theme. Checked in test build 2.0.45.</t>
+        </is>
+      </c>
+      <c r="I37" s="13" t="inlineStr">
+        <is>
+          <t>0f551be87 (PR #21)</t>
+        </is>
+      </c>
+      <c r="J37" s="14" t="n"/>
+      <c r="K37" s="15" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A2:K40"/>
   <dataValidations count="1">
@@ -3136,7 +3181,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I242"/>
+  <dimension ref="A1:I245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -13045,6 +13090,131 @@
           <t>Needs computer control for Radium, or the user.</t>
         </is>
       </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="6" t="inlineStr">
+        <is>
+          <t>T34-S01</t>
+        </is>
+      </c>
+      <c r="B243" s="17" t="inlineStr">
+        <is>
+          <t>Task 34</t>
+        </is>
+      </c>
+      <c r="C243" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D243" s="14" t="inlineStr">
+        <is>
+          <t>One app-wide hover rule</t>
+        </is>
+      </c>
+      <c r="E243" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F243" s="13" t="n"/>
+      <c r="G243" s="14" t="inlineStr">
+        <is>
+          <t>tests/hover-glow.test.mjs (6): coverage, exclusions, 1.33px line, 16px glow, both themes, outside @layer. Browser check: sidebar links and Download buttons in both themes.</t>
+        </is>
+      </c>
+      <c r="H243" s="6" t="inlineStr">
+        <is>
+          <t>web-app/src/index.css</t>
+        </is>
+      </c>
+      <c r="I243" s="15" t="inlineStr">
+        <is>
+          <t>0f551be87</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="6" t="inlineStr">
+        <is>
+          <t>T34-S02</t>
+        </is>
+      </c>
+      <c r="B244" s="17" t="inlineStr">
+        <is>
+          <t>Task 34</t>
+        </is>
+      </c>
+      <c r="C244" s="6" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D244" s="14" t="inlineStr">
+        <is>
+          <t>Line made one third thinner (2px to 1.33px)</t>
+        </is>
+      </c>
+      <c r="E244" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F244" s="13" t="n"/>
+      <c r="G244" s="14" t="inlineStr">
+        <is>
+          <t>At 125% Windows scaling this draws as one screen pixel; at 150% and 200% it is two-thirds of 2px.</t>
+        </is>
+      </c>
+      <c r="H244" s="6" t="inlineStr">
+        <is>
+          <t>web-app/src/index.css</t>
+        </is>
+      </c>
+      <c r="I244" s="15" t="inlineStr">
+        <is>
+          <t>0f551be87</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="6" t="inlineStr">
+        <is>
+          <t>T34-S03</t>
+        </is>
+      </c>
+      <c r="B245" s="17" t="inlineStr">
+        <is>
+          <t>Task 34</t>
+        </is>
+      </c>
+      <c r="C245" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D245" s="14" t="inlineStr">
+        <is>
+          <t>Check in test build 2.0.45</t>
+        </is>
+      </c>
+      <c r="E245" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F245" s="13" t="n"/>
+      <c r="G245" s="14" t="inlineStr">
+        <is>
+          <t>Hover buttons, sidebar links, menu items, switches and cards; the line and glow show and nothing is hidden.</t>
+        </is>
+      </c>
+      <c r="H245" s="6" t="inlineStr">
+        <is>
+          <t>This PC</t>
+        </is>
+      </c>
+      <c r="I245" s="15" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I250"/>
@@ -13063,7 +13233,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -14875,6 +15045,43 @@
         </is>
       </c>
       <c r="G49" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>D43</t>
+        </is>
+      </c>
+      <c r="B50" s="14" t="inlineStr">
+        <is>
+          <t>WHAT DOES HOVERING OVER SOMETHING PRESSABLE LOOK LIKE? (Task 34)</t>
+        </is>
+      </c>
+      <c r="C50" s="12" t="inlineStr">
+        <is>
+          <t>Task 34.</t>
+        </is>
+      </c>
+      <c r="D50" s="14" t="inlineStr">
+        <is>
+          <t>The user's instruction, not a recommendation.</t>
+        </is>
+      </c>
+      <c r="E50" s="15" t="inlineStr">
+        <is>
+          <t>DECIDED BY THE USER 2026-09-14: "Anytime a mouse hovers over an actional button or panel Radium should also have this white line glow. I want mine double the thickness and double the glow." Then: "make the white line 1/3 thinner".</t>
+        </is>
+      </c>
+      <c r="F50" s="13" t="inlineStr">
+        <is>
+          <t>Answered</t>
+        </is>
+      </c>
+      <c r="G50" s="13" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>

</xml_diff>